<commit_message>
Muñeca con una sola voz y herramienta Nota para marcar el golpe
- Luz roja: el archivo de la muñeca que canta y gira se reconoce como canción
  (core/voicing.js separa la voz del giro); la canción suena en verde y acaba
  justo en rojo, el giro suena en rojo y luego el escaneo. Nunca dos voces.
- Libre: herramienta «Nota» (marcar el golpe bailando): la canción suena
  entera y el presentador da a cada uno una nota del 1 al 10 desde el mando
  (freeScore); cada uno se lleva su nota. La tele enseña las notas y la
  clasificación; el móvil, «¡A bailar!» y su nota.
- Plantilla: sección «Marca el golpe» con Nota, canciones «Adivina Cancion n1»
  y «Golpe Cancion n1»; sin columnas Golpe/Silencio. Canciones/ admite
  subcarpetas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/plantilla-concurso.xlsx
+++ b/public/plantilla-concurso.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="751" uniqueCount="499">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="747" uniqueCount="500">
   <si>
     <t>EMPIEZA AQUÍ</t>
   </si>
@@ -168,7 +168,7 @@
     <t>pestaña «Libre»</t>
   </si>
   <si>
-    <t>Pruebas físicas: cronómetro, contador, contrarreloj (las botellas) o con canción (la bachata); tú das los puntos.</t>
+    <t>Pruebas físicas: cronómetro, contador, contrarreloj (las botellas) o nota del 1 al 10 (marcar el golpe bailando); tú das los puntos.</t>
   </si>
   <si>
     <t>Palabras secretas</t>
@@ -342,10 +342,10 @@
     <t>Cuando se ponga en verde… ¡pulsa!</t>
   </si>
   <si>
-    <t>Bachata: marca el golpe</t>
-  </si>
-  <si>
-    <t>La música se calla justo antes del golpe: seguid bailando a ciegas y clavad el golpe cuando vuelva.</t>
+    <t>Marca el golpe</t>
+  </si>
+  <si>
+    <t>Suena la canción: bailad y marcad el golpe a la vez. El presentador da a cada uno una nota del 1 al 10.</t>
   </si>
   <si>
     <t>¿Cuál es la mentira?</t>
@@ -513,7 +513,7 @@
     <t>↳ Solo para ti.</t>
   </si>
   <si>
-    <t>↳ Opcional: nombre del archivo en la carpeta «Canciones» (sin .mp3). Suena al abrir el turno.</t>
+    <t>↳ Opcional: nombre del archivo en «Canciones» (sin .mp3), p. ej. Adivina Cancion n1. Suena al abrir el turno.</t>
   </si>
   <si>
     <t>↳ Segundo de la canción por el que empieza. Vacío = 0.</t>
@@ -591,829 +591,832 @@
     <t>Thriller (Michael Jackson)</t>
   </si>
   <si>
-    <t>Archivo «Thriller.mp3» en «Canciones»</t>
+    <t>Archivo «Adivina Cancion n1» en «Canciones/Adivina la canción»</t>
+  </si>
+  <si>
+    <t>Adivina Cancion n1</t>
+  </si>
+  <si>
+    <t>Despacito (Luis Fonsi)</t>
+  </si>
+  <si>
+    <t>Archivo «Adivina Cancion n2»</t>
+  </si>
+  <si>
+    <t>Adivina Cancion n2</t>
+  </si>
+  <si>
+    <t>Macarena (Los del Río)</t>
+  </si>
+  <si>
+    <t>Archivo «Adivina Cancion n3»</t>
+  </si>
+  <si>
+    <t>Adivina Cancion n3</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>Correcta</t>
+  </si>
+  <si>
+    <t>Dificultad</t>
+  </si>
+  <si>
+    <t>Imagen</t>
+  </si>
+  <si>
+    <t>↳ La pregunta tal cual.</t>
+  </si>
+  <si>
+    <t>↳ Respuesta A</t>
+  </si>
+  <si>
+    <t>↳ Respuesta B</t>
+  </si>
+  <si>
+    <t>↳ C (opcional)</t>
+  </si>
+  <si>
+    <t>↳ D (opcional)</t>
+  </si>
+  <si>
+    <t>↳ Letra: se pinta de verde</t>
+  </si>
+  <si>
+    <t>↳ Música y puntos. Vacía = por orden.</t>
+  </si>
+  <si>
+    <t>↳ Opcional: dirección web (https://…).</t>
+  </si>
+  <si>
+    <t>¿Cuántos lados tiene un hexágono?</t>
+  </si>
+  <si>
+    <t>Cinco</t>
+  </si>
+  <si>
+    <t>Seis</t>
+  </si>
+  <si>
+    <t>Siete</t>
+  </si>
+  <si>
+    <t>Fácil</t>
+  </si>
+  <si>
+    <t>¿Qué usan las brujas de los cuentos para volar?</t>
+  </si>
+  <si>
+    <t>Una escoba</t>
+  </si>
+  <si>
+    <t>Una alfombra</t>
+  </si>
+  <si>
+    <t>Un paraguas</t>
+  </si>
+  <si>
+    <t>Una nube</t>
+  </si>
+  <si>
+    <t>¿Qué planeta es conocido como «el planeta rojo»?</t>
+  </si>
+  <si>
+    <t>Venus</t>
+  </si>
+  <si>
+    <t>Marte</t>
+  </si>
+  <si>
+    <t>Júpiter</t>
+  </si>
+  <si>
+    <t>Mercurio</t>
+  </si>
+  <si>
+    <t>¿Qué animal es Simba en «El rey león»?</t>
+  </si>
+  <si>
+    <t>Un tigre</t>
+  </si>
+  <si>
+    <t>Un guepardo</t>
+  </si>
+  <si>
+    <t>Un león</t>
+  </si>
+  <si>
+    <t>Un lobo</t>
+  </si>
+  <si>
+    <t>¿En qué año llegó el hombre a la Luna?</t>
+  </si>
+  <si>
+    <t>1965</t>
+  </si>
+  <si>
+    <t>1969</t>
+  </si>
+  <si>
+    <t>1972</t>
+  </si>
+  <si>
+    <t>1975</t>
+  </si>
+  <si>
+    <t>Media</t>
+  </si>
+  <si>
+    <t>¿Cuál es el planeta más grande del sistema solar?</t>
+  </si>
+  <si>
+    <t>Saturno</t>
+  </si>
+  <si>
+    <t>Neptuno</t>
+  </si>
+  <si>
+    <t>Urano</t>
+  </si>
+  <si>
+    <t>¿Quién escribió «Frankenstein»?</t>
+  </si>
+  <si>
+    <t>Bram Stoker</t>
+  </si>
+  <si>
+    <t>Mary Shelley</t>
+  </si>
+  <si>
+    <t>Edgar Allan Poe</t>
+  </si>
+  <si>
+    <t>H. P. Lovecraft</t>
+  </si>
+  <si>
+    <t>¿Quién dirigió la película «Psicosis» (1960)?</t>
+  </si>
+  <si>
+    <t>Stanley Kubrick</t>
+  </si>
+  <si>
+    <t>Steven Spielberg</t>
+  </si>
+  <si>
+    <t>John Carpenter</t>
+  </si>
+  <si>
+    <t>Alfred Hitchcock</t>
+  </si>
+  <si>
+    <t>¿Cuál es la capital de provincia española que está a más altitud?</t>
+  </si>
+  <si>
+    <t>Cuenca</t>
+  </si>
+  <si>
+    <t>Soria</t>
+  </si>
+  <si>
+    <t>Teruel</t>
+  </si>
+  <si>
+    <t>Ávila</t>
+  </si>
+  <si>
+    <t>Difícil</t>
+  </si>
+  <si>
+    <t>¿Qué elemento químico tiene el símbolo W?</t>
+  </si>
+  <si>
+    <t>Wolframio</t>
+  </si>
+  <si>
+    <t>Vanadio</t>
+  </si>
+  <si>
+    <t>Osmio</t>
+  </si>
+  <si>
+    <t>Teluro</t>
+  </si>
+  <si>
+    <t>¿Cuántos huesos tiene el cuerpo de un adulto?</t>
+  </si>
+  <si>
+    <t>186</t>
+  </si>
+  <si>
+    <t>206</t>
+  </si>
+  <si>
+    <t>226</t>
+  </si>
+  <si>
+    <t>256</t>
+  </si>
+  <si>
+    <t>¿En qué año se estrenó «La noche de Halloween», de John Carpenter?</t>
+  </si>
+  <si>
+    <t>1974</t>
+  </si>
+  <si>
+    <t>1978</t>
+  </si>
+  <si>
+    <t>1982</t>
+  </si>
+  <si>
+    <t>1986</t>
+  </si>
+  <si>
+    <t>Afirmación</t>
+  </si>
+  <si>
+    <t>↳ Una frase que puede ser verdad o mentira.</t>
+  </si>
+  <si>
+    <t>↳ Elige</t>
+  </si>
+  <si>
+    <t>Los pulpos tienen tres corazones.</t>
+  </si>
+  <si>
+    <t>Verdad</t>
+  </si>
+  <si>
+    <t>La Gran Muralla China se ve desde el espacio a simple vista.</t>
+  </si>
+  <si>
+    <t>Mentira</t>
+  </si>
+  <si>
+    <t>Los murciélagos son ciegos.</t>
+  </si>
+  <si>
+    <t>Para los botánicos, la calabaza es una fruta.</t>
+  </si>
+  <si>
+    <t>La miel bien cerrada no se estropea nunca.</t>
+  </si>
+  <si>
+    <t>En Japón y en Escocia, un gato negro trae buena suerte.</t>
+  </si>
+  <si>
+    <t>Bram Stoker viajó a Transilvania para escribir «Drácula».</t>
+  </si>
+  <si>
+    <t>Un rayo nunca cae dos veces en el mismo sitio.</t>
+  </si>
+  <si>
+    <t>Sobre quién</t>
+  </si>
+  <si>
+    <t>Frase 1</t>
+  </si>
+  <si>
+    <t>Frase 2</t>
+  </si>
+  <si>
+    <t>Frase 3</t>
+  </si>
+  <si>
+    <t>↳ Un jugador (su nombre, como entre: no vota) o un personaje famoso.</t>
+  </si>
+  <si>
+    <t>↳ Tres frases…</t>
+  </si>
+  <si>
+    <t>↳ …dos verdad…</t>
+  </si>
+  <si>
+    <t>↳ …y una mentira.</t>
+  </si>
+  <si>
+    <t>↳ Nº de la falsa: se pinta de rojo</t>
+  </si>
+  <si>
+    <t>Ana</t>
+  </si>
+  <si>
+    <t>He saltado en paracaídas.</t>
+  </si>
+  <si>
+    <t>Hablo japonés.</t>
+  </si>
+  <si>
+    <t>Tengo tres hermanos.</t>
+  </si>
+  <si>
+    <t>Drácula (la novela)</t>
+  </si>
+  <si>
+    <t>Puede convertirse en lobo y en murciélago.</t>
+  </si>
+  <si>
+    <t>No se refleja en los espejos.</t>
+  </si>
+  <si>
+    <t>Muere de un disparo con una bala de plata.</t>
+  </si>
+  <si>
+    <t>El monstruo de Frankenstein</t>
+  </si>
+  <si>
+    <t>En la novela tiene tornillos en el cuello.</t>
+  </si>
+  <si>
+    <t>En la novela no tiene nombre.</t>
+  </si>
+  <si>
+    <t>Mary Shelley empezó a escribirlo con 18 años.</t>
+  </si>
+  <si>
+    <t>Harry Potter</t>
+  </si>
+  <si>
+    <t>Su cumpleaños es el 31 de julio.</t>
+  </si>
+  <si>
+    <t>Su patronus es un lobo.</t>
+  </si>
+  <si>
+    <t>Su varita lleva una pluma de fénix.</t>
+  </si>
+  <si>
+    <t>Pesadilla antes de Navidad</t>
+  </si>
+  <si>
+    <t>Jack Skellington es el rey de Halloween.</t>
+  </si>
+  <si>
+    <t>Su perro fantasma se llama Zero.</t>
+  </si>
+  <si>
+    <t>La dirigió Tim Burton.</t>
+  </si>
+  <si>
+    <t>Los Cazafantasmas</t>
+  </si>
+  <si>
+    <t>Su cuartel es un antiguo parque de bomberos.</t>
+  </si>
+  <si>
+    <t>Cazan fantasmas en Chicago.</t>
+  </si>
+  <si>
+    <t>La película es de 1984.</t>
+  </si>
+  <si>
+    <t>Stephen King</t>
+  </si>
+  <si>
+    <t>Escribió «It».</t>
+  </si>
+  <si>
+    <t>Escribió «El exorcista».</t>
+  </si>
+  <si>
+    <t>Nació en Maine (Estados Unidos).</t>
+  </si>
+  <si>
+    <t>↳ «¿Quién es más probable que…?»: todos votan a un jugador.</t>
+  </si>
+  <si>
+    <t>¿Quién es más probable que llegue tarde a su propia boda?</t>
+  </si>
+  <si>
+    <t>¿Quién es más probable que sobreviva a un apocalipsis zombi?</t>
+  </si>
+  <si>
+    <t>¿Quién es más probable que sea el primero en morir en una película de miedo?</t>
+  </si>
+  <si>
+    <t>¿Quién es más probable que se coma los caramelos de Halloween antes de que llegue nadie?</t>
+  </si>
+  <si>
+    <t>¿Quién es más probable que grite en el pasaje del terror?</t>
+  </si>
+  <si>
+    <t>¿Quién es más probable que se haga amigo del fantasma de su casa?</t>
+  </si>
+  <si>
+    <t>¿Quién es más probable que repita disfraz todos los años?</t>
+  </si>
+  <si>
+    <t>¿Quién es más probable que invoque a un demonio por leer en voz alta un libro raro?</t>
+  </si>
+  <si>
+    <t>Unidad</t>
+  </si>
+  <si>
+    <t>Gana</t>
+  </si>
+  <si>
+    <t>↳ Una pregunta cuya respuesta es un número.</t>
+  </si>
+  <si>
+    <t>↳ El número exacto.</t>
+  </si>
+  <si>
+    <t>↳ Opcional (km, €…).</t>
+  </si>
+  <si>
+    <t>↳ Vacío = más cercano.</t>
+  </si>
+  <si>
+    <t>¿Cuántos kilómetros mide el Ebro?</t>
+  </si>
+  <si>
+    <t>km</t>
+  </si>
+  <si>
+    <t>Más cercano</t>
+  </si>
+  <si>
+    <t>¿Cuántos kilos pesaba la calabaza más pesada del mundo (récord de 2023)?</t>
+  </si>
+  <si>
+    <t>kg</t>
+  </si>
+  <si>
+    <t>¿En qué año se publicó «Drácula», de Bram Stoker?</t>
+  </si>
+  <si>
+    <t>¿Cuántos metros mide la Torre Eiffel (con sus antenas)?</t>
+  </si>
+  <si>
+    <t>m</t>
+  </si>
+  <si>
+    <t>¿Cuántas teclas tiene un piano normal?</t>
+  </si>
+  <si>
+    <t>teclas</t>
+  </si>
+  <si>
+    <t>Sin pasarse</t>
+  </si>
+  <si>
+    <t>¿Cuántos kilómetros hay en línea recta de Madrid a Barcelona?</t>
+  </si>
+  <si>
+    <t>¿Cuántos años vivió Edgar Allan Poe?</t>
+  </si>
+  <si>
+    <t>años</t>
+  </si>
+  <si>
+    <t>¿Cuántos dientes tiene un adulto, con las muelas del juicio?</t>
+  </si>
+  <si>
+    <t>dientes</t>
+  </si>
+  <si>
+    <t>Objetivo (s)</t>
+  </si>
+  <si>
+    <t>Modo</t>
+  </si>
+  <si>
+    <t>Desaparece a los (s)</t>
+  </si>
+  <si>
+    <t>↳ Segundos a los que hay que parar el reloj.</t>
+  </si>
+  <si>
+    <t>↳ ¿Se ve el reloj?</t>
+  </si>
+  <si>
+    <t>↳ Solo con «Desaparece».</t>
+  </si>
+  <si>
+    <t>Visible</t>
+  </si>
+  <si>
+    <t>Desaparece</t>
+  </si>
+  <si>
+    <t>A ciegas</t>
+  </si>
+  <si>
+    <t>Rondas</t>
+  </si>
+  <si>
+    <t>Participan</t>
+  </si>
+  <si>
+    <t>↳ Cuántas veces se juega.</t>
+  </si>
+  <si>
+    <t>↳ Duelo: eliges a dos en el mando.</t>
+  </si>
+  <si>
+    <t>Todos</t>
+  </si>
+  <si>
+    <t>Duelo</t>
+  </si>
+  <si>
+    <t>Prueba</t>
+  </si>
+  <si>
+    <t>Herramienta</t>
+  </si>
+  <si>
+    <t>Piezas</t>
+  </si>
+  <si>
+    <t>↳ Nombre de la prueba.</t>
+  </si>
+  <si>
+    <t>↳ Qué hay que hacer (sale en la tele).</t>
+  </si>
+  <si>
+    <t>↳ Cronómetro: gana quien más aguanta. Contador: +1/−1. Contrarreloj: de uno en uno, gana el más rápido. Nota: das a cada uno del 1 al 10 (sus puntos). Ninguna: eliges tú.</t>
+  </si>
+  <si>
+    <t>↳ ¿Juega cada uno o cada equipo (uno por equipo)?</t>
+  </si>
+  <si>
+    <t>↳ Vacío = los de la sección. Con Nota no cuenta: los puntos son la nota.</t>
+  </si>
+  <si>
+    <t>↳ Contrarreloj: en cada intento apuntas cuántas tiene bien (p. ej. 5 botellas).</t>
+  </si>
+  <si>
+    <t>↳ Opcional: archivo en «Canciones» (sin .mp3), p. ej. Golpe Cancion n1. Suena entera al «¡Empezar!».</t>
+  </si>
+  <si>
+    <t>↳ Segundo por el que empieza la canción.</t>
+  </si>
+  <si>
+    <t>3 de cada equipo con un globo en el tobillo. Gana el equipo al que le quede algún globo.</t>
+  </si>
+  <si>
+    <t>Ninguna</t>
+  </si>
+  <si>
+    <t>Equipos</t>
+  </si>
+  <si>
+    <t>La revancha</t>
+  </si>
+  <si>
+    <t>¡Otra vez! Globos nuevos y los mismos tres… o tres distintos.</t>
+  </si>
+  <si>
+    <t>Uno por equipo. La caja a la cadera, por la espalda: gana quien saque todas las pelotas primero.</t>
+  </si>
+  <si>
+    <t>Twerking: la revancha</t>
+  </si>
+  <si>
+    <t>Otro de cada equipo, la caja llena otra vez.</t>
+  </si>
+  <si>
+    <t>Uno por equipo, manos atadas a la espalda y la galleta en la mesa. ¡A comer!</t>
+  </si>
+  <si>
+    <t>La galleta: segunda carrera</t>
+  </si>
+  <si>
+    <t>Otros dos, otra galleta.</t>
+  </si>
+  <si>
+    <t>Uno por equipo, primero uno y luego el otro. Ordena las 5 botellas como las tiene escondidas el presentador.</t>
+  </si>
+  <si>
+    <t>Contrarreloj</t>
+  </si>
+  <si>
+    <t>Golpe 1</t>
+  </si>
+  <si>
+    <t>En pareja: bailad la canción y marcad el golpe a la vez. Nota del 1 al 10.</t>
+  </si>
+  <si>
+    <t>Nota</t>
+  </si>
+  <si>
+    <t>Jugadores</t>
+  </si>
+  <si>
+    <t>Golpe Cancion n1</t>
+  </si>
+  <si>
+    <t>Golpe 2</t>
+  </si>
+  <si>
+    <t>Otra canción, otro golpe: ¡a clavarlo!</t>
+  </si>
+  <si>
+    <t>Golpe Cancion n2</t>
+  </si>
+  <si>
+    <t>Golpe 3</t>
+  </si>
+  <si>
+    <t>La final: la más difícil.</t>
+  </si>
+  <si>
+    <t>Golpe Cancion n3</t>
+  </si>
+  <si>
+    <t>Plancha</t>
+  </si>
+  <si>
+    <t>Aguanta en plancha. Gana el último.</t>
+  </si>
+  <si>
+    <t>Cronómetro</t>
+  </si>
+  <si>
+    <t>Flexiones</t>
+  </si>
+  <si>
+    <t>Más flexiones en un minuto.</t>
+  </si>
+  <si>
+    <t>Contador</t>
+  </si>
+  <si>
+    <t>Sentadillas</t>
+  </si>
+  <si>
+    <t>Más sentadillas en un minuto (bajando hasta abajo).</t>
+  </si>
+  <si>
+    <t>La silla invisible</t>
+  </si>
+  <si>
+    <t>Espalda en la pared, como sentado en una silla. Gana el último.</t>
+  </si>
+  <si>
+    <t>Flamenco a ciegas</t>
+  </si>
+  <si>
+    <t>A la pata coja y con los ojos cerrados. Gana el último en apoyar el pie.</t>
+  </si>
+  <si>
+    <t>La momia</t>
+  </si>
+  <si>
+    <t>Envolved a un compañero en papel higiénico en un minuto. Gana la mejor momia.</t>
+  </si>
+  <si>
+    <t>Manzana colgante</t>
+  </si>
+  <si>
+    <t>Muerde la manzana que cuelga de un hilo, sin manos. El primero, gana.</t>
+  </si>
+  <si>
+    <t>Burpees</t>
+  </si>
+  <si>
+    <t>Más burpees en 30 segundos, entre todo el equipo.</t>
+  </si>
+  <si>
+    <t>Palabra</t>
+  </si>
+  <si>
+    <t>Prohibidas</t>
+  </si>
+  <si>
+    <t>↳ Lo que hay que adivinar. Solo la ven quien la hace y el equipo rival.</t>
+  </si>
+  <si>
+    <t>↳ Tabú: las que no se pueden decir, separadas por comas.</t>
+  </si>
+  <si>
+    <t>↳ Vacío = Tabú si hay prohibidas; si no, Mímica.</t>
+  </si>
+  <si>
+    <t>Calabaza</t>
+  </si>
+  <si>
+    <t>Halloween, naranja, vela, cara</t>
+  </si>
+  <si>
+    <t>Tabú</t>
+  </si>
+  <si>
+    <t>Vampiro</t>
+  </si>
+  <si>
+    <t>Sangre, Drácula, colmillos, murciélago</t>
+  </si>
+  <si>
+    <t>Fantasma</t>
+  </si>
+  <si>
+    <t>Sábana, espíritu, casa encantada, susto</t>
+  </si>
+  <si>
+    <t>Bruja</t>
+  </si>
+  <si>
+    <t>Escoba, caldero, sombrero, hechizo</t>
+  </si>
+  <si>
+    <t>Telaraña</t>
+  </si>
+  <si>
+    <t>Araña, hilo, red, tejer</t>
+  </si>
+  <si>
+    <t>Esqueleto</t>
+  </si>
+  <si>
+    <t>Huesos, calavera, cuerpo, muerto</t>
+  </si>
+  <si>
+    <t>Cementerio</t>
+  </si>
+  <si>
+    <t>Tumba, muertos, lápida, enterrar</t>
+  </si>
+  <si>
+    <t>Murciélago</t>
+  </si>
+  <si>
+    <t>Vampiro, volar, cueva, noche</t>
+  </si>
+  <si>
+    <t>Caramelo</t>
+  </si>
+  <si>
+    <t>Dulce, azúcar, chuche, truco o trato</t>
+  </si>
+  <si>
+    <t>Luna llena</t>
+  </si>
+  <si>
+    <t>Noche, lobo, redonda, cielo</t>
+  </si>
+  <si>
+    <t>Hombre lobo</t>
+  </si>
+  <si>
+    <t>Mímica</t>
+  </si>
+  <si>
+    <t>Momia</t>
+  </si>
+  <si>
+    <t>Zombi</t>
+  </si>
+  <si>
+    <t>Tallar una calabaza</t>
+  </si>
+  <si>
+    <t>Pedir caramelos</t>
+  </si>
+  <si>
+    <t>Volar en escoba</t>
+  </si>
+  <si>
+    <t>Ver una peli de miedo</t>
+  </si>
+  <si>
+    <t>Salir de un ataúd</t>
+  </si>
+  <si>
+    <t>Gato negro</t>
+  </si>
+  <si>
+    <t>Poción</t>
+  </si>
+  <si>
+    <t>Descríbelo</t>
+  </si>
+  <si>
+    <t>Disfraz</t>
+  </si>
+  <si>
+    <t>Escalofrío</t>
+  </si>
+  <si>
+    <t>Casa encantada</t>
+  </si>
+  <si>
+    <t>Ataúd</t>
   </si>
   <si>
     <t>Thriller</t>
-  </si>
-  <si>
-    <t>Despacito (Luis Fonsi)</t>
-  </si>
-  <si>
-    <t>Archivo «Despacito.mp3» en «Canciones»</t>
-  </si>
-  <si>
-    <t>Despacito</t>
-  </si>
-  <si>
-    <t>Macarena (Los del Río)</t>
-  </si>
-  <si>
-    <t>Archivo «Macarena.mp3» en «Canciones»</t>
-  </si>
-  <si>
-    <t>Macarena</t>
-  </si>
-  <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>B</t>
-  </si>
-  <si>
-    <t>C</t>
-  </si>
-  <si>
-    <t>D</t>
-  </si>
-  <si>
-    <t>Correcta</t>
-  </si>
-  <si>
-    <t>Dificultad</t>
-  </si>
-  <si>
-    <t>Imagen</t>
-  </si>
-  <si>
-    <t>↳ La pregunta tal cual.</t>
-  </si>
-  <si>
-    <t>↳ Respuesta A</t>
-  </si>
-  <si>
-    <t>↳ Respuesta B</t>
-  </si>
-  <si>
-    <t>↳ C (opcional)</t>
-  </si>
-  <si>
-    <t>↳ D (opcional)</t>
-  </si>
-  <si>
-    <t>↳ Letra: se pinta de verde</t>
-  </si>
-  <si>
-    <t>↳ Música y puntos. Vacía = por orden.</t>
-  </si>
-  <si>
-    <t>↳ Opcional: dirección web (https://…).</t>
-  </si>
-  <si>
-    <t>¿Cuántos lados tiene un hexágono?</t>
-  </si>
-  <si>
-    <t>Cinco</t>
-  </si>
-  <si>
-    <t>Seis</t>
-  </si>
-  <si>
-    <t>Siete</t>
-  </si>
-  <si>
-    <t>Fácil</t>
-  </si>
-  <si>
-    <t>¿Qué usan las brujas de los cuentos para volar?</t>
-  </si>
-  <si>
-    <t>Una escoba</t>
-  </si>
-  <si>
-    <t>Una alfombra</t>
-  </si>
-  <si>
-    <t>Un paraguas</t>
-  </si>
-  <si>
-    <t>Una nube</t>
-  </si>
-  <si>
-    <t>¿Qué planeta es conocido como «el planeta rojo»?</t>
-  </si>
-  <si>
-    <t>Venus</t>
-  </si>
-  <si>
-    <t>Marte</t>
-  </si>
-  <si>
-    <t>Júpiter</t>
-  </si>
-  <si>
-    <t>Mercurio</t>
-  </si>
-  <si>
-    <t>¿Qué animal es Simba en «El rey león»?</t>
-  </si>
-  <si>
-    <t>Un tigre</t>
-  </si>
-  <si>
-    <t>Un guepardo</t>
-  </si>
-  <si>
-    <t>Un león</t>
-  </si>
-  <si>
-    <t>Un lobo</t>
-  </si>
-  <si>
-    <t>¿En qué año llegó el hombre a la Luna?</t>
-  </si>
-  <si>
-    <t>1965</t>
-  </si>
-  <si>
-    <t>1969</t>
-  </si>
-  <si>
-    <t>1972</t>
-  </si>
-  <si>
-    <t>1975</t>
-  </si>
-  <si>
-    <t>Media</t>
-  </si>
-  <si>
-    <t>¿Cuál es el planeta más grande del sistema solar?</t>
-  </si>
-  <si>
-    <t>Saturno</t>
-  </si>
-  <si>
-    <t>Neptuno</t>
-  </si>
-  <si>
-    <t>Urano</t>
-  </si>
-  <si>
-    <t>¿Quién escribió «Frankenstein»?</t>
-  </si>
-  <si>
-    <t>Bram Stoker</t>
-  </si>
-  <si>
-    <t>Mary Shelley</t>
-  </si>
-  <si>
-    <t>Edgar Allan Poe</t>
-  </si>
-  <si>
-    <t>H. P. Lovecraft</t>
-  </si>
-  <si>
-    <t>¿Quién dirigió la película «Psicosis» (1960)?</t>
-  </si>
-  <si>
-    <t>Stanley Kubrick</t>
-  </si>
-  <si>
-    <t>Steven Spielberg</t>
-  </si>
-  <si>
-    <t>John Carpenter</t>
-  </si>
-  <si>
-    <t>Alfred Hitchcock</t>
-  </si>
-  <si>
-    <t>¿Cuál es la capital de provincia española que está a más altitud?</t>
-  </si>
-  <si>
-    <t>Cuenca</t>
-  </si>
-  <si>
-    <t>Soria</t>
-  </si>
-  <si>
-    <t>Teruel</t>
-  </si>
-  <si>
-    <t>Ávila</t>
-  </si>
-  <si>
-    <t>Difícil</t>
-  </si>
-  <si>
-    <t>¿Qué elemento químico tiene el símbolo W?</t>
-  </si>
-  <si>
-    <t>Wolframio</t>
-  </si>
-  <si>
-    <t>Vanadio</t>
-  </si>
-  <si>
-    <t>Osmio</t>
-  </si>
-  <si>
-    <t>Teluro</t>
-  </si>
-  <si>
-    <t>¿Cuántos huesos tiene el cuerpo de un adulto?</t>
-  </si>
-  <si>
-    <t>186</t>
-  </si>
-  <si>
-    <t>206</t>
-  </si>
-  <si>
-    <t>226</t>
-  </si>
-  <si>
-    <t>256</t>
-  </si>
-  <si>
-    <t>¿En qué año se estrenó «La noche de Halloween», de John Carpenter?</t>
-  </si>
-  <si>
-    <t>1974</t>
-  </si>
-  <si>
-    <t>1978</t>
-  </si>
-  <si>
-    <t>1982</t>
-  </si>
-  <si>
-    <t>1986</t>
-  </si>
-  <si>
-    <t>Afirmación</t>
-  </si>
-  <si>
-    <t>↳ Una frase que puede ser verdad o mentira.</t>
-  </si>
-  <si>
-    <t>↳ Elige</t>
-  </si>
-  <si>
-    <t>Los pulpos tienen tres corazones.</t>
-  </si>
-  <si>
-    <t>Verdad</t>
-  </si>
-  <si>
-    <t>La Gran Muralla China se ve desde el espacio a simple vista.</t>
-  </si>
-  <si>
-    <t>Mentira</t>
-  </si>
-  <si>
-    <t>Los murciélagos son ciegos.</t>
-  </si>
-  <si>
-    <t>Para los botánicos, la calabaza es una fruta.</t>
-  </si>
-  <si>
-    <t>La miel bien cerrada no se estropea nunca.</t>
-  </si>
-  <si>
-    <t>En Japón y en Escocia, un gato negro trae buena suerte.</t>
-  </si>
-  <si>
-    <t>Bram Stoker viajó a Transilvania para escribir «Drácula».</t>
-  </si>
-  <si>
-    <t>Un rayo nunca cae dos veces en el mismo sitio.</t>
-  </si>
-  <si>
-    <t>Sobre quién</t>
-  </si>
-  <si>
-    <t>Frase 1</t>
-  </si>
-  <si>
-    <t>Frase 2</t>
-  </si>
-  <si>
-    <t>Frase 3</t>
-  </si>
-  <si>
-    <t>↳ Un jugador (su nombre, como entre: no vota) o un personaje famoso.</t>
-  </si>
-  <si>
-    <t>↳ Tres frases…</t>
-  </si>
-  <si>
-    <t>↳ …dos verdad…</t>
-  </si>
-  <si>
-    <t>↳ …y una mentira.</t>
-  </si>
-  <si>
-    <t>↳ Nº de la falsa: se pinta de rojo</t>
-  </si>
-  <si>
-    <t>Ana</t>
-  </si>
-  <si>
-    <t>He saltado en paracaídas.</t>
-  </si>
-  <si>
-    <t>Hablo japonés.</t>
-  </si>
-  <si>
-    <t>Tengo tres hermanos.</t>
-  </si>
-  <si>
-    <t>Drácula (la novela)</t>
-  </si>
-  <si>
-    <t>Puede convertirse en lobo y en murciélago.</t>
-  </si>
-  <si>
-    <t>No se refleja en los espejos.</t>
-  </si>
-  <si>
-    <t>Muere de un disparo con una bala de plata.</t>
-  </si>
-  <si>
-    <t>El monstruo de Frankenstein</t>
-  </si>
-  <si>
-    <t>En la novela tiene tornillos en el cuello.</t>
-  </si>
-  <si>
-    <t>En la novela no tiene nombre.</t>
-  </si>
-  <si>
-    <t>Mary Shelley empezó a escribirlo con 18 años.</t>
-  </si>
-  <si>
-    <t>Harry Potter</t>
-  </si>
-  <si>
-    <t>Su cumpleaños es el 31 de julio.</t>
-  </si>
-  <si>
-    <t>Su patronus es un lobo.</t>
-  </si>
-  <si>
-    <t>Su varita lleva una pluma de fénix.</t>
-  </si>
-  <si>
-    <t>Pesadilla antes de Navidad</t>
-  </si>
-  <si>
-    <t>Jack Skellington es el rey de Halloween.</t>
-  </si>
-  <si>
-    <t>Su perro fantasma se llama Zero.</t>
-  </si>
-  <si>
-    <t>La dirigió Tim Burton.</t>
-  </si>
-  <si>
-    <t>Los Cazafantasmas</t>
-  </si>
-  <si>
-    <t>Su cuartel es un antiguo parque de bomberos.</t>
-  </si>
-  <si>
-    <t>Cazan fantasmas en Chicago.</t>
-  </si>
-  <si>
-    <t>La película es de 1984.</t>
-  </si>
-  <si>
-    <t>Stephen King</t>
-  </si>
-  <si>
-    <t>Escribió «It».</t>
-  </si>
-  <si>
-    <t>Escribió «El exorcista».</t>
-  </si>
-  <si>
-    <t>Nació en Maine (Estados Unidos).</t>
-  </si>
-  <si>
-    <t>↳ «¿Quién es más probable que…?»: todos votan a un jugador.</t>
-  </si>
-  <si>
-    <t>¿Quién es más probable que llegue tarde a su propia boda?</t>
-  </si>
-  <si>
-    <t>¿Quién es más probable que sobreviva a un apocalipsis zombi?</t>
-  </si>
-  <si>
-    <t>¿Quién es más probable que sea el primero en morir en una película de miedo?</t>
-  </si>
-  <si>
-    <t>¿Quién es más probable que se coma los caramelos de Halloween antes de que llegue nadie?</t>
-  </si>
-  <si>
-    <t>¿Quién es más probable que grite en el pasaje del terror?</t>
-  </si>
-  <si>
-    <t>¿Quién es más probable que se haga amigo del fantasma de su casa?</t>
-  </si>
-  <si>
-    <t>¿Quién es más probable que repita disfraz todos los años?</t>
-  </si>
-  <si>
-    <t>¿Quién es más probable que invoque a un demonio por leer en voz alta un libro raro?</t>
-  </si>
-  <si>
-    <t>Unidad</t>
-  </si>
-  <si>
-    <t>Gana</t>
-  </si>
-  <si>
-    <t>↳ Una pregunta cuya respuesta es un número.</t>
-  </si>
-  <si>
-    <t>↳ El número exacto.</t>
-  </si>
-  <si>
-    <t>↳ Opcional (km, €…).</t>
-  </si>
-  <si>
-    <t>↳ Vacío = más cercano.</t>
-  </si>
-  <si>
-    <t>¿Cuántos kilómetros mide el Ebro?</t>
-  </si>
-  <si>
-    <t>km</t>
-  </si>
-  <si>
-    <t>Más cercano</t>
-  </si>
-  <si>
-    <t>¿Cuántos kilos pesaba la calabaza más pesada del mundo (récord de 2023)?</t>
-  </si>
-  <si>
-    <t>kg</t>
-  </si>
-  <si>
-    <t>¿En qué año se publicó «Drácula», de Bram Stoker?</t>
-  </si>
-  <si>
-    <t>¿Cuántos metros mide la Torre Eiffel (con sus antenas)?</t>
-  </si>
-  <si>
-    <t>m</t>
-  </si>
-  <si>
-    <t>¿Cuántas teclas tiene un piano normal?</t>
-  </si>
-  <si>
-    <t>teclas</t>
-  </si>
-  <si>
-    <t>Sin pasarse</t>
-  </si>
-  <si>
-    <t>¿Cuántos kilómetros hay en línea recta de Madrid a Barcelona?</t>
-  </si>
-  <si>
-    <t>¿Cuántos años vivió Edgar Allan Poe?</t>
-  </si>
-  <si>
-    <t>años</t>
-  </si>
-  <si>
-    <t>¿Cuántos dientes tiene un adulto, con las muelas del juicio?</t>
-  </si>
-  <si>
-    <t>dientes</t>
-  </si>
-  <si>
-    <t>Objetivo (s)</t>
-  </si>
-  <si>
-    <t>Modo</t>
-  </si>
-  <si>
-    <t>Desaparece a los (s)</t>
-  </si>
-  <si>
-    <t>↳ Segundos a los que hay que parar el reloj.</t>
-  </si>
-  <si>
-    <t>↳ ¿Se ve el reloj?</t>
-  </si>
-  <si>
-    <t>↳ Solo con «Desaparece».</t>
-  </si>
-  <si>
-    <t>Visible</t>
-  </si>
-  <si>
-    <t>Desaparece</t>
-  </si>
-  <si>
-    <t>A ciegas</t>
-  </si>
-  <si>
-    <t>Rondas</t>
-  </si>
-  <si>
-    <t>Participan</t>
-  </si>
-  <si>
-    <t>↳ Cuántas veces se juega.</t>
-  </si>
-  <si>
-    <t>↳ Duelo: eliges a dos en el mando.</t>
-  </si>
-  <si>
-    <t>Todos</t>
-  </si>
-  <si>
-    <t>Duelo</t>
-  </si>
-  <si>
-    <t>Prueba</t>
-  </si>
-  <si>
-    <t>Herramienta</t>
-  </si>
-  <si>
-    <t>Piezas</t>
-  </si>
-  <si>
-    <t>Golpe (s)</t>
-  </si>
-  <si>
-    <t>Silencio (s)</t>
-  </si>
-  <si>
-    <t>↳ Nombre de la prueba.</t>
-  </si>
-  <si>
-    <t>↳ Qué hay que hacer (sale en la tele).</t>
-  </si>
-  <si>
-    <t>↳ Cronómetro: gana quien más aguanta. Contador: +1/−1. Contrarreloj: de uno en uno, gana el más rápido. Ninguna: eliges tú.</t>
-  </si>
-  <si>
-    <t>↳ ¿Juega cada uno o cada equipo (uno por equipo)?</t>
-  </si>
-  <si>
-    <t>↳ Vacío = los de la sección.</t>
-  </si>
-  <si>
-    <t>↳ Contrarreloj: en cada intento apuntas cuántas tiene bien (p. ej. 5 botellas).</t>
-  </si>
-  <si>
-    <t>↳ Opcional: archivo en la carpeta «Canciones» (sin .mp3). Suena al «¡Empezar!».</t>
-  </si>
-  <si>
-    <t>↳ Segundo por el que empieza la canción.</t>
-  </si>
-  <si>
-    <t>↳ Segundo del golpe (escúchalo en tu archivo). La música se calla antes y vuelve justo ahí.</t>
-  </si>
-  <si>
-    <t>↳ Cuánto se calla antes del golpe. Vacío = 3.</t>
-  </si>
-  <si>
-    <t>3 de cada equipo con un globo en el tobillo. Gana el equipo al que le quede algún globo.</t>
-  </si>
-  <si>
-    <t>Ninguna</t>
-  </si>
-  <si>
-    <t>Equipos</t>
-  </si>
-  <si>
-    <t>La revancha</t>
-  </si>
-  <si>
-    <t>¡Otra vez! Globos nuevos y los mismos tres… o tres distintos.</t>
-  </si>
-  <si>
-    <t>Uno por equipo. La caja a la cadera, por la espalda: gana quien saque todas las pelotas primero.</t>
-  </si>
-  <si>
-    <t>Twerking: la revancha</t>
-  </si>
-  <si>
-    <t>Otro de cada equipo, la caja llena otra vez.</t>
-  </si>
-  <si>
-    <t>Uno por equipo, manos atadas a la espalda y la galleta en la mesa. ¡A comer!</t>
-  </si>
-  <si>
-    <t>La galleta: segunda carrera</t>
-  </si>
-  <si>
-    <t>Otros dos, otra galleta.</t>
-  </si>
-  <si>
-    <t>Uno por equipo, primero uno y luego el otro. Ordena las 5 botellas como las tiene escondidas el presentador.</t>
-  </si>
-  <si>
-    <t>Contrarreloj</t>
-  </si>
-  <si>
-    <t>Bachata 1</t>
-  </si>
-  <si>
-    <t>En pareja. Cuando se calle la música, seguid bailando y marcad el golpe a la vez que vuelve. ¡Congelados 3 segundos!</t>
-  </si>
-  <si>
-    <t>Jugadores</t>
-  </si>
-  <si>
-    <t>Bachata 2</t>
-  </si>
-  <si>
-    <t>Otra canción, más difícil: el golpe llega cuando menos te lo esperas.</t>
-  </si>
-  <si>
-    <t>Bachata 3</t>
-  </si>
-  <si>
-    <t>La final: solo las parejas que han clavado alguna.</t>
-  </si>
-  <si>
-    <t>Plancha</t>
-  </si>
-  <si>
-    <t>Aguanta en plancha. Gana el último.</t>
-  </si>
-  <si>
-    <t>Cronómetro</t>
-  </si>
-  <si>
-    <t>Flexiones</t>
-  </si>
-  <si>
-    <t>Más flexiones en un minuto.</t>
-  </si>
-  <si>
-    <t>Contador</t>
-  </si>
-  <si>
-    <t>Sentadillas</t>
-  </si>
-  <si>
-    <t>Más sentadillas en un minuto (bajando hasta abajo).</t>
-  </si>
-  <si>
-    <t>La silla invisible</t>
-  </si>
-  <si>
-    <t>Espalda en la pared, como sentado en una silla. Gana el último.</t>
-  </si>
-  <si>
-    <t>Flamenco a ciegas</t>
-  </si>
-  <si>
-    <t>A la pata coja y con los ojos cerrados. Gana el último en apoyar el pie.</t>
-  </si>
-  <si>
-    <t>La momia</t>
-  </si>
-  <si>
-    <t>Envolved a un compañero en papel higiénico en un minuto. Gana la mejor momia.</t>
-  </si>
-  <si>
-    <t>Manzana colgante</t>
-  </si>
-  <si>
-    <t>Muerde la manzana que cuelga de un hilo, sin manos. El primero, gana.</t>
-  </si>
-  <si>
-    <t>Burpees</t>
-  </si>
-  <si>
-    <t>Más burpees en 30 segundos, entre todo el equipo.</t>
-  </si>
-  <si>
-    <t>Palabra</t>
-  </si>
-  <si>
-    <t>Prohibidas</t>
-  </si>
-  <si>
-    <t>↳ Lo que hay que adivinar. Solo la ven quien la hace y el equipo rival.</t>
-  </si>
-  <si>
-    <t>↳ Tabú: las que no se pueden decir, separadas por comas.</t>
-  </si>
-  <si>
-    <t>↳ Vacío = Tabú si hay prohibidas; si no, Mímica.</t>
-  </si>
-  <si>
-    <t>Calabaza</t>
-  </si>
-  <si>
-    <t>Halloween, naranja, vela, cara</t>
-  </si>
-  <si>
-    <t>Tabú</t>
-  </si>
-  <si>
-    <t>Vampiro</t>
-  </si>
-  <si>
-    <t>Sangre, Drácula, colmillos, murciélago</t>
-  </si>
-  <si>
-    <t>Fantasma</t>
-  </si>
-  <si>
-    <t>Sábana, espíritu, casa encantada, susto</t>
-  </si>
-  <si>
-    <t>Bruja</t>
-  </si>
-  <si>
-    <t>Escoba, caldero, sombrero, hechizo</t>
-  </si>
-  <si>
-    <t>Telaraña</t>
-  </si>
-  <si>
-    <t>Araña, hilo, red, tejer</t>
-  </si>
-  <si>
-    <t>Esqueleto</t>
-  </si>
-  <si>
-    <t>Huesos, calavera, cuerpo, muerto</t>
-  </si>
-  <si>
-    <t>Cementerio</t>
-  </si>
-  <si>
-    <t>Tumba, muertos, lápida, enterrar</t>
-  </si>
-  <si>
-    <t>Murciélago</t>
-  </si>
-  <si>
-    <t>Vampiro, volar, cueva, noche</t>
-  </si>
-  <si>
-    <t>Caramelo</t>
-  </si>
-  <si>
-    <t>Dulce, azúcar, chuche, truco o trato</t>
-  </si>
-  <si>
-    <t>Luna llena</t>
-  </si>
-  <si>
-    <t>Noche, lobo, redonda, cielo</t>
-  </si>
-  <si>
-    <t>Hombre lobo</t>
-  </si>
-  <si>
-    <t>Mímica</t>
-  </si>
-  <si>
-    <t>Momia</t>
-  </si>
-  <si>
-    <t>Zombi</t>
-  </si>
-  <si>
-    <t>Tallar una calabaza</t>
-  </si>
-  <si>
-    <t>Pedir caramelos</t>
-  </si>
-  <si>
-    <t>Volar en escoba</t>
-  </si>
-  <si>
-    <t>Ver una peli de miedo</t>
-  </si>
-  <si>
-    <t>Salir de un ataúd</t>
-  </si>
-  <si>
-    <t>Gato negro</t>
-  </si>
-  <si>
-    <t>Poción</t>
-  </si>
-  <si>
-    <t>Descríbelo</t>
-  </si>
-  <si>
-    <t>Disfraz</t>
-  </si>
-  <si>
-    <t>Escalofrío</t>
-  </si>
-  <si>
-    <t>Casa encantada</t>
-  </si>
-  <si>
-    <t>Ataúd</t>
   </si>
   <si>
     <t>Tararéalo</t>
@@ -6294,7 +6297,7 @@
   <sheetPr>
     <tabColor rgb="FF1E63D6"/>
   </sheetPr>
-  <dimension ref="A1:K200"/>
+  <dimension ref="A1:I200"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -6302,11 +6305,10 @@
     <col min="3" max="3" width="14" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
     <col min="7" max="7" width="18" customWidth="1"/>
-    <col min="10" max="10" width="10" customWidth="1"/>
-    <col min="11" max="11" width="22" customWidth="1"/>
+    <col min="9" max="9" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="30" customHeight="1" spans="1:9" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>367</v>
       </c>
@@ -6332,200 +6334,176 @@
         <v>156</v>
       </c>
       <c r="I1" s="10" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2" ht="42" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="11" t="s">
         <v>370</v>
       </c>
-      <c r="J1" s="10" t="s">
+      <c r="B2" s="11" t="s">
         <v>371</v>
       </c>
-      <c r="K1" s="10" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="2" ht="42" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
+      <c r="C2" s="11" t="s">
         <v>372</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="D2" s="11" t="s">
         <v>373</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="E2" s="11" t="s">
         <v>374</v>
       </c>
-      <c r="D2" s="11" t="s">
+      <c r="F2" s="11" t="s">
         <v>375</v>
       </c>
-      <c r="E2" s="11" t="s">
+      <c r="G2" s="11" t="s">
         <v>376</v>
       </c>
-      <c r="F2" s="11" t="s">
+      <c r="H2" s="11" t="s">
         <v>377</v>
       </c>
-      <c r="G2" s="11" t="s">
-        <v>378</v>
-      </c>
-      <c r="H2" s="11" t="s">
-        <v>379</v>
-      </c>
       <c r="I2" s="11" t="s">
-        <v>380</v>
-      </c>
-      <c r="J2" s="11" t="s">
-        <v>381</v>
-      </c>
-      <c r="K2" s="11" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
         <v>90</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>384</v>
+        <v>380</v>
       </c>
       <c r="E3" s="12"/>
       <c r="F3" s="12"/>
       <c r="G3" s="12"/>
       <c r="H3" s="12"/>
-      <c r="I3" s="12"/>
-      <c r="J3" s="12"/>
-      <c r="K3" s="12" t="s">
+      <c r="I3" s="12" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>385</v>
+        <v>381</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>386</v>
+        <v>382</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>384</v>
+        <v>380</v>
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="12"/>
       <c r="G4" s="12"/>
       <c r="H4" s="12"/>
-      <c r="I4" s="12"/>
-      <c r="J4" s="12"/>
-      <c r="K4" s="12" t="s">
+      <c r="I4" s="12" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
         <v>100</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>387</v>
+        <v>383</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>384</v>
+        <v>380</v>
       </c>
       <c r="E5" s="12"/>
       <c r="F5" s="12"/>
       <c r="G5" s="12"/>
       <c r="H5" s="12"/>
-      <c r="I5" s="12"/>
-      <c r="J5" s="12"/>
-      <c r="K5" s="12" t="s">
+      <c r="I5" s="12" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>388</v>
+        <v>384</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>389</v>
+        <v>385</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>384</v>
+        <v>380</v>
       </c>
       <c r="E6" s="12"/>
       <c r="F6" s="12"/>
       <c r="G6" s="12"/>
       <c r="H6" s="12"/>
-      <c r="I6" s="12"/>
-      <c r="J6" s="12"/>
-      <c r="K6" s="12" t="s">
+      <c r="I6" s="12" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
         <v>107</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>390</v>
+        <v>386</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>384</v>
+        <v>380</v>
       </c>
       <c r="E7" s="12"/>
       <c r="F7" s="12"/>
       <c r="G7" s="12"/>
       <c r="H7" s="12"/>
-      <c r="I7" s="12"/>
-      <c r="J7" s="12"/>
-      <c r="K7" s="12" t="s">
+      <c r="I7" s="12" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>391</v>
+        <v>387</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>392</v>
+        <v>388</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>384</v>
+        <v>380</v>
       </c>
       <c r="E8" s="12"/>
       <c r="F8" s="12"/>
       <c r="G8" s="12"/>
       <c r="H8" s="12"/>
-      <c r="I8" s="12"/>
-      <c r="J8" s="12"/>
-      <c r="K8" s="12" t="s">
+      <c r="I8" s="12" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
         <v>109</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>384</v>
+        <v>380</v>
       </c>
       <c r="E9" s="12"/>
       <c r="F9" s="12">
@@ -6533,24 +6511,22 @@
       </c>
       <c r="G9" s="12"/>
       <c r="H9" s="12"/>
-      <c r="I9" s="12"/>
-      <c r="J9" s="12"/>
-      <c r="K9" s="12" t="s">
+      <c r="I9" s="12" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>395</v>
+        <v>391</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>396</v>
+        <v>392</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>383</v>
+        <v>393</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="E10" s="12"/>
       <c r="F10" s="12"/>
@@ -6560,24 +6536,22 @@
       <c r="H10" s="12">
         <v>0</v>
       </c>
-      <c r="I10" s="12"/>
-      <c r="J10" s="12"/>
-      <c r="K10" s="12" t="s">
+      <c r="I10" s="12" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>383</v>
+        <v>393</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="E11" s="12"/>
       <c r="F11" s="12"/>
@@ -6587,40 +6561,36 @@
       <c r="H11" s="12">
         <v>0</v>
       </c>
-      <c r="I11" s="12"/>
-      <c r="J11" s="12"/>
-      <c r="K11" s="12" t="s">
+      <c r="I11" s="12" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
+        <v>399</v>
+      </c>
+      <c r="B12" s="14" t="s">
         <v>400</v>
       </c>
-      <c r="B12" s="14" t="s">
-        <v>401</v>
-      </c>
       <c r="C12" s="12" t="s">
-        <v>383</v>
+        <v>393</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="E12" s="12"/>
       <c r="F12" s="12"/>
       <c r="G12" s="12" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="H12" s="12">
         <v>0</v>
       </c>
-      <c r="I12" s="12"/>
-      <c r="J12" s="12"/>
-      <c r="K12" s="12" t="s">
+      <c r="I12" s="12" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
         <v>402</v>
       </c>
@@ -6631,19 +6601,17 @@
         <v>404</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="E13" s="12"/>
       <c r="F13" s="12"/>
       <c r="G13" s="12"/>
       <c r="H13" s="12"/>
-      <c r="I13" s="12"/>
-      <c r="J13" s="12"/>
-      <c r="K13" s="12" t="s">
+      <c r="I13" s="12" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
         <v>405</v>
       </c>
@@ -6654,7 +6622,7 @@
         <v>407</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>384</v>
+        <v>380</v>
       </c>
       <c r="E14" s="12">
         <v>5</v>
@@ -6662,13 +6630,11 @@
       <c r="F14" s="12"/>
       <c r="G14" s="12"/>
       <c r="H14" s="12"/>
-      <c r="I14" s="12"/>
-      <c r="J14" s="12"/>
-      <c r="K14" s="12" t="s">
+      <c r="I14" s="12" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="12" t="s">
         <v>408</v>
       </c>
@@ -6679,19 +6645,17 @@
         <v>407</v>
       </c>
       <c r="D15" s="12" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="E15" s="12"/>
       <c r="F15" s="12"/>
       <c r="G15" s="12"/>
       <c r="H15" s="12"/>
-      <c r="I15" s="12"/>
-      <c r="J15" s="12"/>
-      <c r="K15" s="12" t="s">
+      <c r="I15" s="12" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="12" t="s">
         <v>410</v>
       </c>
@@ -6702,19 +6666,17 @@
         <v>404</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="E16" s="12"/>
       <c r="F16" s="12"/>
       <c r="G16" s="12"/>
       <c r="H16" s="12"/>
-      <c r="I16" s="12"/>
-      <c r="J16" s="12"/>
-      <c r="K16" s="12" t="s">
+      <c r="I16" s="12" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="12" t="s">
         <v>412</v>
       </c>
@@ -6725,19 +6687,17 @@
         <v>404</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="E17" s="12"/>
       <c r="F17" s="12"/>
       <c r="G17" s="12"/>
       <c r="H17" s="12"/>
-      <c r="I17" s="12"/>
-      <c r="J17" s="12"/>
-      <c r="K17" s="12" t="s">
+      <c r="I17" s="12" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="12" t="s">
         <v>414</v>
       </c>
@@ -6745,10 +6705,10 @@
         <v>415</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>384</v>
+        <v>380</v>
       </c>
       <c r="E18" s="12">
         <v>5</v>
@@ -6756,13 +6716,11 @@
       <c r="F18" s="12"/>
       <c r="G18" s="12"/>
       <c r="H18" s="12"/>
-      <c r="I18" s="12"/>
-      <c r="J18" s="12"/>
-      <c r="K18" s="12" t="s">
+      <c r="I18" s="12" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
         <v>416</v>
       </c>
@@ -6770,22 +6728,20 @@
         <v>417</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="E19" s="12"/>
       <c r="F19" s="12"/>
       <c r="G19" s="12"/>
       <c r="H19" s="12"/>
-      <c r="I19" s="12"/>
-      <c r="J19" s="12"/>
-      <c r="K19" s="12" t="s">
+      <c r="I19" s="12" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="12" t="s">
         <v>418</v>
       </c>
@@ -6796,7 +6752,7 @@
         <v>407</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>384</v>
+        <v>380</v>
       </c>
       <c r="E20" s="12">
         <v>5</v>
@@ -6804,13 +6760,11 @@
       <c r="F20" s="12"/>
       <c r="G20" s="12"/>
       <c r="H20" s="12"/>
-      <c r="I20" s="12"/>
-      <c r="J20" s="12"/>
-      <c r="K20" s="12" t="s">
+      <c r="I20" s="12" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="12"/>
       <c r="B21" s="14"/>
       <c r="C21" s="12"/>
@@ -6820,10 +6774,8 @@
       <c r="G21" s="12"/>
       <c r="H21" s="12"/>
       <c r="I21" s="12"/>
-      <c r="J21" s="12"/>
-      <c r="K21" s="12"/>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="12"/>
       <c r="B22" s="14"/>
       <c r="C22" s="12"/>
@@ -6833,10 +6785,8 @@
       <c r="G22" s="12"/>
       <c r="H22" s="12"/>
       <c r="I22" s="12"/>
-      <c r="J22" s="12"/>
-      <c r="K22" s="12"/>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="12"/>
       <c r="B23" s="14"/>
       <c r="C23" s="12"/>
@@ -6846,10 +6796,8 @@
       <c r="G23" s="12"/>
       <c r="H23" s="12"/>
       <c r="I23" s="12"/>
-      <c r="J23" s="12"/>
-      <c r="K23" s="12"/>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="12"/>
       <c r="B24" s="14"/>
       <c r="C24" s="12"/>
@@ -6859,10 +6807,8 @@
       <c r="G24" s="12"/>
       <c r="H24" s="12"/>
       <c r="I24" s="12"/>
-      <c r="J24" s="12"/>
-      <c r="K24" s="12"/>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="12"/>
       <c r="B25" s="14"/>
       <c r="C25" s="12"/>
@@ -6872,10 +6818,8 @@
       <c r="G25" s="12"/>
       <c r="H25" s="12"/>
       <c r="I25" s="12"/>
-      <c r="J25" s="12"/>
-      <c r="K25" s="12"/>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="12"/>
       <c r="B26" s="14"/>
       <c r="C26" s="12"/>
@@ -6885,10 +6829,8 @@
       <c r="G26" s="12"/>
       <c r="H26" s="12"/>
       <c r="I26" s="12"/>
-      <c r="J26" s="12"/>
-      <c r="K26" s="12"/>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="12"/>
       <c r="B27" s="14"/>
       <c r="C27" s="12"/>
@@ -6898,10 +6840,8 @@
       <c r="G27" s="12"/>
       <c r="H27" s="12"/>
       <c r="I27" s="12"/>
-      <c r="J27" s="12"/>
-      <c r="K27" s="12"/>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="12"/>
       <c r="B28" s="14"/>
       <c r="C28" s="12"/>
@@ -6911,10 +6851,8 @@
       <c r="G28" s="12"/>
       <c r="H28" s="12"/>
       <c r="I28" s="12"/>
-      <c r="J28" s="12"/>
-      <c r="K28" s="12"/>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="12"/>
       <c r="B29" s="14"/>
       <c r="C29" s="12"/>
@@ -6924,10 +6862,8 @@
       <c r="G29" s="12"/>
       <c r="H29" s="12"/>
       <c r="I29" s="12"/>
-      <c r="J29" s="12"/>
-      <c r="K29" s="12"/>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="12"/>
       <c r="B30" s="14"/>
       <c r="C30" s="12"/>
@@ -6937,10 +6873,8 @@
       <c r="G30" s="12"/>
       <c r="H30" s="12"/>
       <c r="I30" s="12"/>
-      <c r="J30" s="12"/>
-      <c r="K30" s="12"/>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="12"/>
       <c r="B31" s="14"/>
       <c r="C31" s="12"/>
@@ -6950,10 +6884,8 @@
       <c r="G31" s="12"/>
       <c r="H31" s="12"/>
       <c r="I31" s="12"/>
-      <c r="J31" s="12"/>
-      <c r="K31" s="12"/>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="12"/>
       <c r="B32" s="14"/>
       <c r="C32" s="12"/>
@@ -6963,10 +6895,8 @@
       <c r="G32" s="12"/>
       <c r="H32" s="12"/>
       <c r="I32" s="12"/>
-      <c r="J32" s="12"/>
-      <c r="K32" s="12"/>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="12"/>
       <c r="B33" s="14"/>
       <c r="C33" s="12"/>
@@ -6976,10 +6906,8 @@
       <c r="G33" s="12"/>
       <c r="H33" s="12"/>
       <c r="I33" s="12"/>
-      <c r="J33" s="12"/>
-      <c r="K33" s="12"/>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="12"/>
       <c r="B34" s="14"/>
       <c r="C34" s="12"/>
@@ -6989,10 +6917,8 @@
       <c r="G34" s="12"/>
       <c r="H34" s="12"/>
       <c r="I34" s="12"/>
-      <c r="J34" s="12"/>
-      <c r="K34" s="12"/>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="12"/>
       <c r="B35" s="14"/>
       <c r="C35" s="12"/>
@@ -7002,10 +6928,8 @@
       <c r="G35" s="12"/>
       <c r="H35" s="12"/>
       <c r="I35" s="12"/>
-      <c r="J35" s="12"/>
-      <c r="K35" s="12"/>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="12"/>
       <c r="B36" s="14"/>
       <c r="C36" s="12"/>
@@ -7015,10 +6939,8 @@
       <c r="G36" s="12"/>
       <c r="H36" s="12"/>
       <c r="I36" s="12"/>
-      <c r="J36" s="12"/>
-      <c r="K36" s="12"/>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="12"/>
       <c r="B37" s="14"/>
       <c r="C37" s="12"/>
@@ -7028,10 +6950,8 @@
       <c r="G37" s="12"/>
       <c r="H37" s="12"/>
       <c r="I37" s="12"/>
-      <c r="J37" s="12"/>
-      <c r="K37" s="12"/>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="12"/>
       <c r="B38" s="14"/>
       <c r="C38" s="12"/>
@@ -7041,10 +6961,8 @@
       <c r="G38" s="12"/>
       <c r="H38" s="12"/>
       <c r="I38" s="12"/>
-      <c r="J38" s="12"/>
-      <c r="K38" s="12"/>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="12"/>
       <c r="B39" s="14"/>
       <c r="C39" s="12"/>
@@ -7054,10 +6972,8 @@
       <c r="G39" s="12"/>
       <c r="H39" s="12"/>
       <c r="I39" s="12"/>
-      <c r="J39" s="12"/>
-      <c r="K39" s="12"/>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="12"/>
       <c r="B40" s="14"/>
       <c r="C40" s="12"/>
@@ -7067,10 +6983,8 @@
       <c r="G40" s="12"/>
       <c r="H40" s="12"/>
       <c r="I40" s="12"/>
-      <c r="J40" s="12"/>
-      <c r="K40" s="12"/>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="12"/>
       <c r="B41" s="14"/>
       <c r="C41" s="12"/>
@@ -7080,10 +6994,8 @@
       <c r="G41" s="12"/>
       <c r="H41" s="12"/>
       <c r="I41" s="12"/>
-      <c r="J41" s="12"/>
-      <c r="K41" s="12"/>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="12"/>
       <c r="B42" s="14"/>
       <c r="C42" s="12"/>
@@ -7093,10 +7005,8 @@
       <c r="G42" s="12"/>
       <c r="H42" s="12"/>
       <c r="I42" s="12"/>
-      <c r="J42" s="12"/>
-      <c r="K42" s="12"/>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="12"/>
       <c r="B43" s="14"/>
       <c r="C43" s="12"/>
@@ -7106,10 +7016,8 @@
       <c r="G43" s="12"/>
       <c r="H43" s="12"/>
       <c r="I43" s="12"/>
-      <c r="J43" s="12"/>
-      <c r="K43" s="12"/>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="12"/>
       <c r="B44" s="14"/>
       <c r="C44" s="12"/>
@@ -7119,10 +7027,8 @@
       <c r="G44" s="12"/>
       <c r="H44" s="12"/>
       <c r="I44" s="12"/>
-      <c r="J44" s="12"/>
-      <c r="K44" s="12"/>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="12"/>
       <c r="B45" s="14"/>
       <c r="C45" s="12"/>
@@ -7132,10 +7038,8 @@
       <c r="G45" s="12"/>
       <c r="H45" s="12"/>
       <c r="I45" s="12"/>
-      <c r="J45" s="12"/>
-      <c r="K45" s="12"/>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="12"/>
       <c r="B46" s="14"/>
       <c r="C46" s="12"/>
@@ -7145,10 +7049,8 @@
       <c r="G46" s="12"/>
       <c r="H46" s="12"/>
       <c r="I46" s="12"/>
-      <c r="J46" s="12"/>
-      <c r="K46" s="12"/>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="12"/>
       <c r="B47" s="14"/>
       <c r="C47" s="12"/>
@@ -7158,10 +7060,8 @@
       <c r="G47" s="12"/>
       <c r="H47" s="12"/>
       <c r="I47" s="12"/>
-      <c r="J47" s="12"/>
-      <c r="K47" s="12"/>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="12"/>
       <c r="B48" s="14"/>
       <c r="C48" s="12"/>
@@ -7171,10 +7071,8 @@
       <c r="G48" s="12"/>
       <c r="H48" s="12"/>
       <c r="I48" s="12"/>
-      <c r="J48" s="12"/>
-      <c r="K48" s="12"/>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" s="12"/>
       <c r="B49" s="14"/>
       <c r="C49" s="12"/>
@@ -7184,10 +7082,8 @@
       <c r="G49" s="12"/>
       <c r="H49" s="12"/>
       <c r="I49" s="12"/>
-      <c r="J49" s="12"/>
-      <c r="K49" s="12"/>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" s="12"/>
       <c r="B50" s="14"/>
       <c r="C50" s="12"/>
@@ -7197,10 +7093,8 @@
       <c r="G50" s="12"/>
       <c r="H50" s="12"/>
       <c r="I50" s="12"/>
-      <c r="J50" s="12"/>
-      <c r="K50" s="12"/>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" s="12"/>
       <c r="B51" s="14"/>
       <c r="C51" s="12"/>
@@ -7210,10 +7104,8 @@
       <c r="G51" s="12"/>
       <c r="H51" s="12"/>
       <c r="I51" s="12"/>
-      <c r="J51" s="12"/>
-      <c r="K51" s="12"/>
-    </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" s="12"/>
       <c r="B52" s="14"/>
       <c r="C52" s="12"/>
@@ -7223,10 +7115,8 @@
       <c r="G52" s="12"/>
       <c r="H52" s="12"/>
       <c r="I52" s="12"/>
-      <c r="J52" s="12"/>
-      <c r="K52" s="12"/>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" s="12"/>
       <c r="B53" s="14"/>
       <c r="C53" s="12"/>
@@ -7236,10 +7126,8 @@
       <c r="G53" s="12"/>
       <c r="H53" s="12"/>
       <c r="I53" s="12"/>
-      <c r="J53" s="12"/>
-      <c r="K53" s="12"/>
-    </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" s="12"/>
       <c r="B54" s="14"/>
       <c r="C54" s="12"/>
@@ -7249,10 +7137,8 @@
       <c r="G54" s="12"/>
       <c r="H54" s="12"/>
       <c r="I54" s="12"/>
-      <c r="J54" s="12"/>
-      <c r="K54" s="12"/>
-    </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" s="12"/>
       <c r="B55" s="14"/>
       <c r="C55" s="12"/>
@@ -7262,10 +7148,8 @@
       <c r="G55" s="12"/>
       <c r="H55" s="12"/>
       <c r="I55" s="12"/>
-      <c r="J55" s="12"/>
-      <c r="K55" s="12"/>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" s="12"/>
       <c r="B56" s="14"/>
       <c r="C56" s="12"/>
@@ -7275,10 +7159,8 @@
       <c r="G56" s="12"/>
       <c r="H56" s="12"/>
       <c r="I56" s="12"/>
-      <c r="J56" s="12"/>
-      <c r="K56" s="12"/>
-    </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" s="12"/>
       <c r="B57" s="14"/>
       <c r="C57" s="12"/>
@@ -7288,10 +7170,8 @@
       <c r="G57" s="12"/>
       <c r="H57" s="12"/>
       <c r="I57" s="12"/>
-      <c r="J57" s="12"/>
-      <c r="K57" s="12"/>
-    </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" s="12"/>
       <c r="B58" s="14"/>
       <c r="C58" s="12"/>
@@ -7301,10 +7181,8 @@
       <c r="G58" s="12"/>
       <c r="H58" s="12"/>
       <c r="I58" s="12"/>
-      <c r="J58" s="12"/>
-      <c r="K58" s="12"/>
-    </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" s="12"/>
       <c r="B59" s="14"/>
       <c r="C59" s="12"/>
@@ -7314,10 +7192,8 @@
       <c r="G59" s="12"/>
       <c r="H59" s="12"/>
       <c r="I59" s="12"/>
-      <c r="J59" s="12"/>
-      <c r="K59" s="12"/>
-    </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" s="12"/>
       <c r="B60" s="14"/>
       <c r="C60" s="12"/>
@@ -7327,10 +7203,8 @@
       <c r="G60" s="12"/>
       <c r="H60" s="12"/>
       <c r="I60" s="12"/>
-      <c r="J60" s="12"/>
-      <c r="K60" s="12"/>
-    </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" s="12"/>
       <c r="B61" s="14"/>
       <c r="C61" s="12"/>
@@ -7340,10 +7214,8 @@
       <c r="G61" s="12"/>
       <c r="H61" s="12"/>
       <c r="I61" s="12"/>
-      <c r="J61" s="12"/>
-      <c r="K61" s="12"/>
-    </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" s="12"/>
       <c r="B62" s="14"/>
       <c r="C62" s="12"/>
@@ -7353,10 +7225,8 @@
       <c r="G62" s="12"/>
       <c r="H62" s="12"/>
       <c r="I62" s="12"/>
-      <c r="J62" s="12"/>
-      <c r="K62" s="12"/>
-    </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63" s="12"/>
       <c r="B63" s="14"/>
       <c r="C63" s="12"/>
@@ -7366,10 +7236,8 @@
       <c r="G63" s="12"/>
       <c r="H63" s="12"/>
       <c r="I63" s="12"/>
-      <c r="J63" s="12"/>
-      <c r="K63" s="12"/>
-    </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" s="12"/>
       <c r="B64" s="14"/>
       <c r="C64" s="12"/>
@@ -7379,10 +7247,8 @@
       <c r="G64" s="12"/>
       <c r="H64" s="12"/>
       <c r="I64" s="12"/>
-      <c r="J64" s="12"/>
-      <c r="K64" s="12"/>
-    </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" s="12"/>
       <c r="B65" s="14"/>
       <c r="C65" s="12"/>
@@ -7392,10 +7258,8 @@
       <c r="G65" s="12"/>
       <c r="H65" s="12"/>
       <c r="I65" s="12"/>
-      <c r="J65" s="12"/>
-      <c r="K65" s="12"/>
-    </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66" s="12"/>
       <c r="B66" s="14"/>
       <c r="C66" s="12"/>
@@ -7405,10 +7269,8 @@
       <c r="G66" s="12"/>
       <c r="H66" s="12"/>
       <c r="I66" s="12"/>
-      <c r="J66" s="12"/>
-      <c r="K66" s="12"/>
-    </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67" s="12"/>
       <c r="B67" s="14"/>
       <c r="C67" s="12"/>
@@ -7418,10 +7280,8 @@
       <c r="G67" s="12"/>
       <c r="H67" s="12"/>
       <c r="I67" s="12"/>
-      <c r="J67" s="12"/>
-      <c r="K67" s="12"/>
-    </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A68" s="12"/>
       <c r="B68" s="14"/>
       <c r="C68" s="12"/>
@@ -7431,10 +7291,8 @@
       <c r="G68" s="12"/>
       <c r="H68" s="12"/>
       <c r="I68" s="12"/>
-      <c r="J68" s="12"/>
-      <c r="K68" s="12"/>
-    </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" s="12"/>
       <c r="B69" s="14"/>
       <c r="C69" s="12"/>
@@ -7444,10 +7302,8 @@
       <c r="G69" s="12"/>
       <c r="H69" s="12"/>
       <c r="I69" s="12"/>
-      <c r="J69" s="12"/>
-      <c r="K69" s="12"/>
-    </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70" s="12"/>
       <c r="B70" s="14"/>
       <c r="C70" s="12"/>
@@ -7457,10 +7313,8 @@
       <c r="G70" s="12"/>
       <c r="H70" s="12"/>
       <c r="I70" s="12"/>
-      <c r="J70" s="12"/>
-      <c r="K70" s="12"/>
-    </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71" s="12"/>
       <c r="B71" s="14"/>
       <c r="C71" s="12"/>
@@ -7470,10 +7324,8 @@
       <c r="G71" s="12"/>
       <c r="H71" s="12"/>
       <c r="I71" s="12"/>
-      <c r="J71" s="12"/>
-      <c r="K71" s="12"/>
-    </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" s="12"/>
       <c r="B72" s="14"/>
       <c r="C72" s="12"/>
@@ -7483,10 +7335,8 @@
       <c r="G72" s="12"/>
       <c r="H72" s="12"/>
       <c r="I72" s="12"/>
-      <c r="J72" s="12"/>
-      <c r="K72" s="12"/>
-    </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73" s="12"/>
       <c r="B73" s="14"/>
       <c r="C73" s="12"/>
@@ -7496,10 +7346,8 @@
       <c r="G73" s="12"/>
       <c r="H73" s="12"/>
       <c r="I73" s="12"/>
-      <c r="J73" s="12"/>
-      <c r="K73" s="12"/>
-    </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74" s="12"/>
       <c r="B74" s="14"/>
       <c r="C74" s="12"/>
@@ -7509,10 +7357,8 @@
       <c r="G74" s="12"/>
       <c r="H74" s="12"/>
       <c r="I74" s="12"/>
-      <c r="J74" s="12"/>
-      <c r="K74" s="12"/>
-    </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75" s="12"/>
       <c r="B75" s="14"/>
       <c r="C75" s="12"/>
@@ -7522,10 +7368,8 @@
       <c r="G75" s="12"/>
       <c r="H75" s="12"/>
       <c r="I75" s="12"/>
-      <c r="J75" s="12"/>
-      <c r="K75" s="12"/>
-    </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A76" s="12"/>
       <c r="B76" s="14"/>
       <c r="C76" s="12"/>
@@ -7535,10 +7379,8 @@
       <c r="G76" s="12"/>
       <c r="H76" s="12"/>
       <c r="I76" s="12"/>
-      <c r="J76" s="12"/>
-      <c r="K76" s="12"/>
-    </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A77" s="12"/>
       <c r="B77" s="14"/>
       <c r="C77" s="12"/>
@@ -7548,10 +7390,8 @@
       <c r="G77" s="12"/>
       <c r="H77" s="12"/>
       <c r="I77" s="12"/>
-      <c r="J77" s="12"/>
-      <c r="K77" s="12"/>
-    </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A78" s="12"/>
       <c r="B78" s="14"/>
       <c r="C78" s="12"/>
@@ -7561,10 +7401,8 @@
       <c r="G78" s="12"/>
       <c r="H78" s="12"/>
       <c r="I78" s="12"/>
-      <c r="J78" s="12"/>
-      <c r="K78" s="12"/>
-    </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A79" s="12"/>
       <c r="B79" s="14"/>
       <c r="C79" s="12"/>
@@ -7574,10 +7412,8 @@
       <c r="G79" s="12"/>
       <c r="H79" s="12"/>
       <c r="I79" s="12"/>
-      <c r="J79" s="12"/>
-      <c r="K79" s="12"/>
-    </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80" s="12"/>
       <c r="B80" s="14"/>
       <c r="C80" s="12"/>
@@ -7587,10 +7423,8 @@
       <c r="G80" s="12"/>
       <c r="H80" s="12"/>
       <c r="I80" s="12"/>
-      <c r="J80" s="12"/>
-      <c r="K80" s="12"/>
-    </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A81" s="12"/>
       <c r="B81" s="14"/>
       <c r="C81" s="12"/>
@@ -7600,10 +7434,8 @@
       <c r="G81" s="12"/>
       <c r="H81" s="12"/>
       <c r="I81" s="12"/>
-      <c r="J81" s="12"/>
-      <c r="K81" s="12"/>
-    </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82" s="12"/>
       <c r="B82" s="14"/>
       <c r="C82" s="12"/>
@@ -7613,10 +7445,8 @@
       <c r="G82" s="12"/>
       <c r="H82" s="12"/>
       <c r="I82" s="12"/>
-      <c r="J82" s="12"/>
-      <c r="K82" s="12"/>
-    </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83" s="12"/>
       <c r="B83" s="14"/>
       <c r="C83" s="12"/>
@@ -7626,10 +7456,8 @@
       <c r="G83" s="12"/>
       <c r="H83" s="12"/>
       <c r="I83" s="12"/>
-      <c r="J83" s="12"/>
-      <c r="K83" s="12"/>
-    </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A84" s="12"/>
       <c r="B84" s="14"/>
       <c r="C84" s="12"/>
@@ -7639,10 +7467,8 @@
       <c r="G84" s="12"/>
       <c r="H84" s="12"/>
       <c r="I84" s="12"/>
-      <c r="J84" s="12"/>
-      <c r="K84" s="12"/>
-    </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A85" s="12"/>
       <c r="B85" s="14"/>
       <c r="C85" s="12"/>
@@ -7652,10 +7478,8 @@
       <c r="G85" s="12"/>
       <c r="H85" s="12"/>
       <c r="I85" s="12"/>
-      <c r="J85" s="12"/>
-      <c r="K85" s="12"/>
-    </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A86" s="12"/>
       <c r="B86" s="14"/>
       <c r="C86" s="12"/>
@@ -7665,10 +7489,8 @@
       <c r="G86" s="12"/>
       <c r="H86" s="12"/>
       <c r="I86" s="12"/>
-      <c r="J86" s="12"/>
-      <c r="K86" s="12"/>
-    </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A87" s="12"/>
       <c r="B87" s="14"/>
       <c r="C87" s="12"/>
@@ -7678,10 +7500,8 @@
       <c r="G87" s="12"/>
       <c r="H87" s="12"/>
       <c r="I87" s="12"/>
-      <c r="J87" s="12"/>
-      <c r="K87" s="12"/>
-    </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88" s="12"/>
       <c r="B88" s="14"/>
       <c r="C88" s="12"/>
@@ -7691,10 +7511,8 @@
       <c r="G88" s="12"/>
       <c r="H88" s="12"/>
       <c r="I88" s="12"/>
-      <c r="J88" s="12"/>
-      <c r="K88" s="12"/>
-    </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A89" s="12"/>
       <c r="B89" s="14"/>
       <c r="C89" s="12"/>
@@ -7704,10 +7522,8 @@
       <c r="G89" s="12"/>
       <c r="H89" s="12"/>
       <c r="I89" s="12"/>
-      <c r="J89" s="12"/>
-      <c r="K89" s="12"/>
-    </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A90" s="12"/>
       <c r="B90" s="14"/>
       <c r="C90" s="12"/>
@@ -7717,10 +7533,8 @@
       <c r="G90" s="12"/>
       <c r="H90" s="12"/>
       <c r="I90" s="12"/>
-      <c r="J90" s="12"/>
-      <c r="K90" s="12"/>
-    </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91" s="12"/>
       <c r="B91" s="14"/>
       <c r="C91" s="12"/>
@@ -7730,10 +7544,8 @@
       <c r="G91" s="12"/>
       <c r="H91" s="12"/>
       <c r="I91" s="12"/>
-      <c r="J91" s="12"/>
-      <c r="K91" s="12"/>
-    </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A92" s="12"/>
       <c r="B92" s="14"/>
       <c r="C92" s="12"/>
@@ -7743,10 +7555,8 @@
       <c r="G92" s="12"/>
       <c r="H92" s="12"/>
       <c r="I92" s="12"/>
-      <c r="J92" s="12"/>
-      <c r="K92" s="12"/>
-    </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A93" s="12"/>
       <c r="B93" s="14"/>
       <c r="C93" s="12"/>
@@ -7756,10 +7566,8 @@
       <c r="G93" s="12"/>
       <c r="H93" s="12"/>
       <c r="I93" s="12"/>
-      <c r="J93" s="12"/>
-      <c r="K93" s="12"/>
-    </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A94" s="12"/>
       <c r="B94" s="14"/>
       <c r="C94" s="12"/>
@@ -7769,10 +7577,8 @@
       <c r="G94" s="12"/>
       <c r="H94" s="12"/>
       <c r="I94" s="12"/>
-      <c r="J94" s="12"/>
-      <c r="K94" s="12"/>
-    </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A95" s="12"/>
       <c r="B95" s="14"/>
       <c r="C95" s="12"/>
@@ -7782,10 +7588,8 @@
       <c r="G95" s="12"/>
       <c r="H95" s="12"/>
       <c r="I95" s="12"/>
-      <c r="J95" s="12"/>
-      <c r="K95" s="12"/>
-    </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="96" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A96" s="12"/>
       <c r="B96" s="14"/>
       <c r="C96" s="12"/>
@@ -7795,10 +7599,8 @@
       <c r="G96" s="12"/>
       <c r="H96" s="12"/>
       <c r="I96" s="12"/>
-      <c r="J96" s="12"/>
-      <c r="K96" s="12"/>
-    </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A97" s="12"/>
       <c r="B97" s="14"/>
       <c r="C97" s="12"/>
@@ -7808,10 +7610,8 @@
       <c r="G97" s="12"/>
       <c r="H97" s="12"/>
       <c r="I97" s="12"/>
-      <c r="J97" s="12"/>
-      <c r="K97" s="12"/>
-    </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="98" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A98" s="12"/>
       <c r="B98" s="14"/>
       <c r="C98" s="12"/>
@@ -7821,10 +7621,8 @@
       <c r="G98" s="12"/>
       <c r="H98" s="12"/>
       <c r="I98" s="12"/>
-      <c r="J98" s="12"/>
-      <c r="K98" s="12"/>
-    </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A99" s="12"/>
       <c r="B99" s="14"/>
       <c r="C99" s="12"/>
@@ -7834,10 +7632,8 @@
       <c r="G99" s="12"/>
       <c r="H99" s="12"/>
       <c r="I99" s="12"/>
-      <c r="J99" s="12"/>
-      <c r="K99" s="12"/>
-    </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A100" s="12"/>
       <c r="B100" s="14"/>
       <c r="C100" s="12"/>
@@ -7847,10 +7643,8 @@
       <c r="G100" s="12"/>
       <c r="H100" s="12"/>
       <c r="I100" s="12"/>
-      <c r="J100" s="12"/>
-      <c r="K100" s="12"/>
-    </row>
-    <row r="101" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A101" s="12"/>
       <c r="B101" s="14"/>
       <c r="C101" s="12"/>
@@ -7860,10 +7654,8 @@
       <c r="G101" s="12"/>
       <c r="H101" s="12"/>
       <c r="I101" s="12"/>
-      <c r="J101" s="12"/>
-      <c r="K101" s="12"/>
-    </row>
-    <row r="102" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="102" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A102" s="12"/>
       <c r="B102" s="14"/>
       <c r="C102" s="12"/>
@@ -7873,10 +7665,8 @@
       <c r="G102" s="12"/>
       <c r="H102" s="12"/>
       <c r="I102" s="12"/>
-      <c r="J102" s="12"/>
-      <c r="K102" s="12"/>
-    </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="103" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A103" s="12"/>
       <c r="B103" s="14"/>
       <c r="C103" s="12"/>
@@ -7886,10 +7676,8 @@
       <c r="G103" s="12"/>
       <c r="H103" s="12"/>
       <c r="I103" s="12"/>
-      <c r="J103" s="12"/>
-      <c r="K103" s="12"/>
-    </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="104" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A104" s="12"/>
       <c r="B104" s="14"/>
       <c r="C104" s="12"/>
@@ -7899,10 +7687,8 @@
       <c r="G104" s="12"/>
       <c r="H104" s="12"/>
       <c r="I104" s="12"/>
-      <c r="J104" s="12"/>
-      <c r="K104" s="12"/>
-    </row>
-    <row r="105" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="105" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A105" s="12"/>
       <c r="B105" s="14"/>
       <c r="C105" s="12"/>
@@ -7912,10 +7698,8 @@
       <c r="G105" s="12"/>
       <c r="H105" s="12"/>
       <c r="I105" s="12"/>
-      <c r="J105" s="12"/>
-      <c r="K105" s="12"/>
-    </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="106" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A106" s="12"/>
       <c r="B106" s="14"/>
       <c r="C106" s="12"/>
@@ -7925,10 +7709,8 @@
       <c r="G106" s="12"/>
       <c r="H106" s="12"/>
       <c r="I106" s="12"/>
-      <c r="J106" s="12"/>
-      <c r="K106" s="12"/>
-    </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="107" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A107" s="12"/>
       <c r="B107" s="14"/>
       <c r="C107" s="12"/>
@@ -7938,10 +7720,8 @@
       <c r="G107" s="12"/>
       <c r="H107" s="12"/>
       <c r="I107" s="12"/>
-      <c r="J107" s="12"/>
-      <c r="K107" s="12"/>
-    </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="108" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A108" s="12"/>
       <c r="B108" s="14"/>
       <c r="C108" s="12"/>
@@ -7951,10 +7731,8 @@
       <c r="G108" s="12"/>
       <c r="H108" s="12"/>
       <c r="I108" s="12"/>
-      <c r="J108" s="12"/>
-      <c r="K108" s="12"/>
-    </row>
-    <row r="109" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="109" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A109" s="12"/>
       <c r="B109" s="14"/>
       <c r="C109" s="12"/>
@@ -7964,10 +7742,8 @@
       <c r="G109" s="12"/>
       <c r="H109" s="12"/>
       <c r="I109" s="12"/>
-      <c r="J109" s="12"/>
-      <c r="K109" s="12"/>
-    </row>
-    <row r="110" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="110" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A110" s="12"/>
       <c r="B110" s="14"/>
       <c r="C110" s="12"/>
@@ -7977,10 +7753,8 @@
       <c r="G110" s="12"/>
       <c r="H110" s="12"/>
       <c r="I110" s="12"/>
-      <c r="J110" s="12"/>
-      <c r="K110" s="12"/>
-    </row>
-    <row r="111" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="111" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A111" s="12"/>
       <c r="B111" s="14"/>
       <c r="C111" s="12"/>
@@ -7990,10 +7764,8 @@
       <c r="G111" s="12"/>
       <c r="H111" s="12"/>
       <c r="I111" s="12"/>
-      <c r="J111" s="12"/>
-      <c r="K111" s="12"/>
-    </row>
-    <row r="112" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="112" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A112" s="12"/>
       <c r="B112" s="14"/>
       <c r="C112" s="12"/>
@@ -8003,10 +7775,8 @@
       <c r="G112" s="12"/>
       <c r="H112" s="12"/>
       <c r="I112" s="12"/>
-      <c r="J112" s="12"/>
-      <c r="K112" s="12"/>
-    </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="113" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A113" s="12"/>
       <c r="B113" s="14"/>
       <c r="C113" s="12"/>
@@ -8016,10 +7786,8 @@
       <c r="G113" s="12"/>
       <c r="H113" s="12"/>
       <c r="I113" s="12"/>
-      <c r="J113" s="12"/>
-      <c r="K113" s="12"/>
-    </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="114" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A114" s="12"/>
       <c r="B114" s="14"/>
       <c r="C114" s="12"/>
@@ -8029,10 +7797,8 @@
       <c r="G114" s="12"/>
       <c r="H114" s="12"/>
       <c r="I114" s="12"/>
-      <c r="J114" s="12"/>
-      <c r="K114" s="12"/>
-    </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="115" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A115" s="12"/>
       <c r="B115" s="14"/>
       <c r="C115" s="12"/>
@@ -8042,10 +7808,8 @@
       <c r="G115" s="12"/>
       <c r="H115" s="12"/>
       <c r="I115" s="12"/>
-      <c r="J115" s="12"/>
-      <c r="K115" s="12"/>
-    </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="116" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A116" s="12"/>
       <c r="B116" s="14"/>
       <c r="C116" s="12"/>
@@ -8055,10 +7819,8 @@
       <c r="G116" s="12"/>
       <c r="H116" s="12"/>
       <c r="I116" s="12"/>
-      <c r="J116" s="12"/>
-      <c r="K116" s="12"/>
-    </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="117" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A117" s="12"/>
       <c r="B117" s="14"/>
       <c r="C117" s="12"/>
@@ -8068,10 +7830,8 @@
       <c r="G117" s="12"/>
       <c r="H117" s="12"/>
       <c r="I117" s="12"/>
-      <c r="J117" s="12"/>
-      <c r="K117" s="12"/>
-    </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="118" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A118" s="12"/>
       <c r="B118" s="14"/>
       <c r="C118" s="12"/>
@@ -8081,10 +7841,8 @@
       <c r="G118" s="12"/>
       <c r="H118" s="12"/>
       <c r="I118" s="12"/>
-      <c r="J118" s="12"/>
-      <c r="K118" s="12"/>
-    </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="119" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A119" s="12"/>
       <c r="B119" s="14"/>
       <c r="C119" s="12"/>
@@ -8094,10 +7852,8 @@
       <c r="G119" s="12"/>
       <c r="H119" s="12"/>
       <c r="I119" s="12"/>
-      <c r="J119" s="12"/>
-      <c r="K119" s="12"/>
-    </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="120" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A120" s="12"/>
       <c r="B120" s="14"/>
       <c r="C120" s="12"/>
@@ -8107,10 +7863,8 @@
       <c r="G120" s="12"/>
       <c r="H120" s="12"/>
       <c r="I120" s="12"/>
-      <c r="J120" s="12"/>
-      <c r="K120" s="12"/>
-    </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="121" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A121" s="12"/>
       <c r="B121" s="14"/>
       <c r="C121" s="12"/>
@@ -8120,10 +7874,8 @@
       <c r="G121" s="12"/>
       <c r="H121" s="12"/>
       <c r="I121" s="12"/>
-      <c r="J121" s="12"/>
-      <c r="K121" s="12"/>
-    </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="122" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A122" s="12"/>
       <c r="B122" s="14"/>
       <c r="C122" s="12"/>
@@ -8133,10 +7885,8 @@
       <c r="G122" s="12"/>
       <c r="H122" s="12"/>
       <c r="I122" s="12"/>
-      <c r="J122" s="12"/>
-      <c r="K122" s="12"/>
-    </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="123" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A123" s="12"/>
       <c r="B123" s="14"/>
       <c r="C123" s="12"/>
@@ -8146,10 +7896,8 @@
       <c r="G123" s="12"/>
       <c r="H123" s="12"/>
       <c r="I123" s="12"/>
-      <c r="J123" s="12"/>
-      <c r="K123" s="12"/>
-    </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="124" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A124" s="12"/>
       <c r="B124" s="14"/>
       <c r="C124" s="12"/>
@@ -8159,10 +7907,8 @@
       <c r="G124" s="12"/>
       <c r="H124" s="12"/>
       <c r="I124" s="12"/>
-      <c r="J124" s="12"/>
-      <c r="K124" s="12"/>
-    </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="125" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A125" s="12"/>
       <c r="B125" s="14"/>
       <c r="C125" s="12"/>
@@ -8172,10 +7918,8 @@
       <c r="G125" s="12"/>
       <c r="H125" s="12"/>
       <c r="I125" s="12"/>
-      <c r="J125" s="12"/>
-      <c r="K125" s="12"/>
-    </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="126" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A126" s="12"/>
       <c r="B126" s="14"/>
       <c r="C126" s="12"/>
@@ -8185,10 +7929,8 @@
       <c r="G126" s="12"/>
       <c r="H126" s="12"/>
       <c r="I126" s="12"/>
-      <c r="J126" s="12"/>
-      <c r="K126" s="12"/>
-    </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="127" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A127" s="12"/>
       <c r="B127" s="14"/>
       <c r="C127" s="12"/>
@@ -8198,10 +7940,8 @@
       <c r="G127" s="12"/>
       <c r="H127" s="12"/>
       <c r="I127" s="12"/>
-      <c r="J127" s="12"/>
-      <c r="K127" s="12"/>
-    </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="128" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A128" s="12"/>
       <c r="B128" s="14"/>
       <c r="C128" s="12"/>
@@ -8211,10 +7951,8 @@
       <c r="G128" s="12"/>
       <c r="H128" s="12"/>
       <c r="I128" s="12"/>
-      <c r="J128" s="12"/>
-      <c r="K128" s="12"/>
-    </row>
-    <row r="129" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="129" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A129" s="12"/>
       <c r="B129" s="14"/>
       <c r="C129" s="12"/>
@@ -8224,10 +7962,8 @@
       <c r="G129" s="12"/>
       <c r="H129" s="12"/>
       <c r="I129" s="12"/>
-      <c r="J129" s="12"/>
-      <c r="K129" s="12"/>
-    </row>
-    <row r="130" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="130" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A130" s="12"/>
       <c r="B130" s="14"/>
       <c r="C130" s="12"/>
@@ -8237,10 +7973,8 @@
       <c r="G130" s="12"/>
       <c r="H130" s="12"/>
       <c r="I130" s="12"/>
-      <c r="J130" s="12"/>
-      <c r="K130" s="12"/>
-    </row>
-    <row r="131" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="131" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A131" s="12"/>
       <c r="B131" s="14"/>
       <c r="C131" s="12"/>
@@ -8250,10 +7984,8 @@
       <c r="G131" s="12"/>
       <c r="H131" s="12"/>
       <c r="I131" s="12"/>
-      <c r="J131" s="12"/>
-      <c r="K131" s="12"/>
-    </row>
-    <row r="132" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="132" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A132" s="12"/>
       <c r="B132" s="14"/>
       <c r="C132" s="12"/>
@@ -8263,10 +7995,8 @@
       <c r="G132" s="12"/>
       <c r="H132" s="12"/>
       <c r="I132" s="12"/>
-      <c r="J132" s="12"/>
-      <c r="K132" s="12"/>
-    </row>
-    <row r="133" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="133" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A133" s="12"/>
       <c r="B133" s="14"/>
       <c r="C133" s="12"/>
@@ -8276,10 +8006,8 @@
       <c r="G133" s="12"/>
       <c r="H133" s="12"/>
       <c r="I133" s="12"/>
-      <c r="J133" s="12"/>
-      <c r="K133" s="12"/>
-    </row>
-    <row r="134" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="134" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A134" s="12"/>
       <c r="B134" s="14"/>
       <c r="C134" s="12"/>
@@ -8289,10 +8017,8 @@
       <c r="G134" s="12"/>
       <c r="H134" s="12"/>
       <c r="I134" s="12"/>
-      <c r="J134" s="12"/>
-      <c r="K134" s="12"/>
-    </row>
-    <row r="135" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="135" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A135" s="12"/>
       <c r="B135" s="14"/>
       <c r="C135" s="12"/>
@@ -8302,10 +8028,8 @@
       <c r="G135" s="12"/>
       <c r="H135" s="12"/>
       <c r="I135" s="12"/>
-      <c r="J135" s="12"/>
-      <c r="K135" s="12"/>
-    </row>
-    <row r="136" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="136" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A136" s="12"/>
       <c r="B136" s="14"/>
       <c r="C136" s="12"/>
@@ -8315,10 +8039,8 @@
       <c r="G136" s="12"/>
       <c r="H136" s="12"/>
       <c r="I136" s="12"/>
-      <c r="J136" s="12"/>
-      <c r="K136" s="12"/>
-    </row>
-    <row r="137" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="137" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A137" s="12"/>
       <c r="B137" s="14"/>
       <c r="C137" s="12"/>
@@ -8328,10 +8050,8 @@
       <c r="G137" s="12"/>
       <c r="H137" s="12"/>
       <c r="I137" s="12"/>
-      <c r="J137" s="12"/>
-      <c r="K137" s="12"/>
-    </row>
-    <row r="138" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="138" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A138" s="12"/>
       <c r="B138" s="14"/>
       <c r="C138" s="12"/>
@@ -8341,10 +8061,8 @@
       <c r="G138" s="12"/>
       <c r="H138" s="12"/>
       <c r="I138" s="12"/>
-      <c r="J138" s="12"/>
-      <c r="K138" s="12"/>
-    </row>
-    <row r="139" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="139" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A139" s="12"/>
       <c r="B139" s="14"/>
       <c r="C139" s="12"/>
@@ -8354,10 +8072,8 @@
       <c r="G139" s="12"/>
       <c r="H139" s="12"/>
       <c r="I139" s="12"/>
-      <c r="J139" s="12"/>
-      <c r="K139" s="12"/>
-    </row>
-    <row r="140" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="140" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A140" s="12"/>
       <c r="B140" s="14"/>
       <c r="C140" s="12"/>
@@ -8367,10 +8083,8 @@
       <c r="G140" s="12"/>
       <c r="H140" s="12"/>
       <c r="I140" s="12"/>
-      <c r="J140" s="12"/>
-      <c r="K140" s="12"/>
-    </row>
-    <row r="141" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="141" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A141" s="12"/>
       <c r="B141" s="14"/>
       <c r="C141" s="12"/>
@@ -8380,10 +8094,8 @@
       <c r="G141" s="12"/>
       <c r="H141" s="12"/>
       <c r="I141" s="12"/>
-      <c r="J141" s="12"/>
-      <c r="K141" s="12"/>
-    </row>
-    <row r="142" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="142" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A142" s="12"/>
       <c r="B142" s="14"/>
       <c r="C142" s="12"/>
@@ -8393,10 +8105,8 @@
       <c r="G142" s="12"/>
       <c r="H142" s="12"/>
       <c r="I142" s="12"/>
-      <c r="J142" s="12"/>
-      <c r="K142" s="12"/>
-    </row>
-    <row r="143" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="143" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A143" s="12"/>
       <c r="B143" s="14"/>
       <c r="C143" s="12"/>
@@ -8406,10 +8116,8 @@
       <c r="G143" s="12"/>
       <c r="H143" s="12"/>
       <c r="I143" s="12"/>
-      <c r="J143" s="12"/>
-      <c r="K143" s="12"/>
-    </row>
-    <row r="144" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="144" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A144" s="12"/>
       <c r="B144" s="14"/>
       <c r="C144" s="12"/>
@@ -8419,10 +8127,8 @@
       <c r="G144" s="12"/>
       <c r="H144" s="12"/>
       <c r="I144" s="12"/>
-      <c r="J144" s="12"/>
-      <c r="K144" s="12"/>
-    </row>
-    <row r="145" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="145" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A145" s="12"/>
       <c r="B145" s="14"/>
       <c r="C145" s="12"/>
@@ -8432,10 +8138,8 @@
       <c r="G145" s="12"/>
       <c r="H145" s="12"/>
       <c r="I145" s="12"/>
-      <c r="J145" s="12"/>
-      <c r="K145" s="12"/>
-    </row>
-    <row r="146" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="146" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A146" s="12"/>
       <c r="B146" s="14"/>
       <c r="C146" s="12"/>
@@ -8445,10 +8149,8 @@
       <c r="G146" s="12"/>
       <c r="H146" s="12"/>
       <c r="I146" s="12"/>
-      <c r="J146" s="12"/>
-      <c r="K146" s="12"/>
-    </row>
-    <row r="147" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="147" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A147" s="12"/>
       <c r="B147" s="14"/>
       <c r="C147" s="12"/>
@@ -8458,10 +8160,8 @@
       <c r="G147" s="12"/>
       <c r="H147" s="12"/>
       <c r="I147" s="12"/>
-      <c r="J147" s="12"/>
-      <c r="K147" s="12"/>
-    </row>
-    <row r="148" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="148" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A148" s="12"/>
       <c r="B148" s="14"/>
       <c r="C148" s="12"/>
@@ -8471,10 +8171,8 @@
       <c r="G148" s="12"/>
       <c r="H148" s="12"/>
       <c r="I148" s="12"/>
-      <c r="J148" s="12"/>
-      <c r="K148" s="12"/>
-    </row>
-    <row r="149" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="149" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A149" s="12"/>
       <c r="B149" s="14"/>
       <c r="C149" s="12"/>
@@ -8484,10 +8182,8 @@
       <c r="G149" s="12"/>
       <c r="H149" s="12"/>
       <c r="I149" s="12"/>
-      <c r="J149" s="12"/>
-      <c r="K149" s="12"/>
-    </row>
-    <row r="150" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="150" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A150" s="12"/>
       <c r="B150" s="14"/>
       <c r="C150" s="12"/>
@@ -8497,10 +8193,8 @@
       <c r="G150" s="12"/>
       <c r="H150" s="12"/>
       <c r="I150" s="12"/>
-      <c r="J150" s="12"/>
-      <c r="K150" s="12"/>
-    </row>
-    <row r="151" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="151" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A151" s="12"/>
       <c r="B151" s="14"/>
       <c r="C151" s="12"/>
@@ -8510,10 +8204,8 @@
       <c r="G151" s="12"/>
       <c r="H151" s="12"/>
       <c r="I151" s="12"/>
-      <c r="J151" s="12"/>
-      <c r="K151" s="12"/>
-    </row>
-    <row r="152" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="152" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A152" s="12"/>
       <c r="B152" s="14"/>
       <c r="C152" s="12"/>
@@ -8523,10 +8215,8 @@
       <c r="G152" s="12"/>
       <c r="H152" s="12"/>
       <c r="I152" s="12"/>
-      <c r="J152" s="12"/>
-      <c r="K152" s="12"/>
-    </row>
-    <row r="153" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="153" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A153" s="12"/>
       <c r="B153" s="14"/>
       <c r="C153" s="12"/>
@@ -8536,10 +8226,8 @@
       <c r="G153" s="12"/>
       <c r="H153" s="12"/>
       <c r="I153" s="12"/>
-      <c r="J153" s="12"/>
-      <c r="K153" s="12"/>
-    </row>
-    <row r="154" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="154" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A154" s="12"/>
       <c r="B154" s="14"/>
       <c r="C154" s="12"/>
@@ -8549,10 +8237,8 @@
       <c r="G154" s="12"/>
       <c r="H154" s="12"/>
       <c r="I154" s="12"/>
-      <c r="J154" s="12"/>
-      <c r="K154" s="12"/>
-    </row>
-    <row r="155" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="155" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A155" s="12"/>
       <c r="B155" s="14"/>
       <c r="C155" s="12"/>
@@ -8562,10 +8248,8 @@
       <c r="G155" s="12"/>
       <c r="H155" s="12"/>
       <c r="I155" s="12"/>
-      <c r="J155" s="12"/>
-      <c r="K155" s="12"/>
-    </row>
-    <row r="156" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="156" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A156" s="12"/>
       <c r="B156" s="14"/>
       <c r="C156" s="12"/>
@@ -8575,10 +8259,8 @@
       <c r="G156" s="12"/>
       <c r="H156" s="12"/>
       <c r="I156" s="12"/>
-      <c r="J156" s="12"/>
-      <c r="K156" s="12"/>
-    </row>
-    <row r="157" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="157" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A157" s="12"/>
       <c r="B157" s="14"/>
       <c r="C157" s="12"/>
@@ -8588,10 +8270,8 @@
       <c r="G157" s="12"/>
       <c r="H157" s="12"/>
       <c r="I157" s="12"/>
-      <c r="J157" s="12"/>
-      <c r="K157" s="12"/>
-    </row>
-    <row r="158" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="158" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A158" s="12"/>
       <c r="B158" s="14"/>
       <c r="C158" s="12"/>
@@ -8601,10 +8281,8 @@
       <c r="G158" s="12"/>
       <c r="H158" s="12"/>
       <c r="I158" s="12"/>
-      <c r="J158" s="12"/>
-      <c r="K158" s="12"/>
-    </row>
-    <row r="159" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="159" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A159" s="12"/>
       <c r="B159" s="14"/>
       <c r="C159" s="12"/>
@@ -8614,10 +8292,8 @@
       <c r="G159" s="12"/>
       <c r="H159" s="12"/>
       <c r="I159" s="12"/>
-      <c r="J159" s="12"/>
-      <c r="K159" s="12"/>
-    </row>
-    <row r="160" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="160" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A160" s="12"/>
       <c r="B160" s="14"/>
       <c r="C160" s="12"/>
@@ -8627,10 +8303,8 @@
       <c r="G160" s="12"/>
       <c r="H160" s="12"/>
       <c r="I160" s="12"/>
-      <c r="J160" s="12"/>
-      <c r="K160" s="12"/>
-    </row>
-    <row r="161" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="161" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A161" s="12"/>
       <c r="B161" s="14"/>
       <c r="C161" s="12"/>
@@ -8640,10 +8314,8 @@
       <c r="G161" s="12"/>
       <c r="H161" s="12"/>
       <c r="I161" s="12"/>
-      <c r="J161" s="12"/>
-      <c r="K161" s="12"/>
-    </row>
-    <row r="162" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="162" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A162" s="12"/>
       <c r="B162" s="14"/>
       <c r="C162" s="12"/>
@@ -8653,10 +8325,8 @@
       <c r="G162" s="12"/>
       <c r="H162" s="12"/>
       <c r="I162" s="12"/>
-      <c r="J162" s="12"/>
-      <c r="K162" s="12"/>
-    </row>
-    <row r="163" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="163" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A163" s="12"/>
       <c r="B163" s="14"/>
       <c r="C163" s="12"/>
@@ -8666,10 +8336,8 @@
       <c r="G163" s="12"/>
       <c r="H163" s="12"/>
       <c r="I163" s="12"/>
-      <c r="J163" s="12"/>
-      <c r="K163" s="12"/>
-    </row>
-    <row r="164" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="164" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A164" s="12"/>
       <c r="B164" s="14"/>
       <c r="C164" s="12"/>
@@ -8679,10 +8347,8 @@
       <c r="G164" s="12"/>
       <c r="H164" s="12"/>
       <c r="I164" s="12"/>
-      <c r="J164" s="12"/>
-      <c r="K164" s="12"/>
-    </row>
-    <row r="165" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="165" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A165" s="12"/>
       <c r="B165" s="14"/>
       <c r="C165" s="12"/>
@@ -8692,10 +8358,8 @@
       <c r="G165" s="12"/>
       <c r="H165" s="12"/>
       <c r="I165" s="12"/>
-      <c r="J165" s="12"/>
-      <c r="K165" s="12"/>
-    </row>
-    <row r="166" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="166" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A166" s="12"/>
       <c r="B166" s="14"/>
       <c r="C166" s="12"/>
@@ -8705,10 +8369,8 @@
       <c r="G166" s="12"/>
       <c r="H166" s="12"/>
       <c r="I166" s="12"/>
-      <c r="J166" s="12"/>
-      <c r="K166" s="12"/>
-    </row>
-    <row r="167" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="167" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A167" s="12"/>
       <c r="B167" s="14"/>
       <c r="C167" s="12"/>
@@ -8718,10 +8380,8 @@
       <c r="G167" s="12"/>
       <c r="H167" s="12"/>
       <c r="I167" s="12"/>
-      <c r="J167" s="12"/>
-      <c r="K167" s="12"/>
-    </row>
-    <row r="168" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="168" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A168" s="12"/>
       <c r="B168" s="14"/>
       <c r="C168" s="12"/>
@@ -8731,10 +8391,8 @@
       <c r="G168" s="12"/>
       <c r="H168" s="12"/>
       <c r="I168" s="12"/>
-      <c r="J168" s="12"/>
-      <c r="K168" s="12"/>
-    </row>
-    <row r="169" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="169" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A169" s="12"/>
       <c r="B169" s="14"/>
       <c r="C169" s="12"/>
@@ -8744,10 +8402,8 @@
       <c r="G169" s="12"/>
       <c r="H169" s="12"/>
       <c r="I169" s="12"/>
-      <c r="J169" s="12"/>
-      <c r="K169" s="12"/>
-    </row>
-    <row r="170" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="170" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A170" s="12"/>
       <c r="B170" s="14"/>
       <c r="C170" s="12"/>
@@ -8757,10 +8413,8 @@
       <c r="G170" s="12"/>
       <c r="H170" s="12"/>
       <c r="I170" s="12"/>
-      <c r="J170" s="12"/>
-      <c r="K170" s="12"/>
-    </row>
-    <row r="171" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="171" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A171" s="12"/>
       <c r="B171" s="14"/>
       <c r="C171" s="12"/>
@@ -8770,10 +8424,8 @@
       <c r="G171" s="12"/>
       <c r="H171" s="12"/>
       <c r="I171" s="12"/>
-      <c r="J171" s="12"/>
-      <c r="K171" s="12"/>
-    </row>
-    <row r="172" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="172" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A172" s="12"/>
       <c r="B172" s="14"/>
       <c r="C172" s="12"/>
@@ -8783,10 +8435,8 @@
       <c r="G172" s="12"/>
       <c r="H172" s="12"/>
       <c r="I172" s="12"/>
-      <c r="J172" s="12"/>
-      <c r="K172" s="12"/>
-    </row>
-    <row r="173" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="173" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A173" s="12"/>
       <c r="B173" s="14"/>
       <c r="C173" s="12"/>
@@ -8796,10 +8446,8 @@
       <c r="G173" s="12"/>
       <c r="H173" s="12"/>
       <c r="I173" s="12"/>
-      <c r="J173" s="12"/>
-      <c r="K173" s="12"/>
-    </row>
-    <row r="174" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="174" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A174" s="12"/>
       <c r="B174" s="14"/>
       <c r="C174" s="12"/>
@@ -8809,10 +8457,8 @@
       <c r="G174" s="12"/>
       <c r="H174" s="12"/>
       <c r="I174" s="12"/>
-      <c r="J174" s="12"/>
-      <c r="K174" s="12"/>
-    </row>
-    <row r="175" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="175" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A175" s="12"/>
       <c r="B175" s="14"/>
       <c r="C175" s="12"/>
@@ -8822,10 +8468,8 @@
       <c r="G175" s="12"/>
       <c r="H175" s="12"/>
       <c r="I175" s="12"/>
-      <c r="J175" s="12"/>
-      <c r="K175" s="12"/>
-    </row>
-    <row r="176" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="176" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A176" s="12"/>
       <c r="B176" s="14"/>
       <c r="C176" s="12"/>
@@ -8835,10 +8479,8 @@
       <c r="G176" s="12"/>
       <c r="H176" s="12"/>
       <c r="I176" s="12"/>
-      <c r="J176" s="12"/>
-      <c r="K176" s="12"/>
-    </row>
-    <row r="177" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="177" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A177" s="12"/>
       <c r="B177" s="14"/>
       <c r="C177" s="12"/>
@@ -8848,10 +8490,8 @@
       <c r="G177" s="12"/>
       <c r="H177" s="12"/>
       <c r="I177" s="12"/>
-      <c r="J177" s="12"/>
-      <c r="K177" s="12"/>
-    </row>
-    <row r="178" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="178" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A178" s="12"/>
       <c r="B178" s="14"/>
       <c r="C178" s="12"/>
@@ -8861,10 +8501,8 @@
       <c r="G178" s="12"/>
       <c r="H178" s="12"/>
       <c r="I178" s="12"/>
-      <c r="J178" s="12"/>
-      <c r="K178" s="12"/>
-    </row>
-    <row r="179" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="179" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A179" s="12"/>
       <c r="B179" s="14"/>
       <c r="C179" s="12"/>
@@ -8874,10 +8512,8 @@
       <c r="G179" s="12"/>
       <c r="H179" s="12"/>
       <c r="I179" s="12"/>
-      <c r="J179" s="12"/>
-      <c r="K179" s="12"/>
-    </row>
-    <row r="180" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="180" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A180" s="12"/>
       <c r="B180" s="14"/>
       <c r="C180" s="12"/>
@@ -8887,10 +8523,8 @@
       <c r="G180" s="12"/>
       <c r="H180" s="12"/>
       <c r="I180" s="12"/>
-      <c r="J180" s="12"/>
-      <c r="K180" s="12"/>
-    </row>
-    <row r="181" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="181" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A181" s="12"/>
       <c r="B181" s="14"/>
       <c r="C181" s="12"/>
@@ -8900,10 +8534,8 @@
       <c r="G181" s="12"/>
       <c r="H181" s="12"/>
       <c r="I181" s="12"/>
-      <c r="J181" s="12"/>
-      <c r="K181" s="12"/>
-    </row>
-    <row r="182" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="182" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A182" s="12"/>
       <c r="B182" s="14"/>
       <c r="C182" s="12"/>
@@ -8913,10 +8545,8 @@
       <c r="G182" s="12"/>
       <c r="H182" s="12"/>
       <c r="I182" s="12"/>
-      <c r="J182" s="12"/>
-      <c r="K182" s="12"/>
-    </row>
-    <row r="183" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="183" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A183" s="12"/>
       <c r="B183" s="14"/>
       <c r="C183" s="12"/>
@@ -8926,10 +8556,8 @@
       <c r="G183" s="12"/>
       <c r="H183" s="12"/>
       <c r="I183" s="12"/>
-      <c r="J183" s="12"/>
-      <c r="K183" s="12"/>
-    </row>
-    <row r="184" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="184" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A184" s="12"/>
       <c r="B184" s="14"/>
       <c r="C184" s="12"/>
@@ -8939,10 +8567,8 @@
       <c r="G184" s="12"/>
       <c r="H184" s="12"/>
       <c r="I184" s="12"/>
-      <c r="J184" s="12"/>
-      <c r="K184" s="12"/>
-    </row>
-    <row r="185" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="185" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A185" s="12"/>
       <c r="B185" s="14"/>
       <c r="C185" s="12"/>
@@ -8952,10 +8578,8 @@
       <c r="G185" s="12"/>
       <c r="H185" s="12"/>
       <c r="I185" s="12"/>
-      <c r="J185" s="12"/>
-      <c r="K185" s="12"/>
-    </row>
-    <row r="186" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="186" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A186" s="12"/>
       <c r="B186" s="14"/>
       <c r="C186" s="12"/>
@@ -8965,10 +8589,8 @@
       <c r="G186" s="12"/>
       <c r="H186" s="12"/>
       <c r="I186" s="12"/>
-      <c r="J186" s="12"/>
-      <c r="K186" s="12"/>
-    </row>
-    <row r="187" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="187" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A187" s="12"/>
       <c r="B187" s="14"/>
       <c r="C187" s="12"/>
@@ -8978,10 +8600,8 @@
       <c r="G187" s="12"/>
       <c r="H187" s="12"/>
       <c r="I187" s="12"/>
-      <c r="J187" s="12"/>
-      <c r="K187" s="12"/>
-    </row>
-    <row r="188" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="188" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A188" s="12"/>
       <c r="B188" s="14"/>
       <c r="C188" s="12"/>
@@ -8991,10 +8611,8 @@
       <c r="G188" s="12"/>
       <c r="H188" s="12"/>
       <c r="I188" s="12"/>
-      <c r="J188" s="12"/>
-      <c r="K188" s="12"/>
-    </row>
-    <row r="189" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="189" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A189" s="12"/>
       <c r="B189" s="14"/>
       <c r="C189" s="12"/>
@@ -9004,10 +8622,8 @@
       <c r="G189" s="12"/>
       <c r="H189" s="12"/>
       <c r="I189" s="12"/>
-      <c r="J189" s="12"/>
-      <c r="K189" s="12"/>
-    </row>
-    <row r="190" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="190" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A190" s="12"/>
       <c r="B190" s="14"/>
       <c r="C190" s="12"/>
@@ -9017,10 +8633,8 @@
       <c r="G190" s="12"/>
       <c r="H190" s="12"/>
       <c r="I190" s="12"/>
-      <c r="J190" s="12"/>
-      <c r="K190" s="12"/>
-    </row>
-    <row r="191" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="191" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A191" s="12"/>
       <c r="B191" s="14"/>
       <c r="C191" s="12"/>
@@ -9030,10 +8644,8 @@
       <c r="G191" s="12"/>
       <c r="H191" s="12"/>
       <c r="I191" s="12"/>
-      <c r="J191" s="12"/>
-      <c r="K191" s="12"/>
-    </row>
-    <row r="192" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="192" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A192" s="12"/>
       <c r="B192" s="14"/>
       <c r="C192" s="12"/>
@@ -9043,10 +8655,8 @@
       <c r="G192" s="12"/>
       <c r="H192" s="12"/>
       <c r="I192" s="12"/>
-      <c r="J192" s="12"/>
-      <c r="K192" s="12"/>
-    </row>
-    <row r="193" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="193" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A193" s="12"/>
       <c r="B193" s="14"/>
       <c r="C193" s="12"/>
@@ -9056,10 +8666,8 @@
       <c r="G193" s="12"/>
       <c r="H193" s="12"/>
       <c r="I193" s="12"/>
-      <c r="J193" s="12"/>
-      <c r="K193" s="12"/>
-    </row>
-    <row r="194" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="194" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A194" s="12"/>
       <c r="B194" s="14"/>
       <c r="C194" s="12"/>
@@ -9069,10 +8677,8 @@
       <c r="G194" s="12"/>
       <c r="H194" s="12"/>
       <c r="I194" s="12"/>
-      <c r="J194" s="12"/>
-      <c r="K194" s="12"/>
-    </row>
-    <row r="195" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="195" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A195" s="12"/>
       <c r="B195" s="14"/>
       <c r="C195" s="12"/>
@@ -9082,10 +8688,8 @@
       <c r="G195" s="12"/>
       <c r="H195" s="12"/>
       <c r="I195" s="12"/>
-      <c r="J195" s="12"/>
-      <c r="K195" s="12"/>
-    </row>
-    <row r="196" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="196" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A196" s="12"/>
       <c r="B196" s="14"/>
       <c r="C196" s="12"/>
@@ -9095,10 +8699,8 @@
       <c r="G196" s="12"/>
       <c r="H196" s="12"/>
       <c r="I196" s="12"/>
-      <c r="J196" s="12"/>
-      <c r="K196" s="12"/>
-    </row>
-    <row r="197" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="197" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A197" s="12"/>
       <c r="B197" s="14"/>
       <c r="C197" s="12"/>
@@ -9108,10 +8710,8 @@
       <c r="G197" s="12"/>
       <c r="H197" s="12"/>
       <c r="I197" s="12"/>
-      <c r="J197" s="12"/>
-      <c r="K197" s="12"/>
-    </row>
-    <row r="198" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="198" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A198" s="12"/>
       <c r="B198" s="14"/>
       <c r="C198" s="12"/>
@@ -9121,10 +8721,8 @@
       <c r="G198" s="12"/>
       <c r="H198" s="12"/>
       <c r="I198" s="12"/>
-      <c r="J198" s="12"/>
-      <c r="K198" s="12"/>
-    </row>
-    <row r="199" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="199" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A199" s="12"/>
       <c r="B199" s="14"/>
       <c r="C199" s="12"/>
@@ -9134,10 +8732,8 @@
       <c r="G199" s="12"/>
       <c r="H199" s="12"/>
       <c r="I199" s="12"/>
-      <c r="J199" s="12"/>
-      <c r="K199" s="12"/>
-    </row>
-    <row r="200" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="200" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A200" s="12"/>
       <c r="B200" s="14"/>
       <c r="C200" s="12"/>
@@ -9147,16 +8743,14 @@
       <c r="G200" s="12"/>
       <c r="H200" s="12"/>
       <c r="I200" s="12"/>
-      <c r="J200" s="12"/>
-      <c r="K200" s="12"/>
     </row>
   </sheetData>
   <dataValidations count="6">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Valor no previsto" error="Elige un valor de la lista." sqref="C10:C200">
-      <formula1>"Ninguna,Cronómetro,Contador,Contrarreloj"</formula1>
+      <formula1>"Ninguna,Cronómetro,Contador,Contrarreloj,Nota"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Valor no previsto" error="Elige un valor de la lista." sqref="C3:C200">
-      <formula1>"Ninguna,Cronómetro,Contador,Contrarreloj"</formula1>
+      <formula1>"Ninguna,Cronómetro,Contador,Contrarreloj,Nota"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Valor no previsto" error="Elige un valor de la lista." sqref="D10:D200">
       <formula1>"Jugadores,Equipos"</formula1>
@@ -9164,10 +8758,10 @@
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Valor no previsto" error="Elige un valor de la lista." sqref="D3:D200">
       <formula1>"Jugadores,Equipos"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" errorStyle="warning" errorTitle="Valor no previsto" error="Elige un valor de la lista." sqref="K10:K200">
+    <dataValidation type="list" allowBlank="1" errorStyle="warning" errorTitle="Valor no previsto" error="Elige un valor de la lista." sqref="I10:I200">
       <formula1>Concurso!$B$3:$B$100</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" errorStyle="warning" errorTitle="Valor no previsto" error="Elige un valor de la lista." sqref="K3:K200">
+    <dataValidation type="list" allowBlank="1" errorStyle="warning" errorTitle="Valor no previsto" error="Elige un valor de la lista." sqref="I3:I200">
       <formula1>Concurso!$B$3:$B$100</formula1>
     </dataValidation>
   </dataValidations>
@@ -9480,11 +9074,11 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="12" t="s">
-        <v>188</v>
+        <v>462</v>
       </c>
       <c r="B27" s="14"/>
       <c r="C27" s="12" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="D27" s="12"/>
     </row>
@@ -9494,47 +9088,47 @@
       </c>
       <c r="B28" s="14"/>
       <c r="C28" s="12" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="D28" s="12"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="12" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="B29" s="14"/>
       <c r="C29" s="12" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="D29" s="12"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="12" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="B30" s="14"/>
       <c r="C30" s="12" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="D30" s="12"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="12" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="B31" s="14"/>
       <c r="C31" s="12" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="D31" s="12"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="12" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="B32" s="14"/>
       <c r="C32" s="12" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="D32" s="12"/>
     </row>
@@ -10580,7 +10174,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:2" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="B1" s="10" t="s">
         <v>61</v>
@@ -10588,7 +10182,7 @@
     </row>
     <row r="2" ht="42" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="B2" s="11" t="s">
         <v>163</v>
@@ -11443,7 +11037,7 @@
     </row>
     <row r="2" ht="42" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="B2" s="11" t="s">
         <v>203</v>
@@ -11466,19 +11060,19 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="F3" s="12" t="s">
         <v>195</v>
@@ -11487,19 +11081,19 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
+        <v>476</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>477</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>478</v>
+      </c>
+      <c r="D4" s="14" t="s">
         <v>475</v>
       </c>
-      <c r="B4" s="14" t="s">
-        <v>476</v>
-      </c>
-      <c r="C4" s="14" t="s">
-        <v>477</v>
-      </c>
-      <c r="D4" s="14" t="s">
-        <v>474</v>
-      </c>
       <c r="E4" s="14" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="F4" s="12" t="s">
         <v>197</v>
@@ -13325,13 +12919,13 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>61</v>
@@ -13339,13 +12933,13 @@
     </row>
     <row r="2" ht="42" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="D2" s="11" t="s">
         <v>163</v>
@@ -13353,7 +12947,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="B3" s="12">
         <v>60</v>
@@ -13363,7 +12957,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="B4" s="12">
         <v>75</v>
@@ -13373,7 +12967,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="B5" s="12">
         <v>20</v>
@@ -13383,7 +12977,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="B6" s="12">
         <v>90</v>
@@ -13393,7 +12987,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="B7" s="12">
         <v>20</v>
@@ -14592,52 +14186,52 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:1" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
     </row>
     <row r="2" ht="42" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Lobos contra vampiros (el pañuelo), twerking en la discoteca y panal más exigente
- Juego final: duelos de uno de cada equipo (lobos = 1.er equipo, vampiros = 2.º), sorteo o pareja en secreto, ruleta de caras, 3-2-1 y silbato; 10 puntos por duelo ganado
- Twerking: entorno Discoteca con focos y vídeo de sección (carpeta Vídeos/); Libre con «Jugadores» agrupados por equipo
- Panal: tres pasadas, límite de velocidad de la aguja y 60 s; Squid a 5 puntos y sin canicas en el recorrido
- La canción del título sigue en la conexión, sin lluvia, efectos cortos no se repiten
- Respuesta de «¿Qué canción es?» en grande, cuenta atrás en Nota, elegir el duelo de reflejos tocando nombres
- Plantilla sin silla invisible

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/plantilla-concurso.xlsx
+++ b/public/plantilla-concurso.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="747" uniqueCount="500">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="751" uniqueCount="502">
   <si>
     <t>EMPIEZA AQUÍ</t>
   </si>
@@ -207,6 +207,15 @@
     <t>Juegos seguidos desde el móvil en los que la gente se va eliminando; los supervivientes se reparten la hucha.</t>
   </si>
   <si>
+    <t>Lobos contra vampiros</t>
+  </si>
+  <si>
+    <t>no tiene pestaña</t>
+  </si>
+  <si>
+    <t>El colofón: el juego del pañuelo. Uno del primer equipo (lobos) contra uno del segundo (vampiros), hasta que salen todos; tú dices quién gana cada duelo. Sin pestaña: no tiene preguntas.</t>
+  </si>
+  <si>
     <t>Orden</t>
   </si>
   <si>
@@ -336,6 +345,9 @@
     <t>Caja con pelotas a la cadera, por la espalda: ¡sácalas todas a golpe de twerking antes que tu rival!</t>
   </si>
   <si>
+    <t>Discoteca</t>
+  </si>
+  <si>
     <t>Reflejos</t>
   </si>
   <si>
@@ -372,36 +384,42 @@
     <t>Noche de luna</t>
   </si>
   <si>
-    <t>Cinco juegos seguidos: quien falla, fuera. Los que sobreviven se reparten la hucha.</t>
+    <t>Cuatro juegos seguidos: quien falla, fuera. Los que sobreviven se reparten la hucha.</t>
   </si>
   <si>
     <t>Apostad lo que tenéis. Aquí se decide todo.</t>
   </si>
   <si>
+    <t>El colofón: el juego del pañuelo. Uno de cada equipo, al sillón… ¡y a por el pañuelo!</t>
+  </si>
+  <si>
+    <t>Luna llena</t>
+  </si>
+  <si>
     <t>Equipo</t>
   </si>
   <si>
     <t>Color</t>
   </si>
   <si>
-    <t>↳ Un equipo por fila. Borra todas para jugar sin equipos.</t>
+    <t>↳ Un equipo por fila. Borra todas para jugar sin equipos. En «Lobos contra vampiros», el 1º son los lobos y el 2º los vampiros.</t>
   </si>
   <si>
     <t>↳ Opcional. Cada equipo, uno distinto.</t>
   </si>
   <si>
-    <t>Zombies</t>
+    <t>Hombres lobo</t>
+  </si>
+  <si>
+    <t>Azul</t>
+  </si>
+  <si>
+    <t>Vampiros</t>
   </si>
   <si>
     <t>Rojo</t>
   </si>
   <si>
-    <t>Hombres Lobo</t>
-  </si>
-  <si>
-    <t>Azul</t>
-  </si>
-  <si>
     <t>Ajuste</t>
   </si>
   <si>
@@ -1149,7 +1167,7 @@
     <t>↳ Cronómetro: gana quien más aguanta. Contador: +1/−1. Contrarreloj: de uno en uno, gana el más rápido. Nota: das a cada uno del 1 al 10 (sus puntos). Ninguna: eliges tú.</t>
   </si>
   <si>
-    <t>↳ ¿Juega cada uno o cada equipo (uno por equipo)?</t>
+    <t>↳ Jugadores: eliges quién sale (de cada equipo) y los puntos son para él (y suman a su equipo). Equipos: los puntos van al equipo.</t>
   </si>
   <si>
     <t>↳ Vacío = los de la sección. Con Nota no cuenta: los puntos son la nota.</t>
@@ -1182,6 +1200,9 @@
     <t>Uno por equipo. La caja a la cadera, por la espalda: gana quien saque todas las pelotas primero.</t>
   </si>
   <si>
+    <t>Jugadores</t>
+  </si>
+  <si>
     <t>Twerking: la revancha</t>
   </si>
   <si>
@@ -1212,9 +1233,6 @@
     <t>Nota</t>
   </si>
   <si>
-    <t>Jugadores</t>
-  </si>
-  <si>
     <t>Golpe Cancion n1</t>
   </si>
   <si>
@@ -1260,12 +1278,6 @@
     <t>Más sentadillas en un minuto (bajando hasta abajo).</t>
   </si>
   <si>
-    <t>La silla invisible</t>
-  </si>
-  <si>
-    <t>Espalda en la pared, como sentado en una silla. Gana el último.</t>
-  </si>
-  <si>
     <t>Flamenco a ciegas</t>
   </si>
   <si>
@@ -1362,9 +1374,6 @@
     <t>Dulce, azúcar, chuche, truco o trato</t>
   </si>
   <si>
-    <t>Luna llena</t>
-  </si>
-  <si>
     <t>Noche, lobo, redonda, cielo</t>
   </si>
   <si>
@@ -1476,7 +1485,7 @@
     <t>Tramos</t>
   </si>
   <si>
-    <t>↳ Uno por fila, en el orden en que se juegan. Sin filas = los 5.</t>
+    <t>↳ Uno por fila, en el orden en que se juegan. Sin filas = todos menos Canicas.</t>
   </si>
   <si>
     <t>↳ Cuánto dura (en el puente, el tiempo para elegir cada tramo). Vacío = lo normal.</t>
@@ -1492,9 +1501,6 @@
   </si>
   <si>
     <t>Tira y afloja</t>
-  </si>
-  <si>
-    <t>Canicas</t>
   </si>
   <si>
     <t>El puente</t>
@@ -2182,7 +2188,7 @@
   <sheetPr>
     <tabColor rgb="FFFF8A1F"/>
   </sheetPr>
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -2437,6 +2443,17 @@
       </c>
       <c r="C33" t="s">
         <v>58</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="B34" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="C34" s="9" t="s">
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -2462,153 +2479,153 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>330</v>
+        <v>336</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>331</v>
+        <v>337</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>332</v>
+        <v>338</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>333</v>
+        <v>339</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>334</v>
+        <v>340</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>335</v>
+        <v>341</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>336</v>
+        <v>342</v>
       </c>
       <c r="B3" s="12">
         <v>910</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>337</v>
+        <v>343</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>338</v>
+        <v>344</v>
       </c>
       <c r="E3" s="12"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>339</v>
+        <v>345</v>
       </c>
       <c r="B4" s="12">
         <v>1247</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>338</v>
+        <v>344</v>
       </c>
       <c r="E4" s="12"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
       <c r="B5" s="12">
         <v>1897</v>
       </c>
       <c r="C5" s="12"/>
       <c r="D5" s="12" t="s">
-        <v>338</v>
+        <v>344</v>
       </c>
       <c r="E5" s="12"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>342</v>
+        <v>348</v>
       </c>
       <c r="B6" s="12">
         <v>330</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>338</v>
+        <v>344</v>
       </c>
       <c r="E6" s="12"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>344</v>
+        <v>350</v>
       </c>
       <c r="B7" s="12">
         <v>88</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>345</v>
+        <v>351</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>346</v>
+        <v>352</v>
       </c>
       <c r="E7" s="12"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>347</v>
+        <v>353</v>
       </c>
       <c r="B8" s="12">
         <v>505</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>337</v>
+        <v>343</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>338</v>
+        <v>344</v>
       </c>
       <c r="E8" s="12"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>348</v>
+        <v>354</v>
       </c>
       <c r="B9" s="12">
         <v>40</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>349</v>
+        <v>355</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>346</v>
+        <v>352</v>
       </c>
       <c r="E9" s="12"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>350</v>
+        <v>356</v>
       </c>
       <c r="B10" s="12">
         <v>32</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>351</v>
+        <v>357</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>346</v>
+        <v>352</v>
       </c>
       <c r="E10" s="12"/>
     </row>
@@ -3977,30 +3994,30 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>352</v>
+        <v>358</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>353</v>
+        <v>359</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>354</v>
+        <v>360</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" ht="42" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>355</v>
+        <v>361</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>356</v>
+        <v>362</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>357</v>
+        <v>363</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -4008,7 +4025,7 @@
         <v>10</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>358</v>
+        <v>364</v>
       </c>
       <c r="C3" s="12"/>
       <c r="D3" s="12"/>
@@ -4018,7 +4035,7 @@
         <v>15</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>359</v>
+        <v>365</v>
       </c>
       <c r="C4" s="12">
         <v>3</v>
@@ -4030,7 +4047,7 @@
         <v>7</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>360</v>
+        <v>366</v>
       </c>
       <c r="C5" s="12"/>
       <c r="D5" s="12"/>
@@ -4040,7 +4057,7 @@
         <v>12</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>359</v>
+        <v>365</v>
       </c>
       <c r="C6" s="12">
         <v>5</v>
@@ -4052,7 +4069,7 @@
         <v>20</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>360</v>
+        <v>366</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12"/>
@@ -5250,24 +5267,24 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:3" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>361</v>
+        <v>367</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>362</v>
+        <v>368</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" ht="42" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>363</v>
+        <v>369</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -5275,7 +5292,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>365</v>
+        <v>371</v>
       </c>
       <c r="C3" s="12"/>
     </row>
@@ -5284,7 +5301,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>366</v>
+        <v>372</v>
       </c>
       <c r="C4" s="12"/>
     </row>
@@ -5293,7 +5310,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>365</v>
+        <v>371</v>
       </c>
       <c r="C5" s="12"/>
     </row>
@@ -6310,200 +6327,200 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:9" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>367</v>
+        <v>373</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C1" s="10" t="s">
+        <v>374</v>
+      </c>
+      <c r="D1" s="10" t="s">
         <v>368</v>
       </c>
-      <c r="D1" s="10" t="s">
-        <v>362</v>
-      </c>
       <c r="E1" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>375</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="H1" s="10" t="s">
+        <v>162</v>
+      </c>
+      <c r="I1" s="10" t="s">
         <v>64</v>
-      </c>
-      <c r="F1" s="10" t="s">
-        <v>369</v>
-      </c>
-      <c r="G1" s="10" t="s">
-        <v>155</v>
-      </c>
-      <c r="H1" s="10" t="s">
-        <v>156</v>
-      </c>
-      <c r="I1" s="10" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="2" ht="42" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>370</v>
+        <v>376</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>371</v>
+        <v>377</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>372</v>
+        <v>378</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>373</v>
+        <v>379</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>375</v>
+        <v>381</v>
       </c>
       <c r="G2" s="11" t="s">
-        <v>376</v>
+        <v>382</v>
       </c>
       <c r="H2" s="11" t="s">
-        <v>377</v>
+        <v>383</v>
       </c>
       <c r="I2" s="11" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>378</v>
+        <v>384</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>379</v>
+        <v>385</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>380</v>
+        <v>386</v>
       </c>
       <c r="E3" s="12"/>
       <c r="F3" s="12"/>
       <c r="G3" s="12"/>
       <c r="H3" s="12"/>
       <c r="I3" s="12" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>381</v>
+        <v>387</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>382</v>
+        <v>388</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>379</v>
+        <v>385</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>380</v>
+        <v>386</v>
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="12"/>
       <c r="G4" s="12"/>
       <c r="H4" s="12"/>
       <c r="I4" s="12" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>383</v>
+        <v>389</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>379</v>
+        <v>385</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>380</v>
+        <v>390</v>
       </c>
       <c r="E5" s="12"/>
       <c r="F5" s="12"/>
       <c r="G5" s="12"/>
       <c r="H5" s="12"/>
       <c r="I5" s="12" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>384</v>
+        <v>391</v>
       </c>
       <c r="B6" s="14" t="s">
+        <v>392</v>
+      </c>
+      <c r="C6" s="12" t="s">
         <v>385</v>
       </c>
-      <c r="C6" s="12" t="s">
-        <v>379</v>
-      </c>
       <c r="D6" s="12" t="s">
-        <v>380</v>
+        <v>390</v>
       </c>
       <c r="E6" s="12"/>
       <c r="F6" s="12"/>
       <c r="G6" s="12"/>
       <c r="H6" s="12"/>
       <c r="I6" s="12" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>386</v>
+        <v>393</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>379</v>
+        <v>385</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>380</v>
+        <v>390</v>
       </c>
       <c r="E7" s="12"/>
       <c r="F7" s="12"/>
       <c r="G7" s="12"/>
       <c r="H7" s="12"/>
       <c r="I7" s="12" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>387</v>
+        <v>394</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>388</v>
+        <v>395</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>379</v>
+        <v>385</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>380</v>
+        <v>390</v>
       </c>
       <c r="E8" s="12"/>
       <c r="F8" s="12"/>
       <c r="G8" s="12"/>
       <c r="H8" s="12"/>
       <c r="I8" s="12" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>389</v>
+        <v>396</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>390</v>
+        <v>397</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>380</v>
+        <v>386</v>
       </c>
       <c r="E9" s="12"/>
       <c r="F9" s="12">
@@ -6512,117 +6529,117 @@
       <c r="G9" s="12"/>
       <c r="H9" s="12"/>
       <c r="I9" s="12" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>391</v>
+        <v>398</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>392</v>
+        <v>399</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>393</v>
+        <v>400</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
       <c r="E10" s="12"/>
       <c r="F10" s="12"/>
       <c r="G10" s="12" t="s">
-        <v>395</v>
+        <v>401</v>
       </c>
       <c r="H10" s="12">
         <v>0</v>
       </c>
       <c r="I10" s="12" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
-        <v>396</v>
+        <v>402</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>397</v>
+        <v>403</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>393</v>
+        <v>400</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
       <c r="E11" s="12"/>
       <c r="F11" s="12"/>
       <c r="G11" s="12" t="s">
-        <v>398</v>
+        <v>404</v>
       </c>
       <c r="H11" s="12">
         <v>0</v>
       </c>
       <c r="I11" s="12" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>399</v>
+        <v>405</v>
       </c>
       <c r="B12" s="14" t="s">
+        <v>406</v>
+      </c>
+      <c r="C12" s="12" t="s">
         <v>400</v>
       </c>
-      <c r="C12" s="12" t="s">
-        <v>393</v>
-      </c>
       <c r="D12" s="12" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
       <c r="E12" s="12"/>
       <c r="F12" s="12"/>
       <c r="G12" s="12" t="s">
-        <v>401</v>
+        <v>407</v>
       </c>
       <c r="H12" s="12">
         <v>0</v>
       </c>
       <c r="I12" s="12" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
-        <v>402</v>
+        <v>408</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>403</v>
+        <v>409</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>404</v>
+        <v>410</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
       <c r="E13" s="12"/>
       <c r="F13" s="12"/>
       <c r="G13" s="12"/>
       <c r="H13" s="12"/>
       <c r="I13" s="12" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
-        <v>405</v>
+        <v>411</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>406</v>
+        <v>412</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>407</v>
+        <v>413</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>380</v>
+        <v>390</v>
       </c>
       <c r="E14" s="12">
         <v>5</v>
@@ -6631,138 +6648,128 @@
       <c r="G14" s="12"/>
       <c r="H14" s="12"/>
       <c r="I14" s="12" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="12" t="s">
-        <v>408</v>
+        <v>414</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>409</v>
+        <v>415</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>407</v>
+        <v>413</v>
       </c>
       <c r="D15" s="12" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
       <c r="E15" s="12"/>
       <c r="F15" s="12"/>
       <c r="G15" s="12"/>
       <c r="H15" s="12"/>
       <c r="I15" s="12" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="12" t="s">
+        <v>416</v>
+      </c>
+      <c r="B16" s="14" t="s">
+        <v>417</v>
+      </c>
+      <c r="C16" s="12" t="s">
         <v>410</v>
       </c>
-      <c r="B16" s="14" t="s">
-        <v>411</v>
-      </c>
-      <c r="C16" s="12" t="s">
-        <v>404</v>
-      </c>
       <c r="D16" s="12" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
       <c r="E16" s="12"/>
       <c r="F16" s="12"/>
       <c r="G16" s="12"/>
       <c r="H16" s="12"/>
       <c r="I16" s="12" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="12" t="s">
-        <v>412</v>
+        <v>418</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>413</v>
+        <v>419</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>404</v>
+        <v>385</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>394</v>
-      </c>
-      <c r="E17" s="12"/>
+        <v>386</v>
+      </c>
+      <c r="E17" s="12">
+        <v>5</v>
+      </c>
       <c r="F17" s="12"/>
       <c r="G17" s="12"/>
       <c r="H17" s="12"/>
       <c r="I17" s="12" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="12" t="s">
-        <v>414</v>
+        <v>420</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>415</v>
+        <v>421</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>379</v>
+        <v>385</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>380</v>
-      </c>
-      <c r="E18" s="12">
-        <v>5</v>
-      </c>
+        <v>390</v>
+      </c>
+      <c r="E18" s="12"/>
       <c r="F18" s="12"/>
       <c r="G18" s="12"/>
       <c r="H18" s="12"/>
       <c r="I18" s="12" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
-        <v>416</v>
+        <v>422</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>417</v>
+        <v>423</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>379</v>
+        <v>413</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>394</v>
-      </c>
-      <c r="E19" s="12"/>
+        <v>386</v>
+      </c>
+      <c r="E19" s="12">
+        <v>5</v>
+      </c>
       <c r="F19" s="12"/>
       <c r="G19" s="12"/>
       <c r="H19" s="12"/>
       <c r="I19" s="12" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="12" t="s">
-        <v>418</v>
-      </c>
-      <c r="B20" s="14" t="s">
-        <v>419</v>
-      </c>
-      <c r="C20" s="12" t="s">
-        <v>407</v>
-      </c>
-      <c r="D20" s="12" t="s">
-        <v>380</v>
-      </c>
-      <c r="E20" s="12">
-        <v>5</v>
-      </c>
+      <c r="A20" s="12"/>
+      <c r="B20" s="14"/>
+      <c r="C20" s="12"/>
+      <c r="D20" s="12"/>
+      <c r="E20" s="12"/>
       <c r="F20" s="12"/>
       <c r="G20" s="12"/>
       <c r="H20" s="12"/>
-      <c r="I20" s="12" t="s">
-        <v>111</v>
-      </c>
+      <c r="I20" s="12"/>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="12"/>
@@ -8786,349 +8793,349 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>421</v>
+        <v>425</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>353</v>
+        <v>359</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" ht="42" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>422</v>
+        <v>426</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>423</v>
+        <v>427</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>425</v>
+        <v>429</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>426</v>
+        <v>430</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>427</v>
+        <v>431</v>
       </c>
       <c r="D3" s="12"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>428</v>
+        <v>432</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>429</v>
+        <v>433</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>427</v>
+        <v>431</v>
       </c>
       <c r="D4" s="12"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>430</v>
+        <v>434</v>
       </c>
       <c r="B5" s="14" t="s">
+        <v>435</v>
+      </c>
+      <c r="C5" s="12" t="s">
         <v>431</v>
-      </c>
-      <c r="C5" s="12" t="s">
-        <v>427</v>
       </c>
       <c r="D5" s="12"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>432</v>
+        <v>436</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>433</v>
+        <v>437</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>427</v>
+        <v>431</v>
       </c>
       <c r="D6" s="12"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
-        <v>434</v>
+        <v>438</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>435</v>
+        <v>439</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>427</v>
+        <v>431</v>
       </c>
       <c r="D7" s="12"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>436</v>
+        <v>440</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>437</v>
+        <v>441</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>427</v>
+        <v>431</v>
       </c>
       <c r="D8" s="12"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>438</v>
+        <v>442</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>439</v>
+        <v>443</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>427</v>
+        <v>431</v>
       </c>
       <c r="D9" s="12"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>441</v>
+        <v>445</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>427</v>
+        <v>431</v>
       </c>
       <c r="D10" s="12"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
-        <v>442</v>
+        <v>446</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>443</v>
+        <v>447</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>427</v>
+        <v>431</v>
       </c>
       <c r="D11" s="12"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>444</v>
+        <v>121</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>427</v>
+        <v>431</v>
       </c>
       <c r="D12" s="12"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
       <c r="B13" s="14"/>
       <c r="C13" s="12" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="D13" s="12"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="B14" s="14"/>
       <c r="C14" s="12" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="D14" s="12"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="12" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
       <c r="B15" s="14"/>
       <c r="C15" s="12" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="D15" s="12"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="12" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
       <c r="B16" s="14"/>
       <c r="C16" s="12" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="D16" s="12"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="12" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="B17" s="14"/>
       <c r="C17" s="12" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="D17" s="12"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="12" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
       <c r="B18" s="14"/>
       <c r="C18" s="12" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="D18" s="12"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
       <c r="B19" s="14"/>
       <c r="C19" s="12" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="D19" s="12"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="12" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="B20" s="14"/>
       <c r="C20" s="12" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="D20" s="12"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="12" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
       <c r="B21" s="14"/>
       <c r="C21" s="12" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="D21" s="12"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="12" t="s">
-        <v>456</v>
+        <v>459</v>
       </c>
       <c r="B22" s="14"/>
       <c r="C22" s="12" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="D22" s="12"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
       <c r="B23" s="14"/>
       <c r="C23" s="12" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="D23" s="12"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
       <c r="B24" s="14"/>
       <c r="C24" s="12" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="D24" s="12"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="12" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="B25" s="14"/>
       <c r="C25" s="12" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="D25" s="12"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="12" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
       <c r="B26" s="14"/>
       <c r="C26" s="12" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="D26" s="12"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="12" t="s">
-        <v>462</v>
+        <v>465</v>
       </c>
       <c r="B27" s="14"/>
       <c r="C27" s="12" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="D27" s="12"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="12" t="s">
-        <v>313</v>
+        <v>319</v>
       </c>
       <c r="B28" s="14"/>
       <c r="C28" s="12" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="D28" s="12"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="12" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="B29" s="14"/>
       <c r="C29" s="12" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="D29" s="12"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="12" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="B30" s="14"/>
       <c r="C30" s="12" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="D30" s="12"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="12" t="s">
-        <v>466</v>
+        <v>469</v>
       </c>
       <c r="B31" s="14"/>
       <c r="C31" s="12" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="D31" s="12"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="12" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="B32" s="14"/>
       <c r="C32" s="12" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="D32" s="12"/>
     </row>
@@ -10174,18 +10181,18 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:2" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>468</v>
+        <v>471</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" ht="42" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>469</v>
+        <v>472</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -11014,89 +11021,89 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" ht="42" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="G2" s="11" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
       <c r="F3" s="12" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="G3" s="12"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="C4" s="14" t="s">
+        <v>481</v>
+      </c>
+      <c r="D4" s="14" t="s">
         <v>478</v>
       </c>
-      <c r="D4" s="14" t="s">
-        <v>475</v>
-      </c>
       <c r="E4" s="14" t="s">
-        <v>479</v>
+        <v>482</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="G4" s="12"/>
     </row>
@@ -12919,35 +12926,35 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>480</v>
+        <v>483</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>468</v>
+        <v>471</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" ht="42" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="B3" s="12">
         <v>60</v>
@@ -12957,17 +12964,17 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>486</v>
+        <v>489</v>
       </c>
       <c r="B4" s="12">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="C4" s="12"/>
       <c r="D4" s="12"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>487</v>
+        <v>490</v>
       </c>
       <c r="B5" s="12">
         <v>20</v>
@@ -12977,21 +12984,17 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>488</v>
+        <v>491</v>
       </c>
       <c r="B6" s="12">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="C6" s="12"/>
       <c r="D6" s="12"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="12" t="s">
-        <v>489</v>
-      </c>
-      <c r="B7" s="12">
-        <v>20</v>
-      </c>
+      <c r="A7" s="12"/>
+      <c r="B7" s="12"/>
       <c r="C7" s="12"/>
       <c r="D7" s="12"/>
     </row>
@@ -14186,52 +14189,52 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:1" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
     </row>
     <row r="2" ht="42" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
@@ -14830,66 +14833,66 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>17</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="J1" s="10" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" ht="42" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="G2" s="11" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="H2" s="11" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="I2" s="11" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="J2" s="11" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
@@ -14897,26 +14900,26 @@
         <v>1</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="D3" s="12" t="s">
         <v>20</v>
       </c>
       <c r="E3" s="13" t="str">
-        <f>IF(D3="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D3,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D3="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D3,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v>→ Pulsador</v>
       </c>
       <c r="F3" s="14" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="G3" s="12">
         <v>1</v>
       </c>
       <c r="H3" s="12" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="I3" s="12"/>
       <c r="J3" s="12"/>
@@ -14926,23 +14929,23 @@
         <v>2</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="D4" s="12" t="s">
         <v>23</v>
       </c>
       <c r="E4" s="13" t="str">
-        <f>IF(D4="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D4,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D4="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D4,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v>→ Test</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="H4" s="12"/>
       <c r="I4" s="12"/>
@@ -14953,20 +14956,20 @@
         <v>3</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="D5" s="12" t="s">
         <v>26</v>
       </c>
       <c r="E5" s="13" t="str">
-        <f>IF(D5="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D5,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D5="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D5,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v>→ Verdad o mentira</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="G5" s="12">
         <v>1</v>
@@ -14980,7 +14983,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C6" s="12" t="s">
         <v>47</v>
@@ -14989,11 +14992,11 @@
         <v>47</v>
       </c>
       <c r="E6" s="13" t="str">
-        <f>IF(D6="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D6,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D6="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D6,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v>→ Palabras</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="G6" s="12">
         <v>1</v>
@@ -15007,20 +15010,20 @@
         <v>5</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D7" s="12" t="s">
         <v>32</v>
       </c>
       <c r="E7" s="13" t="str">
-        <f>IF(D7="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D7,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D7="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D7,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v>→ Votación</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="G7" s="12">
         <v>1</v>
@@ -15034,20 +15037,20 @@
         <v>6</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="D8" s="12" t="s">
         <v>44</v>
       </c>
       <c r="E8" s="13" t="str">
-        <f>IF(D8="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D8,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D8="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D8,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v>→ Libre</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="G8" s="12">
         <v>3</v>
@@ -15061,23 +15064,23 @@
         <v>7</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D9" s="12" t="s">
         <v>35</v>
       </c>
       <c r="E9" s="13" t="str">
-        <f>IF(D9="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D9,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D9="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D9,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v>→ Estimación</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="G9" s="12" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="H9" s="12"/>
       <c r="I9" s="12"/>
@@ -15088,7 +15091,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C10" s="12" t="s">
         <v>50</v>
@@ -15097,17 +15100,17 @@
         <v>50</v>
       </c>
       <c r="E10" s="13" t="str">
-        <f>IF(D10="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D10,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D10="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D10,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v>→ Agitar</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="G10" s="12" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="H10" s="12" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="I10" s="12"/>
       <c r="J10" s="12"/>
@@ -15117,26 +15120,26 @@
         <v>9</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="D11" s="12" t="s">
         <v>20</v>
       </c>
       <c r="E11" s="13" t="str">
-        <f>IF(D11="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D11,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D11="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D11,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v>→ Pulsador</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="G11" s="12">
         <v>2</v>
       </c>
       <c r="H11" s="12" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="I11" s="12"/>
       <c r="J11" s="12"/>
@@ -15146,23 +15149,23 @@
         <v>10</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="D12" s="12" t="s">
         <v>38</v>
       </c>
       <c r="E12" s="13" t="str">
-        <f>IF(D12="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D12,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D12="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D12,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v>→ Contador</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="G12" s="12" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="H12" s="12"/>
       <c r="I12" s="12"/>
@@ -15173,50 +15176,52 @@
         <v>11</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="D13" s="12" t="s">
         <v>44</v>
       </c>
       <c r="E13" s="13" t="str">
-        <f>IF(D13="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D13,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D13="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D13,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v>→ Libre</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="G13" s="12">
         <v>3</v>
       </c>
       <c r="H13" s="12"/>
       <c r="I13" s="12"/>
-      <c r="J13" s="12"/>
+      <c r="J13" s="12" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="12">
         <v>12</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="D14" s="12" t="s">
         <v>41</v>
       </c>
       <c r="E14" s="13" t="str">
-        <f>IF(D14="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D14,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D14="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D14,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v>→ Reflejos</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="G14" s="12" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="H14" s="12"/>
       <c r="I14" s="12"/>
@@ -15227,20 +15232,20 @@
         <v>13</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="D15" s="12" t="s">
         <v>44</v>
       </c>
       <c r="E15" s="13" t="str">
-        <f>IF(D15="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D15,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D15="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D15,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v>→ Libre</v>
       </c>
       <c r="F15" s="14" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="G15" s="12">
         <v>2</v>
@@ -15254,7 +15259,7 @@
         <v>14</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C16" s="12" t="s">
         <v>29</v>
@@ -15263,11 +15268,11 @@
         <v>29</v>
       </c>
       <c r="E16" s="13" t="str">
-        <f>IF(D16="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D16,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D16="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D16,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v>→ Dos verdades</v>
       </c>
       <c r="F16" s="14" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="G16" s="12">
         <v>1</v>
@@ -15281,20 +15286,20 @@
         <v>15</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="D17" s="12" t="s">
         <v>44</v>
       </c>
       <c r="E17" s="13" t="str">
-        <f>IF(D17="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D17,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D17="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D17,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v>→ Libre</v>
       </c>
       <c r="F17" s="14" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G17" s="12">
         <v>3</v>
@@ -15308,20 +15313,20 @@
         <v>16</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="D18" s="12" t="s">
         <v>44</v>
       </c>
       <c r="E18" s="13" t="str">
-        <f>IF(D18="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D18,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D18="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D18,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v>→ Libre</v>
       </c>
       <c r="F18" s="14" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="G18" s="12">
         <v>5</v>
@@ -15335,30 +15340,30 @@
         <v>17</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D19" s="12" t="s">
         <v>44</v>
       </c>
       <c r="E19" s="13" t="str">
-        <f>IF(D19="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D19,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D19="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D19,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v>→ Libre</v>
       </c>
       <c r="F19" s="14" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="G19" s="12">
         <v>3</v>
       </c>
       <c r="H19" s="12" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="I19" s="12"/>
       <c r="J19" s="12" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
@@ -15366,7 +15371,7 @@
         <v>18</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C20" s="12" t="s">
         <v>56</v>
@@ -15375,14 +15380,14 @@
         <v>56</v>
       </c>
       <c r="E20" s="13" t="str">
-        <f>IF(D20="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D20,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D20="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D20,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v>→ Squid</v>
       </c>
       <c r="F20" s="14" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="G20" s="12">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H20" s="12"/>
       <c r="I20" s="12"/>
@@ -15393,7 +15398,7 @@
         <v>19</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C21" s="12" t="s">
         <v>53</v>
@@ -15402,11 +15407,11 @@
         <v>53</v>
       </c>
       <c r="E21" s="13" t="str">
-        <f>IF(D21="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D21,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D21="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D21,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v>→ Apuesta</v>
       </c>
       <c r="F21" s="14" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="G21" s="12"/>
       <c r="H21" s="12"/>
@@ -15414,19 +15419,35 @@
       <c r="J21" s="12"/>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A22" s="12"/>
-      <c r="B22" s="12"/>
-      <c r="C22" s="12"/>
-      <c r="D22" s="12"/>
+      <c r="A22" s="12">
+        <v>20</v>
+      </c>
+      <c r="B22" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>59</v>
+      </c>
       <c r="E22" s="13" t="str">
-        <f>IF(D22="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D22,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
-        <v/>
-      </c>
-      <c r="F22" s="14"/>
-      <c r="G22" s="12"/>
-      <c r="H22" s="12"/>
+        <f>IF(D22="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D22,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
+        <v>→ —</v>
+      </c>
+      <c r="F22" s="14" t="s">
+        <v>120</v>
+      </c>
+      <c r="G22" s="12">
+        <v>10</v>
+      </c>
+      <c r="H22" s="12" t="s">
+        <v>84</v>
+      </c>
       <c r="I22" s="12"/>
-      <c r="J22" s="12"/>
+      <c r="J22" s="12" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="12"/>
@@ -15434,7 +15455,7 @@
       <c r="C23" s="12"/>
       <c r="D23" s="12"/>
       <c r="E23" s="13" t="str">
-        <f>IF(D23="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D23,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D23="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D23,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F23" s="14"/>
@@ -15449,7 +15470,7 @@
       <c r="C24" s="12"/>
       <c r="D24" s="12"/>
       <c r="E24" s="13" t="str">
-        <f>IF(D24="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D24,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D24="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D24,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F24" s="14"/>
@@ -15464,7 +15485,7 @@
       <c r="C25" s="12"/>
       <c r="D25" s="12"/>
       <c r="E25" s="13" t="str">
-        <f>IF(D25="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D25,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D25="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D25,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F25" s="14"/>
@@ -15479,7 +15500,7 @@
       <c r="C26" s="12"/>
       <c r="D26" s="12"/>
       <c r="E26" s="13" t="str">
-        <f>IF(D26="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D26,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D26="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D26,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F26" s="14"/>
@@ -15494,7 +15515,7 @@
       <c r="C27" s="12"/>
       <c r="D27" s="12"/>
       <c r="E27" s="13" t="str">
-        <f>IF(D27="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D27,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D27="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D27,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F27" s="14"/>
@@ -15509,7 +15530,7 @@
       <c r="C28" s="12"/>
       <c r="D28" s="12"/>
       <c r="E28" s="13" t="str">
-        <f>IF(D28="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D28,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D28="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D28,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F28" s="14"/>
@@ -15524,7 +15545,7 @@
       <c r="C29" s="12"/>
       <c r="D29" s="12"/>
       <c r="E29" s="13" t="str">
-        <f>IF(D29="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D29,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D29="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D29,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F29" s="14"/>
@@ -15539,7 +15560,7 @@
       <c r="C30" s="12"/>
       <c r="D30" s="12"/>
       <c r="E30" s="13" t="str">
-        <f>IF(D30="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D30,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D30="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D30,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F30" s="14"/>
@@ -15554,7 +15575,7 @@
       <c r="C31" s="12"/>
       <c r="D31" s="12"/>
       <c r="E31" s="13" t="str">
-        <f>IF(D31="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D31,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D31="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D31,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F31" s="14"/>
@@ -15569,7 +15590,7 @@
       <c r="C32" s="12"/>
       <c r="D32" s="12"/>
       <c r="E32" s="13" t="str">
-        <f>IF(D32="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D32,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D32="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D32,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F32" s="14"/>
@@ -15584,7 +15605,7 @@
       <c r="C33" s="12"/>
       <c r="D33" s="12"/>
       <c r="E33" s="13" t="str">
-        <f>IF(D33="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D33,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D33="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D33,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F33" s="14"/>
@@ -15599,7 +15620,7 @@
       <c r="C34" s="12"/>
       <c r="D34" s="12"/>
       <c r="E34" s="13" t="str">
-        <f>IF(D34="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D34,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D34="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D34,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F34" s="14"/>
@@ -15614,7 +15635,7 @@
       <c r="C35" s="12"/>
       <c r="D35" s="12"/>
       <c r="E35" s="13" t="str">
-        <f>IF(D35="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D35,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D35="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D35,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F35" s="14"/>
@@ -15629,7 +15650,7 @@
       <c r="C36" s="12"/>
       <c r="D36" s="12"/>
       <c r="E36" s="13" t="str">
-        <f>IF(D36="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D36,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D36="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D36,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F36" s="14"/>
@@ -15644,7 +15665,7 @@
       <c r="C37" s="12"/>
       <c r="D37" s="12"/>
       <c r="E37" s="13" t="str">
-        <f>IF(D37="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D37,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D37="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D37,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F37" s="14"/>
@@ -15659,7 +15680,7 @@
       <c r="C38" s="12"/>
       <c r="D38" s="12"/>
       <c r="E38" s="13" t="str">
-        <f>IF(D38="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D38,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D38="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D38,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F38" s="14"/>
@@ -15674,7 +15695,7 @@
       <c r="C39" s="12"/>
       <c r="D39" s="12"/>
       <c r="E39" s="13" t="str">
-        <f>IF(D39="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D39,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D39="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D39,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F39" s="14"/>
@@ -15689,7 +15710,7 @@
       <c r="C40" s="12"/>
       <c r="D40" s="12"/>
       <c r="E40" s="13" t="str">
-        <f>IF(D40="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D40,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D40="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D40,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F40" s="14"/>
@@ -15704,7 +15725,7 @@
       <c r="C41" s="12"/>
       <c r="D41" s="12"/>
       <c r="E41" s="13" t="str">
-        <f>IF(D41="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D41,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D41="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D41,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F41" s="14"/>
@@ -15719,7 +15740,7 @@
       <c r="C42" s="12"/>
       <c r="D42" s="12"/>
       <c r="E42" s="13" t="str">
-        <f>IF(D42="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D42,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D42="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D42,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F42" s="14"/>
@@ -15734,7 +15755,7 @@
       <c r="C43" s="12"/>
       <c r="D43" s="12"/>
       <c r="E43" s="13" t="str">
-        <f>IF(D43="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D43,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D43="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D43,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F43" s="14"/>
@@ -15749,7 +15770,7 @@
       <c r="C44" s="12"/>
       <c r="D44" s="12"/>
       <c r="E44" s="13" t="str">
-        <f>IF(D44="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D44,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D44="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D44,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F44" s="14"/>
@@ -15764,7 +15785,7 @@
       <c r="C45" s="12"/>
       <c r="D45" s="12"/>
       <c r="E45" s="13" t="str">
-        <f>IF(D45="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D45,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D45="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D45,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F45" s="14"/>
@@ -15779,7 +15800,7 @@
       <c r="C46" s="12"/>
       <c r="D46" s="12"/>
       <c r="E46" s="13" t="str">
-        <f>IF(D46="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D46,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D46="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D46,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F46" s="14"/>
@@ -15794,7 +15815,7 @@
       <c r="C47" s="12"/>
       <c r="D47" s="12"/>
       <c r="E47" s="13" t="str">
-        <f>IF(D47="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D47,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D47="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D47,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F47" s="14"/>
@@ -15809,7 +15830,7 @@
       <c r="C48" s="12"/>
       <c r="D48" s="12"/>
       <c r="E48" s="13" t="str">
-        <f>IF(D48="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D48,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D48="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D48,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F48" s="14"/>
@@ -15824,7 +15845,7 @@
       <c r="C49" s="12"/>
       <c r="D49" s="12"/>
       <c r="E49" s="13" t="str">
-        <f>IF(D49="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D49,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D49="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D49,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F49" s="14"/>
@@ -15839,7 +15860,7 @@
       <c r="C50" s="12"/>
       <c r="D50" s="12"/>
       <c r="E50" s="13" t="str">
-        <f>IF(D50="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D50,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D50="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D50,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F50" s="14"/>
@@ -15854,7 +15875,7 @@
       <c r="C51" s="12"/>
       <c r="D51" s="12"/>
       <c r="E51" s="13" t="str">
-        <f>IF(D51="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D51,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D51="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D51,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F51" s="14"/>
@@ -15869,7 +15890,7 @@
       <c r="C52" s="12"/>
       <c r="D52" s="12"/>
       <c r="E52" s="13" t="str">
-        <f>IF(D52="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D52,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D52="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D52,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F52" s="14"/>
@@ -15884,7 +15905,7 @@
       <c r="C53" s="12"/>
       <c r="D53" s="12"/>
       <c r="E53" s="13" t="str">
-        <f>IF(D53="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D53,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D53="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D53,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F53" s="14"/>
@@ -15899,7 +15920,7 @@
       <c r="C54" s="12"/>
       <c r="D54" s="12"/>
       <c r="E54" s="13" t="str">
-        <f>IF(D54="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D54,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D54="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D54,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F54" s="14"/>
@@ -15914,7 +15935,7 @@
       <c r="C55" s="12"/>
       <c r="D55" s="12"/>
       <c r="E55" s="13" t="str">
-        <f>IF(D55="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D55,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D55="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D55,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F55" s="14"/>
@@ -15929,7 +15950,7 @@
       <c r="C56" s="12"/>
       <c r="D56" s="12"/>
       <c r="E56" s="13" t="str">
-        <f>IF(D56="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D56,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D56="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D56,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F56" s="14"/>
@@ -15944,7 +15965,7 @@
       <c r="C57" s="12"/>
       <c r="D57" s="12"/>
       <c r="E57" s="13" t="str">
-        <f>IF(D57="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D57,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D57="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D57,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F57" s="14"/>
@@ -15959,7 +15980,7 @@
       <c r="C58" s="12"/>
       <c r="D58" s="12"/>
       <c r="E58" s="13" t="str">
-        <f>IF(D58="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D58,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D58="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D58,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F58" s="14"/>
@@ -15974,7 +15995,7 @@
       <c r="C59" s="12"/>
       <c r="D59" s="12"/>
       <c r="E59" s="13" t="str">
-        <f>IF(D59="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D59,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D59="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D59,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F59" s="14"/>
@@ -15989,7 +16010,7 @@
       <c r="C60" s="12"/>
       <c r="D60" s="12"/>
       <c r="E60" s="13" t="str">
-        <f>IF(D60="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D60,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D60="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D60,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F60" s="14"/>
@@ -16004,7 +16025,7 @@
       <c r="C61" s="12"/>
       <c r="D61" s="12"/>
       <c r="E61" s="13" t="str">
-        <f>IF(D61="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D61,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D61="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D61,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F61" s="14"/>
@@ -16019,7 +16040,7 @@
       <c r="C62" s="12"/>
       <c r="D62" s="12"/>
       <c r="E62" s="13" t="str">
-        <f>IF(D62="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D62,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D62="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D62,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F62" s="14"/>
@@ -16034,7 +16055,7 @@
       <c r="C63" s="12"/>
       <c r="D63" s="12"/>
       <c r="E63" s="13" t="str">
-        <f>IF(D63="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D63,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D63="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D63,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F63" s="14"/>
@@ -16049,7 +16070,7 @@
       <c r="C64" s="12"/>
       <c r="D64" s="12"/>
       <c r="E64" s="13" t="str">
-        <f>IF(D64="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D64,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D64="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D64,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F64" s="14"/>
@@ -16064,7 +16085,7 @@
       <c r="C65" s="12"/>
       <c r="D65" s="12"/>
       <c r="E65" s="13" t="str">
-        <f>IF(D65="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D65,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D65="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D65,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F65" s="14"/>
@@ -16079,7 +16100,7 @@
       <c r="C66" s="12"/>
       <c r="D66" s="12"/>
       <c r="E66" s="13" t="str">
-        <f>IF(D66="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D66,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D66="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D66,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F66" s="14"/>
@@ -16094,7 +16115,7 @@
       <c r="C67" s="12"/>
       <c r="D67" s="12"/>
       <c r="E67" s="13" t="str">
-        <f>IF(D67="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D67,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D67="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D67,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F67" s="14"/>
@@ -16109,7 +16130,7 @@
       <c r="C68" s="12"/>
       <c r="D68" s="12"/>
       <c r="E68" s="13" t="str">
-        <f>IF(D68="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D68,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D68="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D68,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F68" s="14"/>
@@ -16124,7 +16145,7 @@
       <c r="C69" s="12"/>
       <c r="D69" s="12"/>
       <c r="E69" s="13" t="str">
-        <f>IF(D69="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D69,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D69="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D69,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F69" s="14"/>
@@ -16139,7 +16160,7 @@
       <c r="C70" s="12"/>
       <c r="D70" s="12"/>
       <c r="E70" s="13" t="str">
-        <f>IF(D70="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D70,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D70="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D70,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F70" s="14"/>
@@ -16154,7 +16175,7 @@
       <c r="C71" s="12"/>
       <c r="D71" s="12"/>
       <c r="E71" s="13" t="str">
-        <f>IF(D71="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D71,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D71="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D71,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F71" s="14"/>
@@ -16169,7 +16190,7 @@
       <c r="C72" s="12"/>
       <c r="D72" s="12"/>
       <c r="E72" s="13" t="str">
-        <f>IF(D72="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D72,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D72="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D72,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F72" s="14"/>
@@ -16184,7 +16205,7 @@
       <c r="C73" s="12"/>
       <c r="D73" s="12"/>
       <c r="E73" s="13" t="str">
-        <f>IF(D73="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D73,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D73="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D73,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F73" s="14"/>
@@ -16199,7 +16220,7 @@
       <c r="C74" s="12"/>
       <c r="D74" s="12"/>
       <c r="E74" s="13" t="str">
-        <f>IF(D74="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D74,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D74="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D74,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F74" s="14"/>
@@ -16214,7 +16235,7 @@
       <c r="C75" s="12"/>
       <c r="D75" s="12"/>
       <c r="E75" s="13" t="str">
-        <f>IF(D75="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D75,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D75="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D75,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F75" s="14"/>
@@ -16229,7 +16250,7 @@
       <c r="C76" s="12"/>
       <c r="D76" s="12"/>
       <c r="E76" s="13" t="str">
-        <f>IF(D76="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D76,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D76="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D76,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F76" s="14"/>
@@ -16244,7 +16265,7 @@
       <c r="C77" s="12"/>
       <c r="D77" s="12"/>
       <c r="E77" s="13" t="str">
-        <f>IF(D77="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D77,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D77="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D77,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F77" s="14"/>
@@ -16259,7 +16280,7 @@
       <c r="C78" s="12"/>
       <c r="D78" s="12"/>
       <c r="E78" s="13" t="str">
-        <f>IF(D78="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D78,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D78="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D78,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F78" s="14"/>
@@ -16274,7 +16295,7 @@
       <c r="C79" s="12"/>
       <c r="D79" s="12"/>
       <c r="E79" s="13" t="str">
-        <f>IF(D79="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D79,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D79="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D79,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F79" s="14"/>
@@ -16289,7 +16310,7 @@
       <c r="C80" s="12"/>
       <c r="D80" s="12"/>
       <c r="E80" s="13" t="str">
-        <f>IF(D80="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D80,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D80="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D80,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F80" s="14"/>
@@ -16304,7 +16325,7 @@
       <c r="C81" s="12"/>
       <c r="D81" s="12"/>
       <c r="E81" s="13" t="str">
-        <f>IF(D81="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D81,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D81="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D81,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F81" s="14"/>
@@ -16319,7 +16340,7 @@
       <c r="C82" s="12"/>
       <c r="D82" s="12"/>
       <c r="E82" s="13" t="str">
-        <f>IF(D82="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D82,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D82="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D82,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F82" s="14"/>
@@ -16334,7 +16355,7 @@
       <c r="C83" s="12"/>
       <c r="D83" s="12"/>
       <c r="E83" s="13" t="str">
-        <f>IF(D83="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D83,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D83="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D83,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F83" s="14"/>
@@ -16349,7 +16370,7 @@
       <c r="C84" s="12"/>
       <c r="D84" s="12"/>
       <c r="E84" s="13" t="str">
-        <f>IF(D84="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D84,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D84="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D84,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F84" s="14"/>
@@ -16364,7 +16385,7 @@
       <c r="C85" s="12"/>
       <c r="D85" s="12"/>
       <c r="E85" s="13" t="str">
-        <f>IF(D85="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D85,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D85="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D85,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F85" s="14"/>
@@ -16379,7 +16400,7 @@
       <c r="C86" s="12"/>
       <c r="D86" s="12"/>
       <c r="E86" s="13" t="str">
-        <f>IF(D86="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D86,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D86="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D86,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F86" s="14"/>
@@ -16394,7 +16415,7 @@
       <c r="C87" s="12"/>
       <c r="D87" s="12"/>
       <c r="E87" s="13" t="str">
-        <f>IF(D87="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D87,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D87="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D87,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F87" s="14"/>
@@ -16409,7 +16430,7 @@
       <c r="C88" s="12"/>
       <c r="D88" s="12"/>
       <c r="E88" s="13" t="str">
-        <f>IF(D88="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D88,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D88="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D88,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F88" s="14"/>
@@ -16424,7 +16445,7 @@
       <c r="C89" s="12"/>
       <c r="D89" s="12"/>
       <c r="E89" s="13" t="str">
-        <f>IF(D89="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D89,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D89="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D89,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F89" s="14"/>
@@ -16439,7 +16460,7 @@
       <c r="C90" s="12"/>
       <c r="D90" s="12"/>
       <c r="E90" s="13" t="str">
-        <f>IF(D90="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D90,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D90="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D90,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F90" s="14"/>
@@ -16454,7 +16475,7 @@
       <c r="C91" s="12"/>
       <c r="D91" s="12"/>
       <c r="E91" s="13" t="str">
-        <f>IF(D91="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D91,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D91="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D91,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F91" s="14"/>
@@ -16469,7 +16490,7 @@
       <c r="C92" s="12"/>
       <c r="D92" s="12"/>
       <c r="E92" s="13" t="str">
-        <f>IF(D92="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D92,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D92="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D92,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F92" s="14"/>
@@ -16484,7 +16505,7 @@
       <c r="C93" s="12"/>
       <c r="D93" s="12"/>
       <c r="E93" s="13" t="str">
-        <f>IF(D93="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D93,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D93="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D93,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F93" s="14"/>
@@ -16499,7 +16520,7 @@
       <c r="C94" s="12"/>
       <c r="D94" s="12"/>
       <c r="E94" s="13" t="str">
-        <f>IF(D94="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D94,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D94="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D94,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F94" s="14"/>
@@ -16514,7 +16535,7 @@
       <c r="C95" s="12"/>
       <c r="D95" s="12"/>
       <c r="E95" s="13" t="str">
-        <f>IF(D95="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D95,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D95="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D95,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F95" s="14"/>
@@ -16529,7 +16550,7 @@
       <c r="C96" s="12"/>
       <c r="D96" s="12"/>
       <c r="E96" s="13" t="str">
-        <f>IF(D96="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D96,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D96="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D96,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F96" s="14"/>
@@ -16544,7 +16565,7 @@
       <c r="C97" s="12"/>
       <c r="D97" s="12"/>
       <c r="E97" s="13" t="str">
-        <f>IF(D97="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D97,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D97="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D97,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F97" s="14"/>
@@ -16559,7 +16580,7 @@
       <c r="C98" s="12"/>
       <c r="D98" s="12"/>
       <c r="E98" s="13" t="str">
-        <f>IF(D98="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D98,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D98="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D98,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F98" s="14"/>
@@ -16574,7 +16595,7 @@
       <c r="C99" s="12"/>
       <c r="D99" s="12"/>
       <c r="E99" s="13" t="str">
-        <f>IF(D99="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D99,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D99="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D99,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F99" s="14"/>
@@ -16589,7 +16610,7 @@
       <c r="C100" s="12"/>
       <c r="D100" s="12"/>
       <c r="E100" s="13" t="str">
-        <f>IF(D100="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid"},MATCH(D100,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games"},0)),"¿tipo?"))</f>
+        <f>IF(D100="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D100,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
         <v/>
       </c>
       <c r="F100" s="14"/>
@@ -17817,10 +17838,10 @@
       <formula1>"Sí,No"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Valor no previsto" error="Elige un valor de la lista." sqref="D10:D200">
-      <formula1>"Pulsador,Test,Verdad o mentira,Dos verdades y una mentira,Votación,Estimación,Parar el contador,Duelo de reflejos,Libre,Palabras secretas,Agita el móvil,La gran apuesta,Squid Games"</formula1>
+      <formula1>"Pulsador,Test,Verdad o mentira,Dos verdades y una mentira,Votación,Estimación,Parar el contador,Duelo de reflejos,Libre,Palabras secretas,Agita el móvil,La gran apuesta,Squid Games,Lobos contra vampiros"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Valor no previsto" error="Elige un valor de la lista." sqref="D3:D200">
-      <formula1>"Pulsador,Test,Verdad o mentira,Dos verdades y una mentira,Votación,Estimación,Parar el contador,Duelo de reflejos,Libre,Palabras secretas,Agita el móvil,La gran apuesta,Squid Games"</formula1>
+      <formula1>"Pulsador,Test,Verdad o mentira,Dos verdades y una mentira,Votación,Estimación,Parar el contador,Duelo de reflejos,Libre,Palabras secretas,Agita el móvil,La gran apuesta,Squid Games,Lobos contra vampiros"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Valor no previsto" error="Elige un valor de la lista." sqref="H10:I200">
       <formula1>"Sí,No"</formula1>
@@ -17829,10 +17850,10 @@
       <formula1>"Sí,No"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Valor no previsto" error="Elige un valor de la lista." sqref="J10:J200">
-      <formula1>"Noche de luna,Cementerio,Bosque encantado,Huerto de calabazas,Laboratorio,Mansión encantada,Telaraña,Aquelarre,Cripta helada,Tormenta,Plató millonario,Squid Games"</formula1>
+      <formula1>"Noche de luna,Cementerio,Bosque encantado,Huerto de calabazas,Laboratorio,Mansión encantada,Telaraña,Aquelarre,Cripta helada,Tormenta,Plató millonario,Squid Games,Discoteca,Luna llena"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Valor no previsto" error="Elige un valor de la lista." sqref="J3:J200">
-      <formula1>"Noche de luna,Cementerio,Bosque encantado,Huerto de calabazas,Laboratorio,Mansión encantada,Telaraña,Aquelarre,Cripta helada,Tormenta,Plató millonario,Squid Games"</formula1>
+      <formula1>"Noche de luna,Cementerio,Bosque encantado,Huerto de calabazas,Laboratorio,Mansión encantada,Telaraña,Aquelarre,Cripta helada,Tormenta,Plató millonario,Squid Games,Discoteca,Luna llena"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -17854,34 +17875,34 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:2" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" ht="42" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -18697,134 +18718,134 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:3" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2" ht="42" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="B4" s="12">
         <v>1</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="B5" s="12">
         <v>1</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="B6" s="12">
         <v>1</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="B7" s="12">
         <v>1</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="B8" s="12">
         <v>0</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="B10" s="12">
         <v>20</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="B11" s="12">
         <v>60</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="B12" s="12">
         <v>3</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -19791,276 +19812,276 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" ht="42" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="G2" s="11" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D3" s="14"/>
       <c r="E3" s="12"/>
       <c r="F3" s="12"/>
       <c r="G3" s="12" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D4" s="14"/>
       <c r="E4" s="12"/>
       <c r="F4" s="12"/>
       <c r="G4" s="12" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D5" s="14"/>
       <c r="E5" s="12"/>
       <c r="F5" s="12"/>
       <c r="G5" s="12" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D6" s="14"/>
       <c r="E6" s="12"/>
       <c r="F6" s="12"/>
       <c r="G6" s="12" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D7" s="14"/>
       <c r="E7" s="12"/>
       <c r="F7" s="12"/>
       <c r="G7" s="12" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D8" s="14"/>
       <c r="E8" s="12"/>
       <c r="F8" s="12"/>
       <c r="G8" s="12" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="E9" s="12"/>
       <c r="F9" s="12"/>
       <c r="G9" s="12" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="E10" s="12"/>
       <c r="F10" s="12"/>
       <c r="G10" s="12" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="E11" s="12"/>
       <c r="F11" s="12"/>
       <c r="G11" s="12" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="F12" s="12">
         <v>0</v>
       </c>
       <c r="G12" s="12" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="F13" s="12">
         <v>0</v>
       </c>
       <c r="G13" s="12" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="F14" s="12">
         <v>0</v>
       </c>
       <c r="G14" s="12" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -21775,358 +21796,358 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:9" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" ht="42" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="G2" s="11" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="H2" s="11" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="I2" s="11" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="F3" s="12" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="G3" s="12" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="H3" s="12"/>
       <c r="I3" s="12"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="H4" s="12"/>
       <c r="I4" s="12"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
+        <v>226</v>
+      </c>
+      <c r="B5" s="14" t="s">
+        <v>227</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>228</v>
+      </c>
+      <c r="D5" s="14" t="s">
+        <v>229</v>
+      </c>
+      <c r="E5" s="14" t="s">
+        <v>230</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>202</v>
+      </c>
+      <c r="G5" s="12" t="s">
         <v>220</v>
-      </c>
-      <c r="B5" s="14" t="s">
-        <v>221</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>222</v>
-      </c>
-      <c r="D5" s="14" t="s">
-        <v>223</v>
-      </c>
-      <c r="E5" s="14" t="s">
-        <v>224</v>
-      </c>
-      <c r="F5" s="12" t="s">
-        <v>196</v>
-      </c>
-      <c r="G5" s="12" t="s">
-        <v>214</v>
       </c>
       <c r="H5" s="12"/>
       <c r="I5" s="12"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>226</v>
+        <v>232</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>227</v>
+        <v>233</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="G6" s="12" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="H6" s="12"/>
       <c r="I6" s="12"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
       <c r="F7" s="12" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="G7" s="12" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
       <c r="H7" s="12"/>
       <c r="I7" s="12"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="G8" s="12" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
       <c r="H8" s="12"/>
       <c r="I8" s="12"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="B9" s="14" t="s">
+        <v>247</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>248</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>249</v>
+      </c>
+      <c r="E9" s="14" t="s">
+        <v>250</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>202</v>
+      </c>
+      <c r="G9" s="12" t="s">
         <v>241</v>
-      </c>
-      <c r="C9" s="14" t="s">
-        <v>242</v>
-      </c>
-      <c r="D9" s="14" t="s">
-        <v>243</v>
-      </c>
-      <c r="E9" s="14" t="s">
-        <v>244</v>
-      </c>
-      <c r="F9" s="12" t="s">
-        <v>196</v>
-      </c>
-      <c r="G9" s="12" t="s">
-        <v>235</v>
       </c>
       <c r="H9" s="12"/>
       <c r="I9" s="12"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>248</v>
+        <v>254</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>249</v>
+        <v>255</v>
       </c>
       <c r="F10" s="12" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="G10" s="12" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
       <c r="H10" s="12"/>
       <c r="I10" s="12"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>252</v>
+        <v>258</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="F11" s="12" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="G11" s="12" t="s">
-        <v>255</v>
+        <v>261</v>
       </c>
       <c r="H11" s="12"/>
       <c r="I11" s="12"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="F12" s="12" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="G12" s="12" t="s">
-        <v>255</v>
+        <v>261</v>
       </c>
       <c r="H12" s="12"/>
       <c r="I12" s="12"/>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
+        <v>267</v>
+      </c>
+      <c r="B13" s="14" t="s">
+        <v>268</v>
+      </c>
+      <c r="C13" s="14" t="s">
+        <v>269</v>
+      </c>
+      <c r="D13" s="14" t="s">
+        <v>270</v>
+      </c>
+      <c r="E13" s="14" t="s">
+        <v>271</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>202</v>
+      </c>
+      <c r="G13" s="12" t="s">
         <v>261</v>
-      </c>
-      <c r="B13" s="14" t="s">
-        <v>262</v>
-      </c>
-      <c r="C13" s="14" t="s">
-        <v>263</v>
-      </c>
-      <c r="D13" s="14" t="s">
-        <v>264</v>
-      </c>
-      <c r="E13" s="14" t="s">
-        <v>265</v>
-      </c>
-      <c r="F13" s="12" t="s">
-        <v>196</v>
-      </c>
-      <c r="G13" s="12" t="s">
-        <v>255</v>
       </c>
       <c r="H13" s="12"/>
       <c r="I13" s="12"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>270</v>
+        <v>276</v>
       </c>
       <c r="F14" s="12" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="G14" s="12" t="s">
-        <v>255</v>
+        <v>261</v>
       </c>
       <c r="H14" s="12"/>
       <c r="I14" s="12"/>
@@ -24253,95 +24274,95 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:3" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" ht="42" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>272</v>
+        <v>278</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>274</v>
+        <v>280</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>275</v>
+        <v>281</v>
       </c>
       <c r="C3" s="12"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>276</v>
+        <v>282</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
       <c r="C4" s="12"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
       <c r="C5" s="12"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>279</v>
+        <v>285</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>275</v>
+        <v>281</v>
       </c>
       <c r="C6" s="12"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>280</v>
+        <v>286</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>275</v>
+        <v>281</v>
       </c>
       <c r="C7" s="12"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
+        <v>287</v>
+      </c>
+      <c r="B8" s="12" t="s">
         <v>281</v>
-      </c>
-      <c r="B8" s="12" t="s">
-        <v>275</v>
       </c>
       <c r="C8" s="12"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>282</v>
+        <v>288</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
       <c r="C9" s="12"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
+        <v>289</v>
+      </c>
+      <c r="B10" s="12" t="s">
         <v>283</v>
-      </c>
-      <c r="B10" s="12" t="s">
-        <v>277</v>
       </c>
       <c r="C10" s="12"/>
     </row>
@@ -25340,56 +25361,56 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>286</v>
+        <v>292</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" ht="42" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>289</v>
+        <v>295</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>290</v>
+        <v>296</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>291</v>
+        <v>297</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>292</v>
+        <v>298</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>293</v>
+        <v>299</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>294</v>
+        <v>300</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>295</v>
+        <v>301</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>296</v>
+        <v>302</v>
       </c>
       <c r="E3" s="12">
         <v>2</v>
@@ -25398,16 +25419,16 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>297</v>
+        <v>303</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>298</v>
+        <v>304</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>299</v>
+        <v>305</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>300</v>
+        <v>306</v>
       </c>
       <c r="E4" s="12">
         <v>3</v>
@@ -25416,16 +25437,16 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>302</v>
+        <v>308</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>303</v>
+        <v>309</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="E5" s="12">
         <v>1</v>
@@ -25434,16 +25455,16 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>307</v>
+        <v>313</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="E6" s="12">
         <v>2</v>
@@ -25452,16 +25473,16 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>310</v>
+        <v>316</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="E7" s="12">
         <v>3</v>
@@ -25470,16 +25491,16 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>313</v>
+        <v>319</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>314</v>
+        <v>320</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>316</v>
+        <v>322</v>
       </c>
       <c r="E8" s="12">
         <v>2</v>
@@ -25488,16 +25509,16 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>317</v>
+        <v>323</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>318</v>
+        <v>324</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>319</v>
+        <v>325</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>320</v>
+        <v>326</v>
       </c>
       <c r="E9" s="12">
         <v>2</v>
@@ -27081,65 +27102,65 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:2" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" ht="42" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>321</v>
+        <v>327</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>322</v>
+        <v>328</v>
       </c>
       <c r="B3" s="12"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>323</v>
+        <v>329</v>
       </c>
       <c r="B4" s="12"/>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="B5" s="12"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>325</v>
+        <v>331</v>
       </c>
       <c r="B6" s="12"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>326</v>
+        <v>332</v>
       </c>
       <c r="B7" s="12"/>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>327</v>
+        <v>333</v>
       </c>
       <c r="B8" s="12"/>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>328</v>
+        <v>334</v>
       </c>
       <c r="B9" s="12"/>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>329</v>
+        <v>335</v>
       </c>
       <c r="B10" s="12"/>
     </row>

</xml_diff>

<commit_message>
Temáticas, dos presentadores, penalizar y silenciar desde el mando, y ajustes de juego
- Libre: todas con cuenta atrás 3-2-1 y reloj; el contador solo desde el mando; fundido en marcar el golpe
- Mando: 🔇 silenciar la tele, ⚖️ quitar puntos por trampas (aviso en la tele), dos presentadores que se turnan
- Pañuelo: ¡ya! en cuanto la ruleta se para; Squid sin voz de megafonía; luz roja más dura; panal más exigente y sin rastro de la aguja
- Temáticas Verano (Watermelon Sugar, sección nueva), Galletas y Refrescos con decorado flotante; vídeo del twerking sin fondo negro
- Música: una canción suelta en Música/<Sección>/ suena en toda la sección
- Botellas por jugador; título sin «pulsa cualquier tecla»

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/plantilla-concurso.xlsx
+++ b/public/plantilla-concurso.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="751" uniqueCount="502">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="763" uniqueCount="508">
   <si>
     <t>EMPIEZA AQUÍ</t>
   </si>
@@ -369,12 +369,27 @@
     <t>Con las manos atadas a la espalda: el primero que se coma la galleta, gana.</t>
   </si>
   <si>
+    <t>Galletas</t>
+  </si>
+  <si>
     <t>Botellas en orden</t>
   </si>
   <si>
     <t>Adivina el orden de las 5 botellas: en cada intento te decimos cuántas están bien. Gana el más rápido.</t>
   </si>
   <si>
+    <t>Refrescos</t>
+  </si>
+  <si>
+    <t>Watermelon Sugar</t>
+  </si>
+  <si>
+    <t>Uno de cada equipo, una sandía cada uno: ¡el primero que se la acabe, gana!</t>
+  </si>
+  <si>
+    <t>Verano</t>
+  </si>
+  <si>
     <t>Fit o Fat</t>
   </si>
   <si>
@@ -1222,6 +1237,9 @@
   </si>
   <si>
     <t>Contrarreloj</t>
+  </si>
+  <si>
+    <t>Dos participantes, una sandía cada uno: el primero que se la coma entera, gana.</t>
   </si>
   <si>
     <t>Golpe 1</t>
@@ -2479,16 +2497,16 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>337</v>
+        <v>342</v>
       </c>
       <c r="E1" s="10" t="s">
         <v>64</v>
@@ -2496,136 +2514,136 @@
     </row>
     <row r="2" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="B3" s="12">
         <v>910</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="E3" s="12"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="B4" s="12">
         <v>1247</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="E4" s="12"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="B5" s="12">
         <v>1897</v>
       </c>
       <c r="C5" s="12"/>
       <c r="D5" s="12" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="E5" s="12"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="B6" s="12">
         <v>330</v>
       </c>
       <c r="C6" s="12" t="s">
+        <v>354</v>
+      </c>
+      <c r="D6" s="12" t="s">
         <v>349</v>
-      </c>
-      <c r="D6" s="12" t="s">
-        <v>344</v>
       </c>
       <c r="E6" s="12"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>350</v>
+        <v>355</v>
       </c>
       <c r="B7" s="12">
         <v>88</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>351</v>
+        <v>356</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
       <c r="E7" s="12"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>353</v>
+        <v>358</v>
       </c>
       <c r="B8" s="12">
         <v>505</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="E8" s="12"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>354</v>
+        <v>359</v>
       </c>
       <c r="B9" s="12">
         <v>40</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>355</v>
+        <v>360</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
       <c r="E9" s="12"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>356</v>
+        <v>361</v>
       </c>
       <c r="B10" s="12">
         <v>32</v>
       </c>
       <c r="C10" s="12" t="s">
+        <v>362</v>
+      </c>
+      <c r="D10" s="12" t="s">
         <v>357</v>
-      </c>
-      <c r="D10" s="12" t="s">
-        <v>352</v>
       </c>
       <c r="E10" s="12"/>
     </row>
@@ -3994,13 +4012,13 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>359</v>
+        <v>364</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>360</v>
+        <v>365</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>64</v>
@@ -4008,16 +4026,16 @@
     </row>
     <row r="2" ht="42" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>361</v>
+        <v>366</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>362</v>
+        <v>367</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>363</v>
+        <v>368</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -4025,7 +4043,7 @@
         <v>10</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="C3" s="12"/>
       <c r="D3" s="12"/>
@@ -4035,7 +4053,7 @@
         <v>15</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
       <c r="C4" s="12">
         <v>3</v>
@@ -4047,7 +4065,7 @@
         <v>7</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>366</v>
+        <v>371</v>
       </c>
       <c r="C5" s="12"/>
       <c r="D5" s="12"/>
@@ -4057,7 +4075,7 @@
         <v>12</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
       <c r="C6" s="12">
         <v>5</v>
@@ -4069,7 +4087,7 @@
         <v>20</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>366</v>
+        <v>371</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12"/>
@@ -5267,10 +5285,10 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:3" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>367</v>
+        <v>372</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>368</v>
+        <v>373</v>
       </c>
       <c r="C1" s="10" t="s">
         <v>64</v>
@@ -5278,13 +5296,13 @@
     </row>
     <row r="2" ht="42" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>370</v>
+        <v>375</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -5292,7 +5310,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>371</v>
+        <v>376</v>
       </c>
       <c r="C3" s="12"/>
     </row>
@@ -5301,7 +5319,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>372</v>
+        <v>377</v>
       </c>
       <c r="C4" s="12"/>
     </row>
@@ -5310,7 +5328,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>371</v>
+        <v>376</v>
       </c>
       <c r="C5" s="12"/>
     </row>
@@ -6327,28 +6345,28 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:9" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="B1" s="10" t="s">
         <v>66</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>374</v>
+        <v>379</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>368</v>
+        <v>373</v>
       </c>
       <c r="E1" s="10" t="s">
         <v>67</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>375</v>
+        <v>380</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="I1" s="10" t="s">
         <v>64</v>
@@ -6356,31 +6374,31 @@
     </row>
     <row r="2" ht="42" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>377</v>
+        <v>382</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>378</v>
+        <v>383</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="G2" s="11" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="H2" s="11" t="s">
-        <v>383</v>
+        <v>388</v>
       </c>
       <c r="I2" s="11" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -6388,13 +6406,13 @@
         <v>93</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>386</v>
+        <v>391</v>
       </c>
       <c r="E3" s="12"/>
       <c r="F3" s="12"/>
@@ -6406,16 +6424,16 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>387</v>
+        <v>392</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>388</v>
+        <v>393</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>386</v>
+        <v>391</v>
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="12"/>
@@ -6430,13 +6448,13 @@
         <v>103</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>390</v>
+        <v>395</v>
       </c>
       <c r="E5" s="12"/>
       <c r="F5" s="12"/>
@@ -6448,16 +6466,16 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>391</v>
+        <v>396</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>392</v>
+        <v>397</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>390</v>
+        <v>395</v>
       </c>
       <c r="E6" s="12"/>
       <c r="F6" s="12"/>
@@ -6472,13 +6490,13 @@
         <v>111</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>393</v>
+        <v>398</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>390</v>
+        <v>395</v>
       </c>
       <c r="E7" s="12"/>
       <c r="F7" s="12"/>
@@ -6490,16 +6508,16 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="B8" s="14" t="s">
+        <v>400</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>390</v>
+      </c>
+      <c r="D8" s="12" t="s">
         <v>395</v>
-      </c>
-      <c r="C8" s="12" t="s">
-        <v>385</v>
-      </c>
-      <c r="D8" s="12" t="s">
-        <v>390</v>
       </c>
       <c r="E8" s="12"/>
       <c r="F8" s="12"/>
@@ -6511,16 +6529,16 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>396</v>
+        <v>401</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>397</v>
+        <v>402</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>386</v>
+        <v>395</v>
       </c>
       <c r="E9" s="12"/>
       <c r="F9" s="12">
@@ -6529,51 +6547,47 @@
       <c r="G9" s="12"/>
       <c r="H9" s="12"/>
       <c r="I9" s="12" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>398</v>
+        <v>117</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>400</v>
+        <v>390</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>390</v>
+        <v>395</v>
       </c>
       <c r="E10" s="12"/>
       <c r="F10" s="12"/>
-      <c r="G10" s="12" t="s">
-        <v>401</v>
-      </c>
-      <c r="H10" s="12">
-        <v>0</v>
-      </c>
+      <c r="G10" s="12"/>
+      <c r="H10" s="12"/>
       <c r="I10" s="12" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>400</v>
+        <v>406</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>390</v>
+        <v>395</v>
       </c>
       <c r="E11" s="12"/>
       <c r="F11" s="12"/>
       <c r="G11" s="12" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="H11" s="12">
         <v>0</v>
@@ -6584,21 +6598,21 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="B12" s="14" t="s">
+        <v>409</v>
+      </c>
+      <c r="C12" s="12" t="s">
         <v>406</v>
       </c>
-      <c r="C12" s="12" t="s">
-        <v>400</v>
-      </c>
       <c r="D12" s="12" t="s">
-        <v>390</v>
+        <v>395</v>
       </c>
       <c r="E12" s="12"/>
       <c r="F12" s="12"/>
       <c r="G12" s="12" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="H12" s="12">
         <v>0</v>
@@ -6609,167 +6623,181 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>410</v>
+        <v>406</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>390</v>
+        <v>395</v>
       </c>
       <c r="E13" s="12"/>
       <c r="F13" s="12"/>
-      <c r="G13" s="12"/>
-      <c r="H13" s="12"/>
+      <c r="G13" s="12" t="s">
+        <v>413</v>
+      </c>
+      <c r="H13" s="12">
+        <v>0</v>
+      </c>
       <c r="I13" s="12" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>390</v>
-      </c>
-      <c r="E14" s="12">
-        <v>5</v>
-      </c>
+        <v>395</v>
+      </c>
+      <c r="E14" s="12"/>
       <c r="F14" s="12"/>
       <c r="G14" s="12"/>
       <c r="H14" s="12"/>
       <c r="I14" s="12" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="12" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>413</v>
+        <v>419</v>
       </c>
       <c r="D15" s="12" t="s">
-        <v>390</v>
-      </c>
-      <c r="E15" s="12"/>
+        <v>395</v>
+      </c>
+      <c r="E15" s="12">
+        <v>5</v>
+      </c>
       <c r="F15" s="12"/>
       <c r="G15" s="12"/>
       <c r="H15" s="12"/>
       <c r="I15" s="12" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="12" t="s">
-        <v>416</v>
+        <v>420</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>417</v>
+        <v>421</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>410</v>
+        <v>419</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>390</v>
+        <v>395</v>
       </c>
       <c r="E16" s="12"/>
       <c r="F16" s="12"/>
       <c r="G16" s="12"/>
       <c r="H16" s="12"/>
       <c r="I16" s="12" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="12" t="s">
-        <v>418</v>
+        <v>422</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>419</v>
+        <v>423</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>385</v>
+        <v>416</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>386</v>
-      </c>
-      <c r="E17" s="12">
-        <v>5</v>
-      </c>
+        <v>395</v>
+      </c>
+      <c r="E17" s="12"/>
       <c r="F17" s="12"/>
       <c r="G17" s="12"/>
       <c r="H17" s="12"/>
       <c r="I17" s="12" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="12" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>421</v>
+        <v>425</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>390</v>
-      </c>
-      <c r="E18" s="12"/>
+        <v>391</v>
+      </c>
+      <c r="E18" s="12">
+        <v>5</v>
+      </c>
       <c r="F18" s="12"/>
       <c r="G18" s="12"/>
       <c r="H18" s="12"/>
       <c r="I18" s="12" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
-        <v>422</v>
+        <v>426</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>423</v>
+        <v>427</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>413</v>
+        <v>390</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>386</v>
-      </c>
-      <c r="E19" s="12">
-        <v>5</v>
-      </c>
+        <v>395</v>
+      </c>
+      <c r="E19" s="12"/>
       <c r="F19" s="12"/>
       <c r="G19" s="12"/>
       <c r="H19" s="12"/>
       <c r="I19" s="12" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="12"/>
-      <c r="B20" s="14"/>
-      <c r="C20" s="12"/>
-      <c r="D20" s="12"/>
-      <c r="E20" s="12"/>
+      <c r="A20" s="12" t="s">
+        <v>428</v>
+      </c>
+      <c r="B20" s="14" t="s">
+        <v>429</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>419</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>391</v>
+      </c>
+      <c r="E20" s="12">
+        <v>5</v>
+      </c>
       <c r="F20" s="12"/>
       <c r="G20" s="12"/>
       <c r="H20" s="12"/>
-      <c r="I20" s="12"/>
+      <c r="I20" s="12" t="s">
+        <v>120</v>
+      </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="12"/>
@@ -8793,13 +8821,13 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>424</v>
+        <v>430</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>425</v>
+        <v>431</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>359</v>
+        <v>364</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>64</v>
@@ -8807,335 +8835,335 @@
     </row>
     <row r="2" ht="42" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>426</v>
+        <v>432</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>427</v>
+        <v>433</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>428</v>
+        <v>434</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>429</v>
+        <v>435</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>430</v>
+        <v>436</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>431</v>
+        <v>437</v>
       </c>
       <c r="D3" s="12"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>432</v>
+        <v>438</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>433</v>
+        <v>439</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>431</v>
+        <v>437</v>
       </c>
       <c r="D4" s="12"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>434</v>
+        <v>440</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>435</v>
+        <v>441</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>431</v>
+        <v>437</v>
       </c>
       <c r="D5" s="12"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>436</v>
+        <v>442</v>
       </c>
       <c r="B6" s="14" t="s">
+        <v>443</v>
+      </c>
+      <c r="C6" s="12" t="s">
         <v>437</v>
-      </c>
-      <c r="C6" s="12" t="s">
-        <v>431</v>
       </c>
       <c r="D6" s="12"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
-        <v>438</v>
+        <v>444</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>439</v>
+        <v>445</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>431</v>
+        <v>437</v>
       </c>
       <c r="D7" s="12"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>440</v>
+        <v>446</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>441</v>
+        <v>447</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>431</v>
+        <v>437</v>
       </c>
       <c r="D8" s="12"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>442</v>
+        <v>448</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>443</v>
+        <v>449</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>431</v>
+        <v>437</v>
       </c>
       <c r="D9" s="12"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>444</v>
+        <v>450</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>445</v>
+        <v>451</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>431</v>
+        <v>437</v>
       </c>
       <c r="D10" s="12"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
-        <v>446</v>
+        <v>452</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>447</v>
+        <v>453</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>431</v>
+        <v>437</v>
       </c>
       <c r="D11" s="12"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>448</v>
+        <v>454</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>431</v>
+        <v>437</v>
       </c>
       <c r="D12" s="12"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
-        <v>449</v>
+        <v>455</v>
       </c>
       <c r="B13" s="14"/>
       <c r="C13" s="12" t="s">
-        <v>450</v>
+        <v>456</v>
       </c>
       <c r="D13" s="12"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
-        <v>451</v>
+        <v>457</v>
       </c>
       <c r="B14" s="14"/>
       <c r="C14" s="12" t="s">
-        <v>450</v>
+        <v>456</v>
       </c>
       <c r="D14" s="12"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="12" t="s">
-        <v>452</v>
+        <v>458</v>
       </c>
       <c r="B15" s="14"/>
       <c r="C15" s="12" t="s">
-        <v>450</v>
+        <v>456</v>
       </c>
       <c r="D15" s="12"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="12" t="s">
-        <v>453</v>
+        <v>459</v>
       </c>
       <c r="B16" s="14"/>
       <c r="C16" s="12" t="s">
-        <v>450</v>
+        <v>456</v>
       </c>
       <c r="D16" s="12"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="12" t="s">
-        <v>454</v>
+        <v>460</v>
       </c>
       <c r="B17" s="14"/>
       <c r="C17" s="12" t="s">
-        <v>450</v>
+        <v>456</v>
       </c>
       <c r="D17" s="12"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="12" t="s">
-        <v>455</v>
+        <v>461</v>
       </c>
       <c r="B18" s="14"/>
       <c r="C18" s="12" t="s">
-        <v>450</v>
+        <v>456</v>
       </c>
       <c r="D18" s="12"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
-        <v>456</v>
+        <v>462</v>
       </c>
       <c r="B19" s="14"/>
       <c r="C19" s="12" t="s">
-        <v>450</v>
+        <v>456</v>
       </c>
       <c r="D19" s="12"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="12" t="s">
-        <v>457</v>
+        <v>463</v>
       </c>
       <c r="B20" s="14"/>
       <c r="C20" s="12" t="s">
-        <v>450</v>
+        <v>456</v>
       </c>
       <c r="D20" s="12"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="12" t="s">
-        <v>458</v>
+        <v>464</v>
       </c>
       <c r="B21" s="14"/>
       <c r="C21" s="12" t="s">
-        <v>450</v>
+        <v>456</v>
       </c>
       <c r="D21" s="12"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="12" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
       <c r="B22" s="14"/>
       <c r="C22" s="12" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
       <c r="D22" s="12"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
-        <v>461</v>
+        <v>467</v>
       </c>
       <c r="B23" s="14"/>
       <c r="C23" s="12" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
       <c r="D23" s="12"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
-        <v>462</v>
+        <v>468</v>
       </c>
       <c r="B24" s="14"/>
       <c r="C24" s="12" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
       <c r="D24" s="12"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="12" t="s">
-        <v>463</v>
+        <v>469</v>
       </c>
       <c r="B25" s="14"/>
       <c r="C25" s="12" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
       <c r="D25" s="12"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="12" t="s">
-        <v>464</v>
+        <v>470</v>
       </c>
       <c r="B26" s="14"/>
       <c r="C26" s="12" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
       <c r="D26" s="12"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="12" t="s">
-        <v>465</v>
+        <v>471</v>
       </c>
       <c r="B27" s="14"/>
       <c r="C27" s="12" t="s">
-        <v>466</v>
+        <v>472</v>
       </c>
       <c r="D27" s="12"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="12" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
       <c r="B28" s="14"/>
       <c r="C28" s="12" t="s">
-        <v>466</v>
+        <v>472</v>
       </c>
       <c r="D28" s="12"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="12" t="s">
-        <v>467</v>
+        <v>473</v>
       </c>
       <c r="B29" s="14"/>
       <c r="C29" s="12" t="s">
-        <v>466</v>
+        <v>472</v>
       </c>
       <c r="D29" s="12"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="12" t="s">
-        <v>468</v>
+        <v>474</v>
       </c>
       <c r="B30" s="14"/>
       <c r="C30" s="12" t="s">
-        <v>466</v>
+        <v>472</v>
       </c>
       <c r="D30" s="12"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="12" t="s">
-        <v>469</v>
+        <v>475</v>
       </c>
       <c r="B31" s="14"/>
       <c r="C31" s="12" t="s">
-        <v>466</v>
+        <v>472</v>
       </c>
       <c r="D31" s="12"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="12" t="s">
-        <v>470</v>
+        <v>476</v>
       </c>
       <c r="B32" s="14"/>
       <c r="C32" s="12" t="s">
-        <v>466</v>
+        <v>472</v>
       </c>
       <c r="D32" s="12"/>
     </row>
@@ -10181,7 +10209,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:2" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>471</v>
+        <v>477</v>
       </c>
       <c r="B1" s="10" t="s">
         <v>64</v>
@@ -10189,10 +10217,10 @@
     </row>
     <row r="2" ht="42" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>472</v>
+        <v>478</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -11021,22 +11049,22 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="G1" s="10" t="s">
         <v>64</v>
@@ -11044,66 +11072,66 @@
     </row>
     <row r="2" ht="42" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>473</v>
+        <v>479</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="G2" s="11" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>474</v>
+        <v>480</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>475</v>
+        <v>481</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>476</v>
+        <v>482</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>477</v>
+        <v>483</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>478</v>
+        <v>484</v>
       </c>
       <c r="F3" s="12" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="G3" s="12"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>479</v>
+        <v>485</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>480</v>
+        <v>486</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>481</v>
+        <v>487</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>478</v>
+        <v>484</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>482</v>
+        <v>488</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="G4" s="12"/>
     </row>
@@ -12926,13 +12954,13 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>483</v>
+        <v>489</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>471</v>
+        <v>477</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>484</v>
+        <v>490</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>64</v>
@@ -12940,21 +12968,21 @@
     </row>
     <row r="2" ht="42" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>485</v>
+        <v>491</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>486</v>
+        <v>492</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>487</v>
+        <v>493</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>488</v>
+        <v>494</v>
       </c>
       <c r="B3" s="12">
         <v>60</v>
@@ -12964,7 +12992,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>489</v>
+        <v>495</v>
       </c>
       <c r="B4" s="12">
         <v>60</v>
@@ -12974,7 +13002,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>490</v>
+        <v>496</v>
       </c>
       <c r="B5" s="12">
         <v>20</v>
@@ -12984,7 +13012,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>491</v>
+        <v>497</v>
       </c>
       <c r="B6" s="12">
         <v>20</v>
@@ -14189,52 +14217,52 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:1" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>492</v>
+        <v>498</v>
       </c>
     </row>
     <row r="2" ht="42" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>494</v>
+        <v>500</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>495</v>
+        <v>501</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>496</v>
+        <v>502</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>497</v>
+        <v>503</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>498</v>
+        <v>504</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>499</v>
+        <v>505</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>500</v>
+        <v>506</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>501</v>
+        <v>507</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
@@ -15306,7 +15334,9 @@
       </c>
       <c r="H17" s="12"/>
       <c r="I17" s="12"/>
-      <c r="J17" s="12"/>
+      <c r="J17" s="12" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="12">
@@ -15316,7 +15346,7 @@
         <v>84</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D18" s="12" t="s">
         <v>44</v>
@@ -15326,14 +15356,16 @@
         <v>→ Libre</v>
       </c>
       <c r="F18" s="14" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G18" s="12">
         <v>5</v>
       </c>
       <c r="H18" s="12"/>
       <c r="I18" s="12"/>
-      <c r="J18" s="12"/>
+      <c r="J18" s="12" t="s">
+        <v>116</v>
+      </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="12">
@@ -15343,7 +15375,7 @@
         <v>84</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D19" s="12" t="s">
         <v>44</v>
@@ -15353,17 +15385,15 @@
         <v>→ Libre</v>
       </c>
       <c r="F19" s="14" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G19" s="12">
         <v>3</v>
       </c>
-      <c r="H19" s="12" t="s">
-        <v>84</v>
-      </c>
+      <c r="H19" s="12"/>
       <c r="I19" s="12"/>
       <c r="J19" s="12" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
@@ -15374,24 +15404,28 @@
         <v>84</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>56</v>
+        <v>120</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="E20" s="13" t="str">
         <f>IF(D20="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D20,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
-        <v>→ Squid</v>
+        <v>→ Libre</v>
       </c>
       <c r="F20" s="14" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="G20" s="12">
-        <v>5</v>
-      </c>
-      <c r="H20" s="12"/>
+        <v>3</v>
+      </c>
+      <c r="H20" s="12" t="s">
+        <v>84</v>
+      </c>
       <c r="I20" s="12"/>
-      <c r="J20" s="12"/>
+      <c r="J20" s="12" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="12">
@@ -15401,19 +15435,21 @@
         <v>84</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="E21" s="13" t="str">
         <f>IF(D21="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D21,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
-        <v>→ Apuesta</v>
+        <v>→ Squid</v>
       </c>
       <c r="F21" s="14" t="s">
-        <v>119</v>
-      </c>
-      <c r="G21" s="12"/>
+        <v>123</v>
+      </c>
+      <c r="G21" s="12">
+        <v>5</v>
+      </c>
       <c r="H21" s="12"/>
       <c r="I21" s="12"/>
       <c r="J21" s="12"/>
@@ -15426,43 +15462,53 @@
         <v>84</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="E22" s="13" t="str">
         <f>IF(D22="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D22,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
-        <v>→ —</v>
+        <v>→ Apuesta</v>
       </c>
       <c r="F22" s="14" t="s">
-        <v>120</v>
-      </c>
-      <c r="G22" s="12">
-        <v>10</v>
-      </c>
-      <c r="H22" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="G22" s="12"/>
+      <c r="H22" s="12"/>
+      <c r="I22" s="12"/>
+      <c r="J22" s="12"/>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A23" s="12">
+        <v>21</v>
+      </c>
+      <c r="B23" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="I22" s="12"/>
-      <c r="J22" s="12" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A23" s="12"/>
-      <c r="B23" s="12"/>
-      <c r="C23" s="12"/>
-      <c r="D23" s="12"/>
+      <c r="C23" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="D23" s="12" t="s">
+        <v>59</v>
+      </c>
       <c r="E23" s="13" t="str">
         <f>IF(D23="","",IFERROR("→ "&amp;INDEX({"Pulsador","Test","Verdad o mentira","Dos verdades","Votación","Estimación","Contador","Reflejos","Libre","Palabras","Agitar","Apuesta","Squid","—"},MATCH(D23,{"Pulsador","Test","Verdad o mentira","Dos verdades y una mentira","Votación","Estimación","Parar el contador","Duelo de reflejos","Libre","Palabras secretas","Agita el móvil","La gran apuesta","Squid Games","Lobos contra vampiros"},0)),"¿tipo?"))</f>
-        <v/>
-      </c>
-      <c r="F23" s="14"/>
-      <c r="G23" s="12"/>
-      <c r="H23" s="12"/>
+        <v>→ —</v>
+      </c>
+      <c r="F23" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="G23" s="12">
+        <v>10</v>
+      </c>
+      <c r="H23" s="12" t="s">
+        <v>84</v>
+      </c>
       <c r="I23" s="12"/>
-      <c r="J23" s="12"/>
+      <c r="J23" s="12" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="12"/>
@@ -17850,10 +17896,10 @@
       <formula1>"Sí,No"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Valor no previsto" error="Elige un valor de la lista." sqref="J10:J200">
-      <formula1>"Noche de luna,Cementerio,Bosque encantado,Huerto de calabazas,Laboratorio,Mansión encantada,Telaraña,Aquelarre,Cripta helada,Tormenta,Plató millonario,Squid Games,Discoteca,Luna llena"</formula1>
+      <formula1>"Noche de luna,Cementerio,Bosque encantado,Huerto de calabazas,Laboratorio,Mansión encantada,Telaraña,Aquelarre,Cripta helada,Tormenta,Plató millonario,Squid Games,Discoteca,Luna llena,Verano,Galletas,Refrescos"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Valor no previsto" error="Elige un valor de la lista." sqref="J3:J200">
-      <formula1>"Noche de luna,Cementerio,Bosque encantado,Huerto de calabazas,Laboratorio,Mansión encantada,Telaraña,Aquelarre,Cripta helada,Tormenta,Plató millonario,Squid Games,Discoteca,Luna llena"</formula1>
+      <formula1>"Noche de luna,Cementerio,Bosque encantado,Huerto de calabazas,Laboratorio,Mansión encantada,Telaraña,Aquelarre,Cripta helada,Tormenta,Plató millonario,Squid Games,Discoteca,Luna llena,Verano,Galletas,Refrescos"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -17875,34 +17921,34 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:2" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2" ht="42" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -18718,134 +18764,134 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:3" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
     </row>
     <row r="2" ht="42" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="B4" s="12">
         <v>1</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="B5" s="12">
         <v>1</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="B6" s="12">
         <v>1</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="B7" s="12">
         <v>1</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="B8" s="12">
         <v>0</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="B9" s="12" t="s">
         <v>84</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="B10" s="12">
         <v>20</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="B11" s="12">
         <v>60</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="B12" s="12">
         <v>3</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -19812,22 +19858,22 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="G1" s="10" t="s">
         <v>64</v>
@@ -19835,33 +19881,33 @@
     </row>
     <row r="2" ht="42" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="G2" s="11" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="C3" s="12" t="s">
         <v>84</v>
@@ -19875,10 +19921,10 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="C4" s="12" t="s">
         <v>84</v>
@@ -19892,10 +19938,10 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="C5" s="12" t="s">
         <v>84</v>
@@ -19909,10 +19955,10 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="C6" s="12" t="s">
         <v>84</v>
@@ -19926,10 +19972,10 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="C7" s="12" t="s">
         <v>84</v>
@@ -19943,10 +19989,10 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="C8" s="12" t="s">
         <v>84</v>
@@ -19960,16 +20006,16 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="C9" s="12" t="s">
         <v>84</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="E9" s="12"/>
       <c r="F9" s="12"/>
@@ -19979,16 +20025,16 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="C10" s="12" t="s">
         <v>84</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="E10" s="12"/>
       <c r="F10" s="12"/>
@@ -19998,16 +20044,16 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="C11" s="12" t="s">
         <v>84</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="E11" s="12"/>
       <c r="F11" s="12"/>
@@ -20017,19 +20063,19 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="C12" s="12" t="s">
         <v>84</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="F12" s="12">
         <v>0</v>
@@ -20040,19 +20086,19 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="C13" s="12" t="s">
         <v>84</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="F13" s="12">
         <v>0</v>
@@ -20063,19 +20109,19 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="C14" s="12" t="s">
         <v>84</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="F14" s="12">
         <v>0</v>
@@ -21796,28 +21842,28 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:9" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="I1" s="10" t="s">
         <v>64</v>
@@ -21825,329 +21871,329 @@
     </row>
     <row r="2" ht="42" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="G2" s="11" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="H2" s="11" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="I2" s="11" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="F3" s="12" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="G3" s="12" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="H3" s="12"/>
       <c r="I3" s="12"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="E4" s="14" t="s">
+        <v>230</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>206</v>
+      </c>
+      <c r="G4" s="12" t="s">
         <v>225</v>
-      </c>
-      <c r="F4" s="12" t="s">
-        <v>201</v>
-      </c>
-      <c r="G4" s="12" t="s">
-        <v>220</v>
       </c>
       <c r="H4" s="12"/>
       <c r="I4" s="12"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="G5" s="12" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="H5" s="12"/>
       <c r="I5" s="12"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="G6" s="12" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="H6" s="12"/>
       <c r="I6" s="12"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="F7" s="12" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="G7" s="12" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="H7" s="12"/>
       <c r="I7" s="12"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="G8" s="12" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="H8" s="12"/>
       <c r="I8" s="12"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
+        <v>251</v>
+      </c>
+      <c r="B9" s="14" t="s">
+        <v>252</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>253</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>254</v>
+      </c>
+      <c r="E9" s="14" t="s">
+        <v>255</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>207</v>
+      </c>
+      <c r="G9" s="12" t="s">
         <v>246</v>
-      </c>
-      <c r="B9" s="14" t="s">
-        <v>247</v>
-      </c>
-      <c r="C9" s="14" t="s">
-        <v>248</v>
-      </c>
-      <c r="D9" s="14" t="s">
-        <v>249</v>
-      </c>
-      <c r="E9" s="14" t="s">
-        <v>250</v>
-      </c>
-      <c r="F9" s="12" t="s">
-        <v>202</v>
-      </c>
-      <c r="G9" s="12" t="s">
-        <v>241</v>
       </c>
       <c r="H9" s="12"/>
       <c r="I9" s="12"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="F10" s="12" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="G10" s="12" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="H10" s="12"/>
       <c r="I10" s="12"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="F11" s="12" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="G11" s="12" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="H11" s="12"/>
       <c r="I11" s="12"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="E12" s="14" t="s">
+        <v>271</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>206</v>
+      </c>
+      <c r="G12" s="12" t="s">
         <v>266</v>
-      </c>
-      <c r="F12" s="12" t="s">
-        <v>201</v>
-      </c>
-      <c r="G12" s="12" t="s">
-        <v>261</v>
       </c>
       <c r="H12" s="12"/>
       <c r="I12" s="12"/>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="F13" s="12" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="G13" s="12" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="H13" s="12"/>
       <c r="I13" s="12"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="F14" s="12" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="G14" s="12" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="H14" s="12"/>
       <c r="I14" s="12"/>
@@ -24274,10 +24320,10 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:3" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="C1" s="10" t="s">
         <v>64</v>
@@ -24285,84 +24331,84 @@
     </row>
     <row r="2" ht="42" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="C3" s="12"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="C4" s="12"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="C5" s="12"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="C6" s="12"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
+        <v>291</v>
+      </c>
+      <c r="B7" s="12" t="s">
         <v>286</v>
-      </c>
-      <c r="B7" s="12" t="s">
-        <v>281</v>
       </c>
       <c r="C7" s="12"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="C8" s="12"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
+        <v>293</v>
+      </c>
+      <c r="B9" s="12" t="s">
         <v>288</v>
-      </c>
-      <c r="B9" s="12" t="s">
-        <v>283</v>
       </c>
       <c r="C9" s="12"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="C10" s="12"/>
     </row>
@@ -25361,19 +25407,19 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="F1" s="10" t="s">
         <v>64</v>
@@ -25381,36 +25427,36 @@
     </row>
     <row r="2" ht="42" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="E3" s="12">
         <v>2</v>
@@ -25419,16 +25465,16 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="E4" s="12">
         <v>3</v>
@@ -25437,16 +25483,16 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="E5" s="12">
         <v>1</v>
@@ -25455,16 +25501,16 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="E6" s="12">
         <v>2</v>
@@ -25473,16 +25519,16 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
       <c r="E7" s="12">
         <v>3</v>
@@ -25491,16 +25537,16 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="E8" s="12">
         <v>2</v>
@@ -25509,16 +25555,16 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="E9" s="12">
         <v>2</v>
@@ -27102,7 +27148,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:2" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="B1" s="10" t="s">
         <v>64</v>
@@ -27110,57 +27156,57 @@
     </row>
     <row r="2" ht="42" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>327</v>
+        <v>332</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="B3" s="12"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="B4" s="12"/>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="B5" s="12"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
       <c r="B6" s="12"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="B7" s="12"/>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="B8" s="12"/>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="B9" s="12"/>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="B10" s="12"/>
     </row>

</xml_diff>

<commit_message>
Gimnasio para Fit o Fat, canción por juego, hueco de redoble y música que sigue
- Entorno «Gimnasio» (racks, mancuernas, banco, neón a ras de suelo, magnesio) con su música.
- Música/<Sección>/<Juego>/: la canción de cada juego de Libre suena desde el «¡ya!» hasta pararlo.
- Hueco de efecto «Redoble»: tu archivo sustituye al de la app y su golpe cae con el del revelado.
- Un momento sin canción sigue con la que sonaba; el mismo archivo en varios momentos no vuelve a empezar.
- Sin sonido de viento (tampoco en el puente de Squid).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/plantilla-concurso.xlsx
+++ b/public/plantilla-concurso.xlsx
@@ -17896,10 +17896,10 @@
       <formula1>"Sí,No"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Valor no previsto" error="Elige un valor de la lista." sqref="J10:J200">
-      <formula1>"Noche de luna,Cementerio,Bosque encantado,Huerto de calabazas,Laboratorio,Mansión encantada,Telaraña,Aquelarre,Cripta helada,Tormenta,Plató millonario,Squid Games,Discoteca,Luna llena,Verano,Galletas,Refrescos"</formula1>
+      <formula1>"Noche de luna,Cementerio,Bosque encantado,Huerto de calabazas,Laboratorio,Mansión encantada,Telaraña,Aquelarre,Cripta helada,Tormenta,Plató millonario,Squid Games,Discoteca,Luna llena,Verano,Galletas,Refrescos,Gimnasio"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Valor no previsto" error="Elige un valor de la lista." sqref="J3:J200">
-      <formula1>"Noche de luna,Cementerio,Bosque encantado,Huerto de calabazas,Laboratorio,Mansión encantada,Telaraña,Aquelarre,Cripta helada,Tormenta,Plató millonario,Squid Games,Discoteca,Luna llena,Verano,Galletas,Refrescos"</formula1>
+      <formula1>"Noche de luna,Cementerio,Bosque encantado,Huerto de calabazas,Laboratorio,Mansión encantada,Telaraña,Aquelarre,Cripta helada,Tormenta,Plató millonario,Squid Games,Discoteca,Luna llena,Verano,Galletas,Refrescos,Gimnasio"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Temáticas Relojería y Globos, y caras grandes en los duelos de Libre
- Relojería (Reloj interno): reloj de pared con agujas, reloj de péndulo y engranajes; música sin tictac.
- Globos (Guerra de globos): globos rojos y azules que suben y explotan, con música de feria.
- Plantilla con los dos entornos en la lista de Entorno.
- Libre con 4 participantes o menos: cada tarjeta lleva la cara (o el icono) en grande con aro de su color.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/plantilla-concurso.xlsx
+++ b/public/plantilla-concurso.xlsx
@@ -17896,10 +17896,10 @@
       <formula1>"Sí,No"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Valor no previsto" error="Elige un valor de la lista." sqref="J10:J200">
-      <formula1>"Noche de luna,Cementerio,Bosque encantado,Huerto de calabazas,Laboratorio,Mansión encantada,Telaraña,Aquelarre,Cripta helada,Tormenta,Plató millonario,Squid Games,Discoteca,Luna llena,Verano,Galletas,Refrescos,Gimnasio"</formula1>
+      <formula1>"Noche de luna,Cementerio,Bosque encantado,Huerto de calabazas,Laboratorio,Mansión encantada,Telaraña,Aquelarre,Cripta helada,Tormenta,Plató millonario,Squid Games,Discoteca,Luna llena,Verano,Galletas,Refrescos,Gimnasio,Relojería,Globos"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Valor no previsto" error="Elige un valor de la lista." sqref="J3:J200">
-      <formula1>"Noche de luna,Cementerio,Bosque encantado,Huerto de calabazas,Laboratorio,Mansión encantada,Telaraña,Aquelarre,Cripta helada,Tormenta,Plató millonario,Squid Games,Discoteca,Luna llena,Verano,Galletas,Refrescos,Gimnasio"</formula1>
+      <formula1>"Noche de luna,Cementerio,Bosque encantado,Huerto de calabazas,Laboratorio,Mansión encantada,Telaraña,Aquelarre,Cripta helada,Tormenta,Plató millonario,Squid Games,Discoteca,Luna llena,Verano,Galletas,Refrescos,Gimnasio,Relojería,Globos"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>